<commit_message>
Restructure dashboard for alerts and knowledge loop
</commit_message>
<xml_diff>
--- a/data/tiktok-ai-operations-center-wps-kdocs-template.xlsx
+++ b/data/tiktok-ai-operations-center-wps-kdocs-template.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填报首页" sheetId="1" r:id="R0304c03f9b614dee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺日汇总" sheetId="2" r:id="R6767648e80bb460e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商品数据" sheetId="3" r:id="R0324fc1e77844316"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营动作" sheetId="4" r:id="R3ee93319e3c84222"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布趋势" sheetId="5" r:id="Rddf937ed2a834558"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD达人" sheetId="6" r:id="R925bf2277d3d4030"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="广告计划" sheetId="7" r:id="R7e0dcf050d1946f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="短视频数据" sheetId="8" r:id="R04cd79452ee74a9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段字典" sheetId="9" r:id="R0e25b6bbaf404b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填报首页" sheetId="1" r:id="R158f1106a3d14e7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺日汇总" sheetId="2" r:id="R5d4c54b3c7cb4c43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商品数据" sheetId="3" r:id="R9254024da00e430e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营动作" sheetId="4" r:id="Rbf9426a7fb904050"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布趋势" sheetId="5" r:id="R90ea4999689c4ceb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD达人" sheetId="6" r:id="R2c2343c8512644a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="广告计划" sheetId="7" r:id="R2ef7a71a7ef44009"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="短视频数据" sheetId="8" r:id="Re1283371afe44f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段字典" sheetId="9" r:id="R17071b1b50f8497a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -624,9 +624,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ProductsTable" displayName="ProductsTable" ref="A5:N11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:N11"/>
-  <x:tableColumns count="14">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ProductsTable" displayName="ProductsTable" ref="A5:R11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:R11"/>
+  <x:tableColumns count="18">
     <x:tableColumn id="1" name="日期"/>
     <x:tableColumn id="2" name="店铺"/>
     <x:tableColumn id="3" name="商品ID"/>
@@ -638,9 +638,13 @@
     <x:tableColumn id="9" name="销量"/>
     <x:tableColumn id="10" name="GMV(CNY)"/>
     <x:tableColumn id="11" name="GMV变化(%)"/>
-    <x:tableColumn id="12" name="CVR变化(百分点)"/>
-    <x:tableColumn id="13" name="当前状态"/>
-    <x:tableColumn id="14" name="备注"/>
+    <x:tableColumn id="12" name="曝光变化(%)"/>
+    <x:tableColumn id="13" name="CTR变化(百分点)"/>
+    <x:tableColumn id="14" name="CVR变化(百分点)"/>
+    <x:tableColumn id="15" name="预警节点"/>
+    <x:tableColumn id="16" name="建议动作"/>
+    <x:tableColumn id="17" name="当前状态"/>
+    <x:tableColumn id="18" name="备注"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -734,8 +738,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="DictionaryTable" displayName="DictionaryTable" ref="A5:D11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:D11"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="DictionaryTable" displayName="DictionaryTable" ref="A5:D12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:D12"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="字段"/>
     <x:tableColumn id="2" name="所在表"/>
@@ -3302,7 +3306,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9066158fe214c17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fcf6938d8f540da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3322,9 +3326,13 @@
     <x:col min="9" max="9" width="11" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="26" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="14" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="17" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="13" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="34" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="13" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -3343,11 +3351,15 @@
       <x:c r="K1" s="36"/>
       <x:c r="L1" s="36"/>
       <x:c r="M1" s="36"/>
-      <x:c r="N1" s="37"/>
+      <x:c r="N1" s="36"/>
+      <x:c r="O1" s="36"/>
+      <x:c r="P1" s="36"/>
+      <x:c r="Q1" s="36"/>
+      <x:c r="R1" s="37"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="42" t="str">
-        <x:v>一行代表一个日期 + 店铺 + 商品链接；黄色区域可直接替换成真实导出数据。</x:v>
+        <x:v>一行代表一个日期 + 店铺 + 商品链接；黄色区域可直接替换成真实导出数据，预警字段用于 T+1 / T+3 / T+7 核查。</x:v>
       </x:c>
       <x:c r="B2" s="43"/>
       <x:c r="C2" s="43"/>
@@ -3361,7 +3373,11 @@
       <x:c r="K2" s="43"/>
       <x:c r="L2" s="43"/>
       <x:c r="M2" s="43"/>
-      <x:c r="N2" s="44"/>
+      <x:c r="N2" s="43"/>
+      <x:c r="O2" s="43"/>
+      <x:c r="P2" s="43"/>
+      <x:c r="Q2" s="43"/>
+      <x:c r="R2" s="44"/>
     </x:row>
     <x:row r="3" ht="21" customHeight="1">
       <x:c r="A3" s="24"/>
@@ -3377,7 +3393,11 @@
       <x:c r="K3" s="3"/>
       <x:c r="L3" s="3"/>
       <x:c r="M3" s="3"/>
-      <x:c r="N3" s="25"/>
+      <x:c r="N3" s="3"/>
+      <x:c r="O3" s="3"/>
+      <x:c r="P3" s="3"/>
+      <x:c r="Q3" s="3"/>
+      <x:c r="R3" s="25"/>
     </x:row>
     <x:row r="4" ht="21" customHeight="1">
       <x:c r="A4" s="24"/>
@@ -3393,7 +3413,11 @@
       <x:c r="K4" s="3"/>
       <x:c r="L4" s="3"/>
       <x:c r="M4" s="3"/>
-      <x:c r="N4" s="25"/>
+      <x:c r="N4" s="3"/>
+      <x:c r="O4" s="3"/>
+      <x:c r="P4" s="3"/>
+      <x:c r="Q4" s="3"/>
+      <x:c r="R4" s="25"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="50" t="str">
@@ -3430,12 +3454,24 @@
         <x:v>GMV变化(%)</x:v>
       </x:c>
       <x:c r="L5" s="50" t="str">
+        <x:v>曝光变化(%)</x:v>
+      </x:c>
+      <x:c r="M5" s="50" t="str">
+        <x:v>CTR变化(百分点)</x:v>
+      </x:c>
+      <x:c r="N5" s="50" t="str">
         <x:v>CVR变化(百分点)</x:v>
       </x:c>
-      <x:c r="M5" s="50" t="str">
+      <x:c r="O5" s="50" t="str">
+        <x:v>预警节点</x:v>
+      </x:c>
+      <x:c r="P5" s="50" t="str">
+        <x:v>建议动作</x:v>
+      </x:c>
+      <x:c r="Q5" s="50" t="str">
         <x:v>当前状态</x:v>
       </x:c>
-      <x:c r="N5" s="50" t="str">
+      <x:c r="R5" s="50" t="str">
         <x:v>备注</x:v>
       </x:c>
     </x:row>
@@ -3474,12 +3510,22 @@
         <x:v>18.6</x:v>
       </x:c>
       <x:c r="L6" s="61" t="n">
+        <x:v>8.4</x:v>
+      </x:c>
+      <x:c r="M6" s="61" t="n">
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="N6" s="61" t="n">
         <x:v>0.72</x:v>
       </x:c>
-      <x:c r="M6" s="12" t="str">
+      <x:c r="O6" s="12" t="str">
+        <x:v>T+3</x:v>
+      </x:c>
+      <x:c r="P6" s="12" t="str"/>
+      <x:c r="Q6" s="12" t="str">
         <x:v>表现良好</x:v>
       </x:c>
-      <x:c r="N6" s="74" t="str"/>
+      <x:c r="R6" s="74" t="str"/>
     </x:row>
     <x:row r="7" ht="21" customHeight="1">
       <x:c r="A7" s="59" t="n">
@@ -3516,12 +3562,24 @@
         <x:v>-12.4</x:v>
       </x:c>
       <x:c r="L7" s="61" t="n">
+        <x:v>-28</x:v>
+      </x:c>
+      <x:c r="M7" s="61" t="n">
+        <x:v>-0.62</x:v>
+      </x:c>
+      <x:c r="N7" s="61" t="n">
         <x:v>-1.18</x:v>
       </x:c>
-      <x:c r="M7" s="12" t="str">
+      <x:c r="O7" s="12" t="str">
+        <x:v>T+1</x:v>
+      </x:c>
+      <x:c r="P7" s="12" t="str">
+        <x:v>先核查推荐流量与主图承接，再决定是否调整标题。</x:v>
+      </x:c>
+      <x:c r="Q7" s="12" t="str">
         <x:v>需处理</x:v>
       </x:c>
-      <x:c r="N7" s="74" t="str"/>
+      <x:c r="R7" s="74" t="str"/>
     </x:row>
     <x:row r="8" ht="21" customHeight="1">
       <x:c r="A8" s="59" t="n">
@@ -3558,12 +3616,24 @@
         <x:v>6.8</x:v>
       </x:c>
       <x:c r="L8" s="61" t="n">
+        <x:v>-12</x:v>
+      </x:c>
+      <x:c r="M8" s="61" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="N8" s="61" t="n">
         <x:v>-0.42</x:v>
       </x:c>
-      <x:c r="M8" s="12" t="str">
+      <x:c r="O8" s="12" t="str">
+        <x:v>T+7</x:v>
+      </x:c>
+      <x:c r="P8" s="12" t="str">
+        <x:v>检查商品承接和优惠设置，继续观察 CVR 是否恢复。</x:v>
+      </x:c>
+      <x:c r="Q8" s="12" t="str">
         <x:v>需观察</x:v>
       </x:c>
-      <x:c r="N8" s="74" t="str"/>
+      <x:c r="R8" s="74" t="str"/>
     </x:row>
     <x:row r="9" ht="21" customHeight="1">
       <x:c r="A9" s="59" t="n">
@@ -3600,12 +3670,22 @@
         <x:v>24.1</x:v>
       </x:c>
       <x:c r="L9" s="61" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="M9" s="61" t="n">
+        <x:v>0.18</x:v>
+      </x:c>
+      <x:c r="N9" s="61" t="n">
         <x:v>0.38</x:v>
       </x:c>
-      <x:c r="M9" s="12" t="str">
+      <x:c r="O9" s="12" t="str">
+        <x:v>T+3</x:v>
+      </x:c>
+      <x:c r="P9" s="12" t="str"/>
+      <x:c r="Q9" s="12" t="str">
         <x:v>表现良好</x:v>
       </x:c>
-      <x:c r="N9" s="74" t="str"/>
+      <x:c r="R9" s="74" t="str"/>
     </x:row>
     <x:row r="10" ht="21" customHeight="1">
       <x:c r="A10" s="59" t="n">
@@ -3642,12 +3722,24 @@
         <x:v>-26.5</x:v>
       </x:c>
       <x:c r="L10" s="61" t="n">
+        <x:v>-31</x:v>
+      </x:c>
+      <x:c r="M10" s="61" t="n">
+        <x:v>-0.84</x:v>
+      </x:c>
+      <x:c r="N10" s="61" t="n">
         <x:v>-1.46</x:v>
       </x:c>
-      <x:c r="M10" s="12" t="str">
+      <x:c r="O10" s="12" t="str">
+        <x:v>T+3</x:v>
+      </x:c>
+      <x:c r="P10" s="12" t="str">
+        <x:v>优先检查广告落地页、流量来源和商品库存承接。</x:v>
+      </x:c>
+      <x:c r="Q10" s="12" t="str">
         <x:v>需处理</x:v>
       </x:c>
-      <x:c r="N10" s="74" t="str"/>
+      <x:c r="R10" s="74" t="str"/>
     </x:row>
     <x:row r="11" ht="21" customHeight="1">
       <x:c r="A11" s="62" t="n">
@@ -3684,12 +3776,24 @@
         <x:v>-3.7</x:v>
       </x:c>
       <x:c r="L11" s="65" t="n">
+        <x:v>-8.2</x:v>
+      </x:c>
+      <x:c r="M11" s="65" t="n">
+        <x:v>-0.22</x:v>
+      </x:c>
+      <x:c r="N11" s="65" t="n">
         <x:v>-0.24</x:v>
       </x:c>
-      <x:c r="M11" s="63" t="str">
+      <x:c r="O11" s="63" t="str">
+        <x:v>T+1</x:v>
+      </x:c>
+      <x:c r="P11" s="63" t="str">
+        <x:v>继续观察，不足以单独判定为异常。</x:v>
+      </x:c>
+      <x:c r="Q11" s="63" t="str">
         <x:v>需观察</x:v>
       </x:c>
-      <x:c r="N11" s="76" t="str"/>
+      <x:c r="R11" s="76" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="66"/>
@@ -3706,6 +3810,10 @@
       <x:c r="L12" s="66"/>
       <x:c r="M12" s="66"/>
       <x:c r="N12" s="66"/>
+      <x:c r="O12" s="66"/>
+      <x:c r="P12" s="66"/>
+      <x:c r="Q12" s="66"/>
+      <x:c r="R12" s="66"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="66"/>
@@ -3722,6 +3830,10 @@
       <x:c r="L13" s="66"/>
       <x:c r="M13" s="66"/>
       <x:c r="N13" s="66"/>
+      <x:c r="O13" s="66"/>
+      <x:c r="P13" s="66"/>
+      <x:c r="Q13" s="66"/>
+      <x:c r="R13" s="66"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="66"/>
@@ -3738,6 +3850,10 @@
       <x:c r="L14" s="66"/>
       <x:c r="M14" s="66"/>
       <x:c r="N14" s="66"/>
+      <x:c r="O14" s="66"/>
+      <x:c r="P14" s="66"/>
+      <x:c r="Q14" s="66"/>
+      <x:c r="R14" s="66"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="66"/>
@@ -3754,6 +3870,10 @@
       <x:c r="L15" s="66"/>
       <x:c r="M15" s="66"/>
       <x:c r="N15" s="66"/>
+      <x:c r="O15" s="66"/>
+      <x:c r="P15" s="66"/>
+      <x:c r="Q15" s="66"/>
+      <x:c r="R15" s="66"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="66"/>
@@ -3770,6 +3890,10 @@
       <x:c r="L16" s="66"/>
       <x:c r="M16" s="66"/>
       <x:c r="N16" s="66"/>
+      <x:c r="O16" s="66"/>
+      <x:c r="P16" s="66"/>
+      <x:c r="Q16" s="66"/>
+      <x:c r="R16" s="66"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="66"/>
@@ -3786,6 +3910,10 @@
       <x:c r="L17" s="66"/>
       <x:c r="M17" s="66"/>
       <x:c r="N17" s="66"/>
+      <x:c r="O17" s="66"/>
+      <x:c r="P17" s="66"/>
+      <x:c r="Q17" s="66"/>
+      <x:c r="R17" s="66"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="66"/>
@@ -3802,6 +3930,10 @@
       <x:c r="L18" s="66"/>
       <x:c r="M18" s="66"/>
       <x:c r="N18" s="66"/>
+      <x:c r="O18" s="66"/>
+      <x:c r="P18" s="66"/>
+      <x:c r="Q18" s="66"/>
+      <x:c r="R18" s="66"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="66"/>
@@ -3818,6 +3950,10 @@
       <x:c r="L19" s="66"/>
       <x:c r="M19" s="66"/>
       <x:c r="N19" s="66"/>
+      <x:c r="O19" s="66"/>
+      <x:c r="P19" s="66"/>
+      <x:c r="Q19" s="66"/>
+      <x:c r="R19" s="66"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="66"/>
@@ -3834,6 +3970,10 @@
       <x:c r="L20" s="66"/>
       <x:c r="M20" s="66"/>
       <x:c r="N20" s="66"/>
+      <x:c r="O20" s="66"/>
+      <x:c r="P20" s="66"/>
+      <x:c r="Q20" s="66"/>
+      <x:c r="R20" s="66"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="66"/>
@@ -3850,6 +3990,10 @@
       <x:c r="L21" s="66"/>
       <x:c r="M21" s="66"/>
       <x:c r="N21" s="66"/>
+      <x:c r="O21" s="66"/>
+      <x:c r="P21" s="66"/>
+      <x:c r="Q21" s="66"/>
+      <x:c r="R21" s="66"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="66"/>
@@ -3866,6 +4010,10 @@
       <x:c r="L22" s="66"/>
       <x:c r="M22" s="66"/>
       <x:c r="N22" s="66"/>
+      <x:c r="O22" s="66"/>
+      <x:c r="P22" s="66"/>
+      <x:c r="Q22" s="66"/>
+      <x:c r="R22" s="66"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="66"/>
@@ -3882,6 +4030,10 @@
       <x:c r="L23" s="66"/>
       <x:c r="M23" s="66"/>
       <x:c r="N23" s="66"/>
+      <x:c r="O23" s="66"/>
+      <x:c r="P23" s="66"/>
+      <x:c r="Q23" s="66"/>
+      <x:c r="R23" s="66"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="66"/>
@@ -3898,6 +4050,10 @@
       <x:c r="L24" s="66"/>
       <x:c r="M24" s="66"/>
       <x:c r="N24" s="66"/>
+      <x:c r="O24" s="66"/>
+      <x:c r="P24" s="66"/>
+      <x:c r="Q24" s="66"/>
+      <x:c r="R24" s="66"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="66"/>
@@ -3914,6 +4070,10 @@
       <x:c r="L25" s="66"/>
       <x:c r="M25" s="66"/>
       <x:c r="N25" s="66"/>
+      <x:c r="O25" s="66"/>
+      <x:c r="P25" s="66"/>
+      <x:c r="Q25" s="66"/>
+      <x:c r="R25" s="66"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="66"/>
@@ -3930,6 +4090,10 @@
       <x:c r="L26" s="66"/>
       <x:c r="M26" s="66"/>
       <x:c r="N26" s="66"/>
+      <x:c r="O26" s="66"/>
+      <x:c r="P26" s="66"/>
+      <x:c r="Q26" s="66"/>
+      <x:c r="R26" s="66"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="66"/>
@@ -3946,6 +4110,10 @@
       <x:c r="L27" s="66"/>
       <x:c r="M27" s="66"/>
       <x:c r="N27" s="66"/>
+      <x:c r="O27" s="66"/>
+      <x:c r="P27" s="66"/>
+      <x:c r="Q27" s="66"/>
+      <x:c r="R27" s="66"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="66"/>
@@ -3962,6 +4130,10 @@
       <x:c r="L28" s="66"/>
       <x:c r="M28" s="66"/>
       <x:c r="N28" s="66"/>
+      <x:c r="O28" s="66"/>
+      <x:c r="P28" s="66"/>
+      <x:c r="Q28" s="66"/>
+      <x:c r="R28" s="66"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="66"/>
@@ -3978,6 +4150,10 @@
       <x:c r="L29" s="66"/>
       <x:c r="M29" s="66"/>
       <x:c r="N29" s="66"/>
+      <x:c r="O29" s="66"/>
+      <x:c r="P29" s="66"/>
+      <x:c r="Q29" s="66"/>
+      <x:c r="R29" s="66"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="66"/>
@@ -3994,6 +4170,10 @@
       <x:c r="L30" s="66"/>
       <x:c r="M30" s="66"/>
       <x:c r="N30" s="66"/>
+      <x:c r="O30" s="66"/>
+      <x:c r="P30" s="66"/>
+      <x:c r="Q30" s="66"/>
+      <x:c r="R30" s="66"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="66"/>
@@ -4010,6 +4190,10 @@
       <x:c r="L31" s="66"/>
       <x:c r="M31" s="66"/>
       <x:c r="N31" s="66"/>
+      <x:c r="O31" s="66"/>
+      <x:c r="P31" s="66"/>
+      <x:c r="Q31" s="66"/>
+      <x:c r="R31" s="66"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="66"/>
@@ -4026,6 +4210,10 @@
       <x:c r="L32" s="66"/>
       <x:c r="M32" s="66"/>
       <x:c r="N32" s="66"/>
+      <x:c r="O32" s="66"/>
+      <x:c r="P32" s="66"/>
+      <x:c r="Q32" s="66"/>
+      <x:c r="R32" s="66"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="66"/>
@@ -4042,6 +4230,10 @@
       <x:c r="L33" s="66"/>
       <x:c r="M33" s="66"/>
       <x:c r="N33" s="66"/>
+      <x:c r="O33" s="66"/>
+      <x:c r="P33" s="66"/>
+      <x:c r="Q33" s="66"/>
+      <x:c r="R33" s="66"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="66"/>
@@ -4058,6 +4250,10 @@
       <x:c r="L34" s="66"/>
       <x:c r="M34" s="66"/>
       <x:c r="N34" s="66"/>
+      <x:c r="O34" s="66"/>
+      <x:c r="P34" s="66"/>
+      <x:c r="Q34" s="66"/>
+      <x:c r="R34" s="66"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="66"/>
@@ -4074,6 +4270,10 @@
       <x:c r="L35" s="66"/>
       <x:c r="M35" s="66"/>
       <x:c r="N35" s="66"/>
+      <x:c r="O35" s="66"/>
+      <x:c r="P35" s="66"/>
+      <x:c r="Q35" s="66"/>
+      <x:c r="R35" s="66"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="66"/>
@@ -4090,6 +4290,10 @@
       <x:c r="L36" s="66"/>
       <x:c r="M36" s="66"/>
       <x:c r="N36" s="66"/>
+      <x:c r="O36" s="66"/>
+      <x:c r="P36" s="66"/>
+      <x:c r="Q36" s="66"/>
+      <x:c r="R36" s="66"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="66"/>
@@ -4106,6 +4310,10 @@
       <x:c r="L37" s="66"/>
       <x:c r="M37" s="66"/>
       <x:c r="N37" s="66"/>
+      <x:c r="O37" s="66"/>
+      <x:c r="P37" s="66"/>
+      <x:c r="Q37" s="66"/>
+      <x:c r="R37" s="66"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="66"/>
@@ -4122,6 +4330,10 @@
       <x:c r="L38" s="66"/>
       <x:c r="M38" s="66"/>
       <x:c r="N38" s="66"/>
+      <x:c r="O38" s="66"/>
+      <x:c r="P38" s="66"/>
+      <x:c r="Q38" s="66"/>
+      <x:c r="R38" s="66"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="66"/>
@@ -4138,6 +4350,10 @@
       <x:c r="L39" s="66"/>
       <x:c r="M39" s="66"/>
       <x:c r="N39" s="66"/>
+      <x:c r="O39" s="66"/>
+      <x:c r="P39" s="66"/>
+      <x:c r="Q39" s="66"/>
+      <x:c r="R39" s="66"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="66"/>
@@ -4154,6 +4370,10 @@
       <x:c r="L40" s="66"/>
       <x:c r="M40" s="66"/>
       <x:c r="N40" s="66"/>
+      <x:c r="O40" s="66"/>
+      <x:c r="P40" s="66"/>
+      <x:c r="Q40" s="66"/>
+      <x:c r="R40" s="66"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="66"/>
@@ -4170,6 +4390,10 @@
       <x:c r="L41" s="66"/>
       <x:c r="M41" s="66"/>
       <x:c r="N41" s="66"/>
+      <x:c r="O41" s="66"/>
+      <x:c r="P41" s="66"/>
+      <x:c r="Q41" s="66"/>
+      <x:c r="R41" s="66"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="66"/>
@@ -4186,6 +4410,10 @@
       <x:c r="L42" s="66"/>
       <x:c r="M42" s="66"/>
       <x:c r="N42" s="66"/>
+      <x:c r="O42" s="66"/>
+      <x:c r="P42" s="66"/>
+      <x:c r="Q42" s="66"/>
+      <x:c r="R42" s="66"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="66"/>
@@ -4202,6 +4430,10 @@
       <x:c r="L43" s="66"/>
       <x:c r="M43" s="66"/>
       <x:c r="N43" s="66"/>
+      <x:c r="O43" s="66"/>
+      <x:c r="P43" s="66"/>
+      <x:c r="Q43" s="66"/>
+      <x:c r="R43" s="66"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="66"/>
@@ -4218,6 +4450,10 @@
       <x:c r="L44" s="66"/>
       <x:c r="M44" s="66"/>
       <x:c r="N44" s="66"/>
+      <x:c r="O44" s="66"/>
+      <x:c r="P44" s="66"/>
+      <x:c r="Q44" s="66"/>
+      <x:c r="R44" s="66"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="66"/>
@@ -4234,6 +4470,10 @@
       <x:c r="L45" s="66"/>
       <x:c r="M45" s="66"/>
       <x:c r="N45" s="66"/>
+      <x:c r="O45" s="66"/>
+      <x:c r="P45" s="66"/>
+      <x:c r="Q45" s="66"/>
+      <x:c r="R45" s="66"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="66"/>
@@ -4250,6 +4490,10 @@
       <x:c r="L46" s="66"/>
       <x:c r="M46" s="66"/>
       <x:c r="N46" s="66"/>
+      <x:c r="O46" s="66"/>
+      <x:c r="P46" s="66"/>
+      <x:c r="Q46" s="66"/>
+      <x:c r="R46" s="66"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="66"/>
@@ -4266,6 +4510,10 @@
       <x:c r="L47" s="66"/>
       <x:c r="M47" s="66"/>
       <x:c r="N47" s="66"/>
+      <x:c r="O47" s="66"/>
+      <x:c r="P47" s="66"/>
+      <x:c r="Q47" s="66"/>
+      <x:c r="R47" s="66"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="66"/>
@@ -4282,6 +4530,10 @@
       <x:c r="L48" s="66"/>
       <x:c r="M48" s="66"/>
       <x:c r="N48" s="66"/>
+      <x:c r="O48" s="66"/>
+      <x:c r="P48" s="66"/>
+      <x:c r="Q48" s="66"/>
+      <x:c r="R48" s="66"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="66"/>
@@ -4298,6 +4550,10 @@
       <x:c r="L49" s="66"/>
       <x:c r="M49" s="66"/>
       <x:c r="N49" s="66"/>
+      <x:c r="O49" s="66"/>
+      <x:c r="P49" s="66"/>
+      <x:c r="Q49" s="66"/>
+      <x:c r="R49" s="66"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="66"/>
@@ -4314,6 +4570,10 @@
       <x:c r="L50" s="66"/>
       <x:c r="M50" s="66"/>
       <x:c r="N50" s="66"/>
+      <x:c r="O50" s="66"/>
+      <x:c r="P50" s="66"/>
+      <x:c r="Q50" s="66"/>
+      <x:c r="R50" s="66"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="66"/>
@@ -4330,6 +4590,10 @@
       <x:c r="L51" s="66"/>
       <x:c r="M51" s="66"/>
       <x:c r="N51" s="66"/>
+      <x:c r="O51" s="66"/>
+      <x:c r="P51" s="66"/>
+      <x:c r="Q51" s="66"/>
+      <x:c r="R51" s="66"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="66"/>
@@ -4346,6 +4610,10 @@
       <x:c r="L52" s="66"/>
       <x:c r="M52" s="66"/>
       <x:c r="N52" s="66"/>
+      <x:c r="O52" s="66"/>
+      <x:c r="P52" s="66"/>
+      <x:c r="Q52" s="66"/>
+      <x:c r="R52" s="66"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="66"/>
@@ -4362,6 +4630,10 @@
       <x:c r="L53" s="66"/>
       <x:c r="M53" s="66"/>
       <x:c r="N53" s="66"/>
+      <x:c r="O53" s="66"/>
+      <x:c r="P53" s="66"/>
+      <x:c r="Q53" s="66"/>
+      <x:c r="R53" s="66"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="66"/>
@@ -4378,6 +4650,10 @@
       <x:c r="L54" s="66"/>
       <x:c r="M54" s="66"/>
       <x:c r="N54" s="66"/>
+      <x:c r="O54" s="66"/>
+      <x:c r="P54" s="66"/>
+      <x:c r="Q54" s="66"/>
+      <x:c r="R54" s="66"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="66"/>
@@ -4394,6 +4670,10 @@
       <x:c r="L55" s="66"/>
       <x:c r="M55" s="66"/>
       <x:c r="N55" s="66"/>
+      <x:c r="O55" s="66"/>
+      <x:c r="P55" s="66"/>
+      <x:c r="Q55" s="66"/>
+      <x:c r="R55" s="66"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="66"/>
@@ -4410,6 +4690,10 @@
       <x:c r="L56" s="66"/>
       <x:c r="M56" s="66"/>
       <x:c r="N56" s="66"/>
+      <x:c r="O56" s="66"/>
+      <x:c r="P56" s="66"/>
+      <x:c r="Q56" s="66"/>
+      <x:c r="R56" s="66"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="66"/>
@@ -4426,6 +4710,10 @@
       <x:c r="L57" s="66"/>
       <x:c r="M57" s="66"/>
       <x:c r="N57" s="66"/>
+      <x:c r="O57" s="66"/>
+      <x:c r="P57" s="66"/>
+      <x:c r="Q57" s="66"/>
+      <x:c r="R57" s="66"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="66"/>
@@ -4442,6 +4730,10 @@
       <x:c r="L58" s="66"/>
       <x:c r="M58" s="66"/>
       <x:c r="N58" s="66"/>
+      <x:c r="O58" s="66"/>
+      <x:c r="P58" s="66"/>
+      <x:c r="Q58" s="66"/>
+      <x:c r="R58" s="66"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="66"/>
@@ -4458,6 +4750,10 @@
       <x:c r="L59" s="66"/>
       <x:c r="M59" s="66"/>
       <x:c r="N59" s="66"/>
+      <x:c r="O59" s="66"/>
+      <x:c r="P59" s="66"/>
+      <x:c r="Q59" s="66"/>
+      <x:c r="R59" s="66"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="66"/>
@@ -4474,6 +4770,10 @@
       <x:c r="L60" s="66"/>
       <x:c r="M60" s="66"/>
       <x:c r="N60" s="66"/>
+      <x:c r="O60" s="66"/>
+      <x:c r="P60" s="66"/>
+      <x:c r="Q60" s="66"/>
+      <x:c r="R60" s="66"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="66"/>
@@ -4490,6 +4790,10 @@
       <x:c r="L61" s="66"/>
       <x:c r="M61" s="66"/>
       <x:c r="N61" s="66"/>
+      <x:c r="O61" s="66"/>
+      <x:c r="P61" s="66"/>
+      <x:c r="Q61" s="66"/>
+      <x:c r="R61" s="66"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="66"/>
@@ -4506,6 +4810,10 @@
       <x:c r="L62" s="66"/>
       <x:c r="M62" s="66"/>
       <x:c r="N62" s="66"/>
+      <x:c r="O62" s="66"/>
+      <x:c r="P62" s="66"/>
+      <x:c r="Q62" s="66"/>
+      <x:c r="R62" s="66"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="66"/>
@@ -4522,6 +4830,10 @@
       <x:c r="L63" s="66"/>
       <x:c r="M63" s="66"/>
       <x:c r="N63" s="66"/>
+      <x:c r="O63" s="66"/>
+      <x:c r="P63" s="66"/>
+      <x:c r="Q63" s="66"/>
+      <x:c r="R63" s="66"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="66"/>
@@ -4538,6 +4850,10 @@
       <x:c r="L64" s="66"/>
       <x:c r="M64" s="66"/>
       <x:c r="N64" s="66"/>
+      <x:c r="O64" s="66"/>
+      <x:c r="P64" s="66"/>
+      <x:c r="Q64" s="66"/>
+      <x:c r="R64" s="66"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="66"/>
@@ -4554,6 +4870,10 @@
       <x:c r="L65" s="66"/>
       <x:c r="M65" s="66"/>
       <x:c r="N65" s="66"/>
+      <x:c r="O65" s="66"/>
+      <x:c r="P65" s="66"/>
+      <x:c r="Q65" s="66"/>
+      <x:c r="R65" s="66"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="66"/>
@@ -4570,6 +4890,10 @@
       <x:c r="L66" s="66"/>
       <x:c r="M66" s="66"/>
       <x:c r="N66" s="66"/>
+      <x:c r="O66" s="66"/>
+      <x:c r="P66" s="66"/>
+      <x:c r="Q66" s="66"/>
+      <x:c r="R66" s="66"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="66"/>
@@ -4586,6 +4910,10 @@
       <x:c r="L67" s="66"/>
       <x:c r="M67" s="66"/>
       <x:c r="N67" s="66"/>
+      <x:c r="O67" s="66"/>
+      <x:c r="P67" s="66"/>
+      <x:c r="Q67" s="66"/>
+      <x:c r="R67" s="66"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="66"/>
@@ -4602,6 +4930,10 @@
       <x:c r="L68" s="66"/>
       <x:c r="M68" s="66"/>
       <x:c r="N68" s="66"/>
+      <x:c r="O68" s="66"/>
+      <x:c r="P68" s="66"/>
+      <x:c r="Q68" s="66"/>
+      <x:c r="R68" s="66"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="66"/>
@@ -4618,6 +4950,10 @@
       <x:c r="L69" s="66"/>
       <x:c r="M69" s="66"/>
       <x:c r="N69" s="66"/>
+      <x:c r="O69" s="66"/>
+      <x:c r="P69" s="66"/>
+      <x:c r="Q69" s="66"/>
+      <x:c r="R69" s="66"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="66"/>
@@ -4634,6 +4970,10 @@
       <x:c r="L70" s="66"/>
       <x:c r="M70" s="66"/>
       <x:c r="N70" s="66"/>
+      <x:c r="O70" s="66"/>
+      <x:c r="P70" s="66"/>
+      <x:c r="Q70" s="66"/>
+      <x:c r="R70" s="66"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="66"/>
@@ -4650,6 +4990,10 @@
       <x:c r="L71" s="66"/>
       <x:c r="M71" s="66"/>
       <x:c r="N71" s="66"/>
+      <x:c r="O71" s="66"/>
+      <x:c r="P71" s="66"/>
+      <x:c r="Q71" s="66"/>
+      <x:c r="R71" s="66"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="66"/>
@@ -4666,6 +5010,10 @@
       <x:c r="L72" s="66"/>
       <x:c r="M72" s="66"/>
       <x:c r="N72" s="66"/>
+      <x:c r="O72" s="66"/>
+      <x:c r="P72" s="66"/>
+      <x:c r="Q72" s="66"/>
+      <x:c r="R72" s="66"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="66"/>
@@ -4682,6 +5030,10 @@
       <x:c r="L73" s="66"/>
       <x:c r="M73" s="66"/>
       <x:c r="N73" s="66"/>
+      <x:c r="O73" s="66"/>
+      <x:c r="P73" s="66"/>
+      <x:c r="Q73" s="66"/>
+      <x:c r="R73" s="66"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="66"/>
@@ -4698,6 +5050,10 @@
       <x:c r="L74" s="66"/>
       <x:c r="M74" s="66"/>
       <x:c r="N74" s="66"/>
+      <x:c r="O74" s="66"/>
+      <x:c r="P74" s="66"/>
+      <x:c r="Q74" s="66"/>
+      <x:c r="R74" s="66"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="66"/>
@@ -4714,6 +5070,10 @@
       <x:c r="L75" s="66"/>
       <x:c r="M75" s="66"/>
       <x:c r="N75" s="66"/>
+      <x:c r="O75" s="66"/>
+      <x:c r="P75" s="66"/>
+      <x:c r="Q75" s="66"/>
+      <x:c r="R75" s="66"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="66"/>
@@ -4730,6 +5090,10 @@
       <x:c r="L76" s="66"/>
       <x:c r="M76" s="66"/>
       <x:c r="N76" s="66"/>
+      <x:c r="O76" s="66"/>
+      <x:c r="P76" s="66"/>
+      <x:c r="Q76" s="66"/>
+      <x:c r="R76" s="66"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="66"/>
@@ -4746,6 +5110,10 @@
       <x:c r="L77" s="66"/>
       <x:c r="M77" s="66"/>
       <x:c r="N77" s="66"/>
+      <x:c r="O77" s="66"/>
+      <x:c r="P77" s="66"/>
+      <x:c r="Q77" s="66"/>
+      <x:c r="R77" s="66"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="66"/>
@@ -4762,6 +5130,10 @@
       <x:c r="L78" s="66"/>
       <x:c r="M78" s="66"/>
       <x:c r="N78" s="66"/>
+      <x:c r="O78" s="66"/>
+      <x:c r="P78" s="66"/>
+      <x:c r="Q78" s="66"/>
+      <x:c r="R78" s="66"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="66"/>
@@ -4778,6 +5150,10 @@
       <x:c r="L79" s="66"/>
       <x:c r="M79" s="66"/>
       <x:c r="N79" s="66"/>
+      <x:c r="O79" s="66"/>
+      <x:c r="P79" s="66"/>
+      <x:c r="Q79" s="66"/>
+      <x:c r="R79" s="66"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="66"/>
@@ -4794,6 +5170,10 @@
       <x:c r="L80" s="66"/>
       <x:c r="M80" s="66"/>
       <x:c r="N80" s="66"/>
+      <x:c r="O80" s="66"/>
+      <x:c r="P80" s="66"/>
+      <x:c r="Q80" s="66"/>
+      <x:c r="R80" s="66"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="66"/>
@@ -4810,6 +5190,10 @@
       <x:c r="L81" s="66"/>
       <x:c r="M81" s="66"/>
       <x:c r="N81" s="66"/>
+      <x:c r="O81" s="66"/>
+      <x:c r="P81" s="66"/>
+      <x:c r="Q81" s="66"/>
+      <x:c r="R81" s="66"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="66"/>
@@ -4826,6 +5210,10 @@
       <x:c r="L82" s="66"/>
       <x:c r="M82" s="66"/>
       <x:c r="N82" s="66"/>
+      <x:c r="O82" s="66"/>
+      <x:c r="P82" s="66"/>
+      <x:c r="Q82" s="66"/>
+      <x:c r="R82" s="66"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="66"/>
@@ -4842,6 +5230,10 @@
       <x:c r="L83" s="66"/>
       <x:c r="M83" s="66"/>
       <x:c r="N83" s="66"/>
+      <x:c r="O83" s="66"/>
+      <x:c r="P83" s="66"/>
+      <x:c r="Q83" s="66"/>
+      <x:c r="R83" s="66"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="66"/>
@@ -4858,6 +5250,10 @@
       <x:c r="L84" s="66"/>
       <x:c r="M84" s="66"/>
       <x:c r="N84" s="66"/>
+      <x:c r="O84" s="66"/>
+      <x:c r="P84" s="66"/>
+      <x:c r="Q84" s="66"/>
+      <x:c r="R84" s="66"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="66"/>
@@ -4874,6 +5270,10 @@
       <x:c r="L85" s="66"/>
       <x:c r="M85" s="66"/>
       <x:c r="N85" s="66"/>
+      <x:c r="O85" s="66"/>
+      <x:c r="P85" s="66"/>
+      <x:c r="Q85" s="66"/>
+      <x:c r="R85" s="66"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="66"/>
@@ -4890,6 +5290,10 @@
       <x:c r="L86" s="66"/>
       <x:c r="M86" s="66"/>
       <x:c r="N86" s="66"/>
+      <x:c r="O86" s="66"/>
+      <x:c r="P86" s="66"/>
+      <x:c r="Q86" s="66"/>
+      <x:c r="R86" s="66"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="66"/>
@@ -4906,6 +5310,10 @@
       <x:c r="L87" s="66"/>
       <x:c r="M87" s="66"/>
       <x:c r="N87" s="66"/>
+      <x:c r="O87" s="66"/>
+      <x:c r="P87" s="66"/>
+      <x:c r="Q87" s="66"/>
+      <x:c r="R87" s="66"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="66"/>
@@ -4922,6 +5330,10 @@
       <x:c r="L88" s="66"/>
       <x:c r="M88" s="66"/>
       <x:c r="N88" s="66"/>
+      <x:c r="O88" s="66"/>
+      <x:c r="P88" s="66"/>
+      <x:c r="Q88" s="66"/>
+      <x:c r="R88" s="66"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="66"/>
@@ -4938,6 +5350,10 @@
       <x:c r="L89" s="66"/>
       <x:c r="M89" s="66"/>
       <x:c r="N89" s="66"/>
+      <x:c r="O89" s="66"/>
+      <x:c r="P89" s="66"/>
+      <x:c r="Q89" s="66"/>
+      <x:c r="R89" s="66"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="66"/>
@@ -4954,6 +5370,10 @@
       <x:c r="L90" s="66"/>
       <x:c r="M90" s="66"/>
       <x:c r="N90" s="66"/>
+      <x:c r="O90" s="66"/>
+      <x:c r="P90" s="66"/>
+      <x:c r="Q90" s="66"/>
+      <x:c r="R90" s="66"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="66"/>
@@ -4970,6 +5390,10 @@
       <x:c r="L91" s="66"/>
       <x:c r="M91" s="66"/>
       <x:c r="N91" s="66"/>
+      <x:c r="O91" s="66"/>
+      <x:c r="P91" s="66"/>
+      <x:c r="Q91" s="66"/>
+      <x:c r="R91" s="66"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="66"/>
@@ -4986,6 +5410,10 @@
       <x:c r="L92" s="66"/>
       <x:c r="M92" s="66"/>
       <x:c r="N92" s="66"/>
+      <x:c r="O92" s="66"/>
+      <x:c r="P92" s="66"/>
+      <x:c r="Q92" s="66"/>
+      <x:c r="R92" s="66"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="66"/>
@@ -5002,6 +5430,10 @@
       <x:c r="L93" s="66"/>
       <x:c r="M93" s="66"/>
       <x:c r="N93" s="66"/>
+      <x:c r="O93" s="66"/>
+      <x:c r="P93" s="66"/>
+      <x:c r="Q93" s="66"/>
+      <x:c r="R93" s="66"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="66"/>
@@ -5018,6 +5450,10 @@
       <x:c r="L94" s="66"/>
       <x:c r="M94" s="66"/>
       <x:c r="N94" s="66"/>
+      <x:c r="O94" s="66"/>
+      <x:c r="P94" s="66"/>
+      <x:c r="Q94" s="66"/>
+      <x:c r="R94" s="66"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="66"/>
@@ -5034,6 +5470,10 @@
       <x:c r="L95" s="66"/>
       <x:c r="M95" s="66"/>
       <x:c r="N95" s="66"/>
+      <x:c r="O95" s="66"/>
+      <x:c r="P95" s="66"/>
+      <x:c r="Q95" s="66"/>
+      <x:c r="R95" s="66"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="66"/>
@@ -5050,6 +5490,10 @@
       <x:c r="L96" s="66"/>
       <x:c r="M96" s="66"/>
       <x:c r="N96" s="66"/>
+      <x:c r="O96" s="66"/>
+      <x:c r="P96" s="66"/>
+      <x:c r="Q96" s="66"/>
+      <x:c r="R96" s="66"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="66"/>
@@ -5066,6 +5510,10 @@
       <x:c r="L97" s="66"/>
       <x:c r="M97" s="66"/>
       <x:c r="N97" s="66"/>
+      <x:c r="O97" s="66"/>
+      <x:c r="P97" s="66"/>
+      <x:c r="Q97" s="66"/>
+      <x:c r="R97" s="66"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="66"/>
@@ -5082,6 +5530,10 @@
       <x:c r="L98" s="66"/>
       <x:c r="M98" s="66"/>
       <x:c r="N98" s="66"/>
+      <x:c r="O98" s="66"/>
+      <x:c r="P98" s="66"/>
+      <x:c r="Q98" s="66"/>
+      <x:c r="R98" s="66"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="66"/>
@@ -5098,6 +5550,10 @@
       <x:c r="L99" s="66"/>
       <x:c r="M99" s="66"/>
       <x:c r="N99" s="66"/>
+      <x:c r="O99" s="66"/>
+      <x:c r="P99" s="66"/>
+      <x:c r="Q99" s="66"/>
+      <x:c r="R99" s="66"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="66"/>
@@ -5114,6 +5570,10 @@
       <x:c r="L100" s="66"/>
       <x:c r="M100" s="66"/>
       <x:c r="N100" s="66"/>
+      <x:c r="O100" s="66"/>
+      <x:c r="P100" s="66"/>
+      <x:c r="Q100" s="66"/>
+      <x:c r="R100" s="66"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="66"/>
@@ -5130,6 +5590,10 @@
       <x:c r="L101" s="66"/>
       <x:c r="M101" s="66"/>
       <x:c r="N101" s="66"/>
+      <x:c r="O101" s="66"/>
+      <x:c r="P101" s="66"/>
+      <x:c r="Q101" s="66"/>
+      <x:c r="R101" s="66"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="66"/>
@@ -5146,6 +5610,10 @@
       <x:c r="L102" s="66"/>
       <x:c r="M102" s="66"/>
       <x:c r="N102" s="66"/>
+      <x:c r="O102" s="66"/>
+      <x:c r="P102" s="66"/>
+      <x:c r="Q102" s="66"/>
+      <x:c r="R102" s="66"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="66"/>
@@ -5162,6 +5630,10 @@
       <x:c r="L103" s="66"/>
       <x:c r="M103" s="66"/>
       <x:c r="N103" s="66"/>
+      <x:c r="O103" s="66"/>
+      <x:c r="P103" s="66"/>
+      <x:c r="Q103" s="66"/>
+      <x:c r="R103" s="66"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="66"/>
@@ -5178,6 +5650,10 @@
       <x:c r="L104" s="66"/>
       <x:c r="M104" s="66"/>
       <x:c r="N104" s="66"/>
+      <x:c r="O104" s="66"/>
+      <x:c r="P104" s="66"/>
+      <x:c r="Q104" s="66"/>
+      <x:c r="R104" s="66"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="66"/>
@@ -5194,6 +5670,10 @@
       <x:c r="L105" s="66"/>
       <x:c r="M105" s="66"/>
       <x:c r="N105" s="66"/>
+      <x:c r="O105" s="66"/>
+      <x:c r="P105" s="66"/>
+      <x:c r="Q105" s="66"/>
+      <x:c r="R105" s="66"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="66"/>
@@ -5210,6 +5690,10 @@
       <x:c r="L106" s="66"/>
       <x:c r="M106" s="66"/>
       <x:c r="N106" s="66"/>
+      <x:c r="O106" s="66"/>
+      <x:c r="P106" s="66"/>
+      <x:c r="Q106" s="66"/>
+      <x:c r="R106" s="66"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="66"/>
@@ -5226,6 +5710,10 @@
       <x:c r="L107" s="66"/>
       <x:c r="M107" s="66"/>
       <x:c r="N107" s="66"/>
+      <x:c r="O107" s="66"/>
+      <x:c r="P107" s="66"/>
+      <x:c r="Q107" s="66"/>
+      <x:c r="R107" s="66"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="66"/>
@@ -5242,6 +5730,10 @@
       <x:c r="L108" s="66"/>
       <x:c r="M108" s="66"/>
       <x:c r="N108" s="66"/>
+      <x:c r="O108" s="66"/>
+      <x:c r="P108" s="66"/>
+      <x:c r="Q108" s="66"/>
+      <x:c r="R108" s="66"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="66"/>
@@ -5258,6 +5750,10 @@
       <x:c r="L109" s="66"/>
       <x:c r="M109" s="66"/>
       <x:c r="N109" s="66"/>
+      <x:c r="O109" s="66"/>
+      <x:c r="P109" s="66"/>
+      <x:c r="Q109" s="66"/>
+      <x:c r="R109" s="66"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="66"/>
@@ -5274,28 +5770,35 @@
       <x:c r="L110" s="66"/>
       <x:c r="M110" s="66"/>
       <x:c r="N110" s="66"/>
+      <x:c r="O110" s="66"/>
+      <x:c r="P110" s="66"/>
+      <x:c r="Q110" s="66"/>
+      <x:c r="R110" s="66"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:N1"/>
-    <x:mergeCell ref="A2:N2"/>
+    <x:mergeCell ref="A1:R1"/>
+    <x:mergeCell ref="A2:R2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="M6:M110">
+  <x:conditionalFormatting sqref="Q6:Q110">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="待"/>
     <x:cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="有效"/>
     <x:cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="无效"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B6:B110">
       <x:formula1>"US-旗舰店,US-日用店,TH-主店,新增店铺"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="M6:M110">
+    <x:dataValidation type="list" sqref="O6:O110">
+      <x:formula1>"T+1,T+3,T+7"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="Q6:Q110">
       <x:formula1>"表现良好,需观察,需处理,待填写"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a48519337a34dc8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d995f15a71a4473"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7022,7 +7525,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R597d75af76c2406c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc47f75886464763"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7763,7 +8266,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e70a32fc3584d0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb80a17cbe2f3445e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8821,7 +9324,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bcf100ade0d4592"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R537fcc7cba164373"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10373,7 +10876,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb3465b939e94dab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd76e507cf5d84112"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11534,7 +12037,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f86a987fd6d4652"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2854c84570f643d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11635,13 +12138,13 @@
     </x:row>
     <x:row r="9" ht="21" customHeight="1">
       <x:c r="A9" s="38" t="str">
-        <x:v>CVR(%)</x:v>
+        <x:v>曝光/CTR/CVR变化</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
         <x:v>商品数据</x:v>
       </x:c>
       <x:c r="C9" s="7" t="str">
-        <x:v>例如 3.86 表示 3.86%；缺失留空。</x:v>
+        <x:v>按上一周期或验证节点填写变化；曝光/GMV用百分比，CTR/CVR用百分点；缺失留空。</x:v>
       </x:c>
       <x:c r="D9" s="74" t="str">
         <x:v>黄色输入</x:v>
@@ -11649,29 +12152,43 @@
     </x:row>
     <x:row r="10" ht="21" customHeight="1">
       <x:c r="A10" s="38" t="str">
-        <x:v>验证状态</x:v>
+        <x:v>预警节点</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>运营动作</x:v>
+        <x:v>商品数据</x:v>
       </x:c>
       <x:c r="C10" s="7" t="str">
-        <x:v>只有真实 T+1/T+3/T+7 证据才能填有效或无效。</x:v>
+        <x:v>使用 T+1、T+3、T+7 标记异常数据的核查节点。</x:v>
       </x:c>
       <x:c r="D10" s="74" t="str">
         <x:v>黄色输入</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="21" customHeight="1">
-      <x:c r="A11" s="85" t="str">
+      <x:c r="A11" s="38" t="str">
+        <x:v>验证状态</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="str">
+        <x:v>运营动作</x:v>
+      </x:c>
+      <x:c r="C11" s="7" t="str">
+        <x:v>只有真实 T+1/T+3/T+7 证据才能填有效或无效。</x:v>
+      </x:c>
+      <x:c r="D11" s="74" t="str">
+        <x:v>黄色输入</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="21" customHeight="1">
+      <x:c r="A12" s="85" t="str">
         <x:v>动作进度</x:v>
       </x:c>
-      <x:c r="B11" s="86" t="str">
+      <x:c r="B12" s="86" t="str">
         <x:v>店铺日汇总</x:v>
       </x:c>
-      <x:c r="C11" s="86" t="str">
+      <x:c r="C12" s="86" t="str">
         <x:v>例如 6 / 9；表示有效验证数 / 总动作数。</x:v>
       </x:c>
-      <x:c r="D11" s="76" t="str">
+      <x:c r="D12" s="76" t="str">
         <x:v>黄色输入</x:v>
       </x:c>
     </x:row>
@@ -11682,7 +12199,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fa1c2256cfe49f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c087ed893e549b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add v3 WPS Kdocs data document
</commit_message>
<xml_diff>
--- a/data/tiktok-ai-operations-center-wps-kdocs-template.xlsx
+++ b/data/tiktok-ai-operations-center-wps-kdocs-template.xlsx
@@ -2,15 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填报首页" sheetId="1" r:id="R158f1106a3d14e7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺日汇总" sheetId="2" r:id="R5d4c54b3c7cb4c43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商品数据" sheetId="3" r:id="R9254024da00e430e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营动作" sheetId="4" r:id="Rbf9426a7fb904050"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布趋势" sheetId="5" r:id="R90ea4999689c4ceb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD达人" sheetId="6" r:id="R2c2343c8512644a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="广告计划" sheetId="7" r:id="R2ef7a71a7ef44009"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="短视频数据" sheetId="8" r:id="Re1283371afe44f88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段字典" sheetId="9" r:id="R17071b1b50f8497a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填报首页" sheetId="1" r:id="Re4c4734162514bd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺日汇总" sheetId="2" r:id="R4873af065775491d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商品数据" sheetId="3" r:id="R3ef20b9028c647c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营动作" sheetId="4" r:id="Rd9ce15900f2d436c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布趋势" sheetId="5" r:id="R7d7a0bf6a2194a7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD达人" sheetId="6" r:id="Rfdb542c1e7aa446b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="广告计划" sheetId="7" r:id="R48c0e4bfa0ee4fa1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="短视频数据" sheetId="8" r:id="Rbba2111c7d0341df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段字典" sheetId="9" r:id="Ra5771170fc40468a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺字典" sheetId="10" r:id="R4bc46cdc8f3346f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="五组排行" sheetId="11" r:id="R7db5de9247b24b30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="预警规则" sheetId="12" r:id="R25ad1ab0282f435f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营知识库" sheetId="13" r:id="R82cd823e47c14ed7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent调度" sheetId="14" r:id="R9316d242fa2f4567"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,15 +26,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="8">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="¥#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0.00"/>
     <x:numFmt numFmtId="203" formatCode="#,##0"/>
     <x:numFmt numFmtId="204" formatCode="0.0"/>
     <x:numFmt numFmtId="205" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="206" formatCode="&quot;¥&quot;#,##0"/>
+    <x:numFmt numFmtId="207" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -66,8 +73,47 @@
       <x:color rgb="FF9A6700"/>
       <x:name val="Microsoft YaHei"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF64748B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1E3A8A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF0F172A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1E3A8A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="13"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF92400E"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -107,6 +153,56 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF4DE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1E3A8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEFF6FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1E3A8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEFF6FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -196,7 +292,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="88">
+  <x:cellXfs count="145">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -441,6 +537,107 @@
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="9" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="10" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="10" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="10" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="10" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="10" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="10" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -451,7 +648,7 @@
         <x:color rgb="FF9A6700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4DE"/>
         </x:patternFill>
       </x:fill>
@@ -461,7 +658,7 @@
         <x:color rgb="FF07865A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F7F0"/>
         </x:patternFill>
       </x:fill>
@@ -471,7 +668,7 @@
         <x:color rgb="FFD64545"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0F0"/>
         </x:patternFill>
       </x:fill>
@@ -481,7 +678,7 @@
         <x:color rgb="FF9A6700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4DE"/>
         </x:patternFill>
       </x:fill>
@@ -491,7 +688,7 @@
         <x:color rgb="FF07865A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F7F0"/>
         </x:patternFill>
       </x:fill>
@@ -501,7 +698,7 @@
         <x:color rgb="FFD64545"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0F0"/>
         </x:patternFill>
       </x:fill>
@@ -511,7 +708,7 @@
         <x:color rgb="FF9A6700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4DE"/>
         </x:patternFill>
       </x:fill>
@@ -521,7 +718,7 @@
         <x:color rgb="FF07865A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F7F0"/>
         </x:patternFill>
       </x:fill>
@@ -531,7 +728,7 @@
         <x:color rgb="FFD64545"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0F0"/>
         </x:patternFill>
       </x:fill>
@@ -541,7 +738,7 @@
         <x:color rgb="FF9A6700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4DE"/>
         </x:patternFill>
       </x:fill>
@@ -551,7 +748,7 @@
         <x:color rgb="FF07865A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F7F0"/>
         </x:patternFill>
       </x:fill>
@@ -561,7 +758,7 @@
         <x:color rgb="FFD64545"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0F0"/>
         </x:patternFill>
       </x:fill>
@@ -571,7 +768,7 @@
         <x:color rgb="FF9A6700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4DE"/>
         </x:patternFill>
       </x:fill>
@@ -581,7 +778,7 @@
         <x:color rgb="FF07865A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F7F0"/>
         </x:patternFill>
       </x:fill>
@@ -591,7 +788,7 @@
         <x:color rgb="FFD64545"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0F0"/>
         </x:patternFill>
       </x:fill>
@@ -618,6 +815,144 @@
     <x:tableColumn id="12" name="动作进度"/>
     <x:tableColumn id="13" name="数据状态"/>
     <x:tableColumn id="14" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="StoreDictionaryTable" displayName="StoreDictionaryTable" ref="A5:D9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="店铺名称"/>
+    <x:tableColumn id="2" name="店铺编码"/>
+    <x:tableColumn id="3" name="市场/用途"/>
+    <x:tableColumn id="4" name="状态"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="SalesTop5Table" displayName="SalesTop5Table" ref="A5:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="GMVTop5Table" displayName="GMVTop5Table" ref="A13:F18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="GMVUpTop5Table" displayName="GMVUpTop5Table" ref="A21:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="GMVDownTop5Table" displayName="GMVDownTop5Table" ref="A29:F34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="CVRDownTop5Table" displayName="CVRDownTop5Table" ref="A37:F42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="SalesTop5Table" displayName="SalesTop5Table" ref="A5:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="GMVTop5Table" displayName="GMVTop5Table" ref="A13:F18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="GMVUpTop5Table" displayName="GMVUpTop5Table" ref="A21:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="GMVDownTop5Table" displayName="GMVDownTop5Table" ref="A29:F34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -650,6 +985,151 @@
 </x:table>
 </file>
 
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="CVRDownTop5Table" displayName="CVRDownTop5Table" ref="A37:F42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="WarningRulesTable" displayName="WarningRulesTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="预警指标"/>
+    <x:tableColumn id="2" name="触发条件"/>
+    <x:tableColumn id="3" name="建议节点"/>
+    <x:tableColumn id="4" name="启用"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="WarningSummaryTable" displayName="WarningSummaryTable" ref="F5:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="汇总指标"/>
+    <x:tableColumn id="2" name="当前值"/>
+    <x:tableColumn id="3" name="说明"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="WarningQueueTable" displayName="WarningQueueTable" ref="A13:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="商品ID"/>
+    <x:tableColumn id="2" name="店铺"/>
+    <x:tableColumn id="3" name="预警类型"/>
+    <x:tableColumn id="4" name="当前指标"/>
+    <x:tableColumn id="5" name="变化值"/>
+    <x:tableColumn id="6" name="建议动作"/>
+    <x:tableColumn id="7" name="处理状态"/>
+    <x:tableColumn id="8" name="证据/备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="WarningRulesTable" displayName="WarningRulesTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="预警指标"/>
+    <x:tableColumn id="2" name="触发条件"/>
+    <x:tableColumn id="3" name="建议节点"/>
+    <x:tableColumn id="4" name="启用"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="WarningSummaryTable" displayName="WarningSummaryTable" ref="F5:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="汇总指标"/>
+    <x:tableColumn id="2" name="当前值"/>
+    <x:tableColumn id="3" name="说明"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WarningQueueTable" displayName="WarningQueueTable" ref="A13:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="商品ID"/>
+    <x:tableColumn id="2" name="店铺"/>
+    <x:tableColumn id="3" name="预警类型"/>
+    <x:tableColumn id="4" name="当前指标"/>
+    <x:tableColumn id="5" name="变化值"/>
+    <x:tableColumn id="6" name="建议动作"/>
+    <x:tableColumn id="7" name="处理状态"/>
+    <x:tableColumn id="8" name="证据/备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="方法ID"/>
+    <x:tableColumn id="2" name="方法标题"/>
+    <x:tableColumn id="3" name="分类"/>
+    <x:tableColumn id="4" name="适用场景"/>
+    <x:tableColumn id="5" name="验证商品/对象"/>
+    <x:tableColumn id="6" name="证据摘要"/>
+    <x:tableColumn id="7" name="验证状态"/>
+    <x:tableColumn id="8" name="负责人"/>
+    <x:tableColumn id="9" name="复用次数"/>
+    <x:tableColumn id="10" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="方法ID"/>
+    <x:tableColumn id="2" name="方法标题"/>
+    <x:tableColumn id="3" name="分类"/>
+    <x:tableColumn id="4" name="适用场景"/>
+    <x:tableColumn id="5" name="验证商品/对象"/>
+    <x:tableColumn id="6" name="证据摘要"/>
+    <x:tableColumn id="7" name="验证状态"/>
+    <x:tableColumn id="8" name="负责人"/>
+    <x:tableColumn id="9" name="复用次数"/>
+    <x:tableColumn id="10" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="AgentDispatchTable" displayName="AgentDispatchTable" ref="A5:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="任务日期"/>
+    <x:tableColumn id="2" name="Agent名称"/>
+    <x:tableColumn id="3" name="触发入口"/>
+    <x:tableColumn id="4" name="输入范围"/>
+    <x:tableColumn id="5" name="任务目标"/>
+    <x:tableColumn id="6" name="输出物"/>
+    <x:tableColumn id="7" name="状态"/>
+    <x:tableColumn id="8" name="复核人"/>
+    <x:tableColumn id="9" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ActionsTable" displayName="ActionsTable" ref="A5:L10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:L10"/>
@@ -666,6 +1146,23 @@
     <x:tableColumn id="10" name="验证证据"/>
     <x:tableColumn id="11" name="是否已执行"/>
     <x:tableColumn id="12" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="AgentDispatchTable" displayName="AgentDispatchTable" ref="A5:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="任务日期"/>
+    <x:tableColumn id="2" name="Agent名称"/>
+    <x:tableColumn id="3" name="触发入口"/>
+    <x:tableColumn id="4" name="输入范围"/>
+    <x:tableColumn id="5" name="任务目标"/>
+    <x:tableColumn id="6" name="输出物"/>
+    <x:tableColumn id="7" name="状态"/>
+    <x:tableColumn id="8" name="复核人"/>
+    <x:tableColumn id="9" name="备注"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -745,6 +1242,18 @@
     <x:tableColumn id="2" name="所在表"/>
     <x:tableColumn id="3" name="填写口径"/>
     <x:tableColumn id="4" name="字段属性"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="StoreDictionaryTable" displayName="StoreDictionaryTable" ref="A5:D9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="店铺名称"/>
+    <x:tableColumn id="2" name="店铺编码"/>
+    <x:tableColumn id="3" name="市场/用途"/>
+    <x:tableColumn id="4" name="状态"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -947,8 +1456,8 @@
   <x:cols>
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="4" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
@@ -1156,14 +1665,1887 @@
       <x:c r="G14" s="19"/>
       <x:c r="H14" s="19"/>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="141" t="str">
+        <x:v>v3 网站数据接入工作流</x:v>
+      </x:c>
+      <x:c r="B16" s="141"/>
+      <x:c r="C16" s="141"/>
+      <x:c r="D16" s="141"/>
+      <x:c r="E16" s="141"/>
+      <x:c r="F16" s="141"/>
+      <x:c r="G16" s="141"/>
+      <x:c r="H16" s="141"/>
+    </x:row>
+    <x:row r="17" ht="32" customHeight="1">
+      <x:c r="A17" s="142" t="str">
+        <x:v>步骤</x:v>
+      </x:c>
+      <x:c r="B17" s="142" t="str">
+        <x:v>运营操作</x:v>
+      </x:c>
+      <x:c r="C17" s="142" t="str">
+        <x:v>涉及工作表</x:v>
+      </x:c>
+      <x:c r="D17" s="142" t="str">
+        <x:v>网站对应页面</x:v>
+      </x:c>
+      <x:c r="E17"/>
+      <x:c r="F17"/>
+      <x:c r="G17"/>
+      <x:c r="H17"/>
+    </x:row>
+    <x:row r="18" ht="32" customHeight="1">
+      <x:c r="A18" s="143" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B18" s="143" t="str">
+        <x:v>上传到 WPS/Kdocs，设置团队协作权限</x:v>
+      </x:c>
+      <x:c r="C18" s="143" t="str">
+        <x:v>整本工作簿</x:v>
+      </x:c>
+      <x:c r="D18" s="143" t="str">
+        <x:v>数据接入</x:v>
+      </x:c>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
+      <x:c r="G18"/>
+      <x:c r="H18"/>
+    </x:row>
+    <x:row r="19" ht="32" customHeight="1">
+      <x:c r="A19" s="143" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B19" s="143" t="str">
+        <x:v>先维护店铺字典，再填写店铺、商品和动作数据</x:v>
+      </x:c>
+      <x:c r="C19" s="143" t="str">
+        <x:v>店铺字典 / 店铺日汇总 / 商品数据 / 运营动作</x:v>
+      </x:c>
+      <x:c r="D19" s="143" t="str">
+        <x:v>经营总览 / 商品数据预警</x:v>
+      </x:c>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+      <x:c r="G19"/>
+      <x:c r="H19"/>
+    </x:row>
+    <x:row r="20" ht="32" customHeight="1">
+      <x:c r="A20" s="143" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B20" s="143" t="str">
+        <x:v>核对五组排行、预警队列、Agent 任务和知识库</x:v>
+      </x:c>
+      <x:c r="C20" s="143" t="str">
+        <x:v>五组排行 / 预警规则 / Agent调度 / 运营知识库</x:v>
+      </x:c>
+      <x:c r="D20" s="143" t="str">
+        <x:v>经营总览 / Agent 调度中心 / 运营知识库</x:v>
+      </x:c>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
+      <x:c r="G20"/>
+      <x:c r="H20"/>
+    </x:row>
+    <x:row r="21" ht="32" customHeight="1">
+      <x:c r="A21" s="143" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B21" s="143" t="str">
+        <x:v>导出 CSV 或接入后端 API；静态 GitHub Pages 不会自动读取私有文档</x:v>
+      </x:c>
+      <x:c r="C21" s="143" t="str">
+        <x:v>按字段字典映射</x:v>
+      </x:c>
+      <x:c r="D21" s="143" t="str">
+        <x:v>数据接入</x:v>
+      </x:c>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
+      <x:c r="G21"/>
+      <x:c r="H21"/>
+    </x:row>
+    <x:row r="23" ht="36" customHeight="1">
+      <x:c r="A23" s="144" t="str">
+        <x:v>重要说明：当前公开 v3 网站仍是主管提供的静态演示版；本工作簿已作为 WPS/Kdocs 统一填报源整理好，但要让真实数据自动驱动网页，仍需后端同步/API 和权限控制。</x:v>
+      </x:c>
+      <x:c r="B23" s="144"/>
+      <x:c r="C23" s="144"/>
+      <x:c r="D23" s="144"/>
+      <x:c r="E23" s="144"/>
+      <x:c r="F23" s="144"/>
+      <x:c r="G23" s="144"/>
+      <x:c r="H23" s="144"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
     <x:mergeCell ref="A12:H12"/>
     <x:mergeCell ref="A14:H14"/>
+    <x:mergeCell ref="A16:H16"/>
+    <x:mergeCell ref="A23:H23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="127" t="str">
+        <x:v>店铺字典｜网站筛选来源</x:v>
+      </x:c>
+      <x:c r="B1" s="127"/>
+      <x:c r="C1" s="127"/>
+      <x:c r="D1" s="127"/>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="128" t="str">
+        <x:v>真实店铺上线前请把黄色示例名称替换为团队实际店铺；“全部店铺”只作为汇总口径，不是一个真实店铺。</x:v>
+      </x:c>
+      <x:c r="B2" s="128"/>
+      <x:c r="C2" s="128"/>
+      <x:c r="D2" s="128"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="129" t="str">
+        <x:v>店铺名称</x:v>
+      </x:c>
+      <x:c r="B5" s="129" t="str">
+        <x:v>店铺编码</x:v>
+      </x:c>
+      <x:c r="C5" s="129" t="str">
+        <x:v>市场/用途</x:v>
+      </x:c>
+      <x:c r="D5" s="129" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="130" t="str">
+        <x:v>全部店铺</x:v>
+      </x:c>
+      <x:c r="B6" s="130" t="str">
+        <x:v>ALL</x:v>
+      </x:c>
+      <x:c r="C6" s="130" t="str">
+        <x:v>跨店汇总口径</x:v>
+      </x:c>
+      <x:c r="D6" s="130" t="str">
+        <x:v>汇总</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="130" t="str">
+        <x:v>US-旗舰店</x:v>
+      </x:c>
+      <x:c r="B7" s="130" t="str">
+        <x:v>US-MAIN</x:v>
+      </x:c>
+      <x:c r="C7" s="130" t="str">
+        <x:v>美国站主店</x:v>
+      </x:c>
+      <x:c r="D7" s="130" t="str">
+        <x:v>示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="130" t="str">
+        <x:v>US-日用店</x:v>
+      </x:c>
+      <x:c r="B8" s="130" t="str">
+        <x:v>US-DAY</x:v>
+      </x:c>
+      <x:c r="C8" s="130" t="str">
+        <x:v>美国站日用店</x:v>
+      </x:c>
+      <x:c r="D8" s="130" t="str">
+        <x:v>示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="130" t="str">
+        <x:v>TH-主店</x:v>
+      </x:c>
+      <x:c r="B9" s="130" t="str">
+        <x:v>TH-MAIN</x:v>
+      </x:c>
+      <x:c r="C9" s="130" t="str">
+        <x:v>泰国站主店</x:v>
+      </x:c>
+      <x:c r="D9" s="130" t="str">
+        <x:v>示例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="A11" s="131" t="str">
+        <x:v>填写规则：网站顶部的“全部店铺 / 单店”筛选，应与本表店铺名称、店铺日汇总、商品数据、运营动作中的店铺字段完全一致。</x:v>
+      </x:c>
+      <x:c r="B11" s="131"/>
+      <x:c r="C11" s="131"/>
+      <x:c r="D11" s="131"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="A11:D11"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="2">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb905e17429514d49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d86b795d80b41f0"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="127" t="str">
+        <x:v>五组链接对比排行｜网站经营总览</x:v>
+      </x:c>
+      <x:c r="B1" s="127"/>
+      <x:c r="C1" s="127"/>
+      <x:c r="D1" s="127"/>
+      <x:c r="E1" s="127"/>
+      <x:c r="F1" s="127"/>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="128" t="str">
+        <x:v>蓝色区域为公式结果；公式从“商品数据”读取，运营只需更新商品数据。缺少上一周期数据时，GMV/CVR 变化不要填 0。</x:v>
+      </x:c>
+      <x:c r="B2" s="128"/>
+      <x:c r="C2" s="128"/>
+      <x:c r="D2" s="128"/>
+      <x:c r="E2" s="128"/>
+      <x:c r="F2" s="128"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="132" t="str">
+        <x:v>销量 Top5｜按成交销量降序</x:v>
+      </x:c>
+      <x:c r="B4" s="132"/>
+      <x:c r="C4" s="132"/>
+      <x:c r="D4" s="132"/>
+      <x:c r="E4" s="132"/>
+      <x:c r="F4" s="132"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="129" t="str">
+        <x:v>排名</x:v>
+      </x:c>
+      <x:c r="B5" s="129" t="str">
+        <x:v>商品ID</x:v>
+      </x:c>
+      <x:c r="C5" s="129" t="str">
+        <x:v>商品名称</x:v>
+      </x:c>
+      <x:c r="D5" s="129" t="str">
+        <x:v>店铺</x:v>
+      </x:c>
+      <x:c r="E5" s="129" t="str">
+        <x:v>指标值</x:v>
+      </x:c>
+      <x:c r="F5" s="129" t="str">
+        <x:v>口径</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="133" t="n">
+        <x:f>ROW()-5</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B6" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E6,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>100176</x:v>
+      </x:c>
+      <x:c r="C6" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E6,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>3D磁吸积木套装</x:v>
+      </x:c>
+      <x:c r="D6" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E6,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>US-旗舰店</x:v>
+      </x:c>
+      <x:c r="E6" s="134" t="n">
+        <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
+        <x:v>428</x:v>
+      </x:c>
+      <x:c r="F6" s="133" t="str">
+        <x:v>按成交销量降序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="133" t="n">
+        <x:f>ROW()-5</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E7,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>100238</x:v>
+      </x:c>
+      <x:c r="C7" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E7,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>儿童户外泡泡机</x:v>
+      </x:c>
+      <x:c r="D7" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E7,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>US-日用店</x:v>
+      </x:c>
+      <x:c r="E7" s="134" t="n">
+        <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="F7" s="133" t="str">
+        <x:v>按成交销量降序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="133" t="n">
+        <x:f>ROW()-5</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B8" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E8,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>100091</x:v>
+      </x:c>
+      <x:c r="C8" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E8,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>益智拼图礼盒</x:v>
+      </x:c>
+      <x:c r="D8" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E8,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>TH-主店</x:v>
+      </x:c>
+      <x:c r="E8" s="134" t="n">
+        <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="F8" s="133" t="str">
+        <x:v>按成交销量降序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="133" t="n">
+        <x:f>ROW()-5</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E9,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>100314</x:v>
+      </x:c>
+      <x:c r="C9" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E9,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>儿童绘画水彩笔</x:v>
+      </x:c>
+      <x:c r="D9" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E9,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>US-旗舰店</x:v>
+      </x:c>
+      <x:c r="E9" s="134" t="n">
+        <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="F9" s="133" t="str">
+        <x:v>按成交销量降序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="133" t="n">
+        <x:f>ROW()-5</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B10" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E10,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>100407</x:v>
+      </x:c>
+      <x:c r="C10" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E10,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>磁力迷宫玩具</x:v>
+      </x:c>
+      <x:c r="D10" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E10,'商品数据'!$I$6:$I$11,0))</x:f>
+        <x:v>TH-主店</x:v>
+      </x:c>
+      <x:c r="E10" s="134" t="n">
+        <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="F10" s="133" t="str">
+        <x:v>按成交销量降序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="132" t="str">
+        <x:v>全店 GMV Top5｜按商品链接 GMV 降序</x:v>
+      </x:c>
+      <x:c r="B12" s="132"/>
+      <x:c r="C12" s="132"/>
+      <x:c r="D12" s="132"/>
+      <x:c r="E12" s="132"/>
+      <x:c r="F12" s="132"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>排名</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>商品ID</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>商品名称</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>店铺</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>指标值</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>口径</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="133" t="n">
+        <x:f>ROW()-13</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B14" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E14,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>100176</x:v>
+      </x:c>
+      <x:c r="C14" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E14,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>3D磁吸积木套装</x:v>
+      </x:c>
+      <x:c r="D14" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E14,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>US-旗舰店</x:v>
+      </x:c>
+      <x:c r="E14" s="135" t="n">
+        <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
+        <x:v>42680</x:v>
+      </x:c>
+      <x:c r="F14" s="133" t="str">
+        <x:v>按商品链接 GMV 降序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="133" t="n">
+        <x:f>ROW()-13</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B15" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E15,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>100238</x:v>
+      </x:c>
+      <x:c r="C15" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E15,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>儿童户外泡泡机</x:v>
+      </x:c>
+      <x:c r="D15" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E15,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>US-日用店</x:v>
+      </x:c>
+      <x:c r="E15" s="135" t="n">
+        <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
+        <x:v>18420</x:v>
+      </x:c>
+      <x:c r="F15" s="133" t="str">
+        <x:v>按商品链接 GMV 降序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="133" t="n">
+        <x:f>ROW()-13</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B16" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E16,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>100091</x:v>
+      </x:c>
+      <x:c r="C16" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E16,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>益智拼图礼盒</x:v>
+      </x:c>
+      <x:c r="D16" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E16,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>TH-主店</x:v>
+      </x:c>
+      <x:c r="E16" s="135" t="n">
+        <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
+        <x:v>15760</x:v>
+      </x:c>
+      <x:c r="F16" s="133" t="str">
+        <x:v>按商品链接 GMV 降序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="133" t="n">
+        <x:f>ROW()-13</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B17" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E17,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>100314</x:v>
+      </x:c>
+      <x:c r="C17" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E17,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>儿童绘画水彩笔</x:v>
+      </x:c>
+      <x:c r="D17" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E17,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>US-旗舰店</x:v>
+      </x:c>
+      <x:c r="E17" s="135" t="n">
+        <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
+        <x:v>12360</x:v>
+      </x:c>
+      <x:c r="F17" s="133" t="str">
+        <x:v>按商品链接 GMV 降序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="133" t="n">
+        <x:f>ROW()-13</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B18" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E18,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>100407</x:v>
+      </x:c>
+      <x:c r="C18" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E18,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>磁力迷宫玩具</x:v>
+      </x:c>
+      <x:c r="D18" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E18,'商品数据'!$J$6:$J$11,0))</x:f>
+        <x:v>TH-主店</x:v>
+      </x:c>
+      <x:c r="E18" s="135" t="n">
+        <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
+        <x:v>8120</x:v>
+      </x:c>
+      <x:c r="F18" s="133" t="str">
+        <x:v>按商品链接 GMV 降序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="132" t="str">
+        <x:v>GMV 上涨 Top5｜按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
+      </x:c>
+      <x:c r="B20" s="132"/>
+      <x:c r="C20" s="132"/>
+      <x:c r="D20" s="132"/>
+      <x:c r="E20" s="132"/>
+      <x:c r="F20" s="132"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>排名</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>商品ID</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>商品名称</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>店铺</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>指标值</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>口径</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="133" t="n">
+        <x:f>ROW()-21</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B22" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E22,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>100314</x:v>
+      </x:c>
+      <x:c r="C22" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E22,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>儿童绘画水彩笔</x:v>
+      </x:c>
+      <x:c r="D22" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E22,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>US-旗舰店</x:v>
+      </x:c>
+      <x:c r="E22" s="137" t="n">
+        <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
+        <x:v>24.1</x:v>
+      </x:c>
+      <x:c r="F22" s="133" t="str">
+        <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="133" t="n">
+        <x:f>ROW()-21</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B23" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E23,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>100176</x:v>
+      </x:c>
+      <x:c r="C23" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E23,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>3D磁吸积木套装</x:v>
+      </x:c>
+      <x:c r="D23" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E23,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>US-旗舰店</x:v>
+      </x:c>
+      <x:c r="E23" s="137" t="n">
+        <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
+        <x:v>18.6</x:v>
+      </x:c>
+      <x:c r="F23" s="133" t="str">
+        <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="133" t="n">
+        <x:f>ROW()-21</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B24" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E24,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>100091</x:v>
+      </x:c>
+      <x:c r="C24" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E24,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>益智拼图礼盒</x:v>
+      </x:c>
+      <x:c r="D24" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E24,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>TH-主店</x:v>
+      </x:c>
+      <x:c r="E24" s="137" t="n">
+        <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
+        <x:v>6.8</x:v>
+      </x:c>
+      <x:c r="F24" s="133" t="str">
+        <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="133" t="n">
+        <x:f>ROW()-21</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B25" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E25,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>100512</x:v>
+      </x:c>
+      <x:c r="C25" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E25,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>折叠儿童画板</x:v>
+      </x:c>
+      <x:c r="D25" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E25,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>US-日用店</x:v>
+      </x:c>
+      <x:c r="E25" s="137" t="n">
+        <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
+        <x:v>-3.7</x:v>
+      </x:c>
+      <x:c r="F25" s="133" t="str">
+        <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="133" t="n">
+        <x:f>ROW()-21</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B26" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E26,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>100238</x:v>
+      </x:c>
+      <x:c r="C26" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E26,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>儿童户外泡泡机</x:v>
+      </x:c>
+      <x:c r="D26" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E26,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>US-日用店</x:v>
+      </x:c>
+      <x:c r="E26" s="137" t="n">
+        <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
+        <x:v>-12.4</x:v>
+      </x:c>
+      <x:c r="F26" s="133" t="str">
+        <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="132" t="str">
+        <x:v>GMV 下降 Top5｜按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
+      </x:c>
+      <x:c r="B28" s="132"/>
+      <x:c r="C28" s="132"/>
+      <x:c r="D28" s="132"/>
+      <x:c r="E28" s="132"/>
+      <x:c r="F28" s="132"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>排名</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>商品ID</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>商品名称</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>店铺</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>指标值</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>口径</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="133" t="n">
+        <x:f>ROW()-29</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B30" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E30,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>100407</x:v>
+      </x:c>
+      <x:c r="C30" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E30,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>磁力迷宫玩具</x:v>
+      </x:c>
+      <x:c r="D30" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E30,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>TH-主店</x:v>
+      </x:c>
+      <x:c r="E30" s="137" t="n">
+        <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
+        <x:v>-26.5</x:v>
+      </x:c>
+      <x:c r="F30" s="133" t="str">
+        <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="133" t="n">
+        <x:f>ROW()-29</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B31" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E31,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>100238</x:v>
+      </x:c>
+      <x:c r="C31" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E31,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>儿童户外泡泡机</x:v>
+      </x:c>
+      <x:c r="D31" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E31,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>US-日用店</x:v>
+      </x:c>
+      <x:c r="E31" s="137" t="n">
+        <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
+        <x:v>-12.4</x:v>
+      </x:c>
+      <x:c r="F31" s="133" t="str">
+        <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="133" t="n">
+        <x:f>ROW()-29</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B32" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E32,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>100512</x:v>
+      </x:c>
+      <x:c r="C32" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E32,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>折叠儿童画板</x:v>
+      </x:c>
+      <x:c r="D32" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E32,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>US-日用店</x:v>
+      </x:c>
+      <x:c r="E32" s="137" t="n">
+        <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
+        <x:v>-3.7</x:v>
+      </x:c>
+      <x:c r="F32" s="133" t="str">
+        <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="133" t="n">
+        <x:f>ROW()-29</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B33" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E33,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>100091</x:v>
+      </x:c>
+      <x:c r="C33" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E33,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>益智拼图礼盒</x:v>
+      </x:c>
+      <x:c r="D33" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E33,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>TH-主店</x:v>
+      </x:c>
+      <x:c r="E33" s="137" t="n">
+        <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
+        <x:v>6.8</x:v>
+      </x:c>
+      <x:c r="F33" s="133" t="str">
+        <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="133" t="n">
+        <x:f>ROW()-29</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B34" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E34,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>100176</x:v>
+      </x:c>
+      <x:c r="C34" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E34,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>3D磁吸积木套装</x:v>
+      </x:c>
+      <x:c r="D34" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E34,'商品数据'!$K$6:$K$11,0))</x:f>
+        <x:v>US-旗舰店</x:v>
+      </x:c>
+      <x:c r="E34" s="137" t="n">
+        <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
+        <x:v>18.6</x:v>
+      </x:c>
+      <x:c r="F34" s="133" t="str">
+        <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="132" t="str">
+        <x:v>CVR 下降 Top5｜按 CVR 变化百分点升序</x:v>
+      </x:c>
+      <x:c r="B36" s="132"/>
+      <x:c r="C36" s="132"/>
+      <x:c r="D36" s="132"/>
+      <x:c r="E36" s="132"/>
+      <x:c r="F36" s="132"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>排名</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>商品ID</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>商品名称</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>店铺</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>指标值</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>口径</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="133" t="n">
+        <x:f>ROW()-37</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B38" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E38,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>100407</x:v>
+      </x:c>
+      <x:c r="C38" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E38,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>磁力迷宫玩具</x:v>
+      </x:c>
+      <x:c r="D38" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E38,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>TH-主店</x:v>
+      </x:c>
+      <x:c r="E38" s="138" t="n">
+        <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
+        <x:v>-1.46</x:v>
+      </x:c>
+      <x:c r="F38" s="133" t="str">
+        <x:v>按 CVR 变化百分点升序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="133" t="n">
+        <x:f>ROW()-37</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B39" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E39,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>100238</x:v>
+      </x:c>
+      <x:c r="C39" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E39,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>儿童户外泡泡机</x:v>
+      </x:c>
+      <x:c r="D39" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E39,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>US-日用店</x:v>
+      </x:c>
+      <x:c r="E39" s="138" t="n">
+        <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
+        <x:v>-1.18</x:v>
+      </x:c>
+      <x:c r="F39" s="133" t="str">
+        <x:v>按 CVR 变化百分点升序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="133" t="n">
+        <x:f>ROW()-37</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B40" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E40,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>100091</x:v>
+      </x:c>
+      <x:c r="C40" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E40,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>益智拼图礼盒</x:v>
+      </x:c>
+      <x:c r="D40" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E40,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>TH-主店</x:v>
+      </x:c>
+      <x:c r="E40" s="138" t="n">
+        <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
+        <x:v>-0.42</x:v>
+      </x:c>
+      <x:c r="F40" s="133" t="str">
+        <x:v>按 CVR 变化百分点升序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="133" t="n">
+        <x:f>ROW()-37</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B41" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E41,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>100512</x:v>
+      </x:c>
+      <x:c r="C41" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E41,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>折叠儿童画板</x:v>
+      </x:c>
+      <x:c r="D41" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E41,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>US-日用店</x:v>
+      </x:c>
+      <x:c r="E41" s="138" t="n">
+        <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
+        <x:v>-0.24</x:v>
+      </x:c>
+      <x:c r="F41" s="133" t="str">
+        <x:v>按 CVR 变化百分点升序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="133" t="n">
+        <x:f>ROW()-37</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B42" s="133" t="n">
+        <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E42,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>100314</x:v>
+      </x:c>
+      <x:c r="C42" s="133" t="str">
+        <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E42,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>儿童绘画水彩笔</x:v>
+      </x:c>
+      <x:c r="D42" s="133" t="str">
+        <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E42,'商品数据'!$N$6:$N$11,0))</x:f>
+        <x:v>US-旗舰店</x:v>
+      </x:c>
+      <x:c r="E42" s="138" t="n">
+        <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
+        <x:v>0.38</x:v>
+      </x:c>
+      <x:c r="F42" s="133" t="str">
+        <x:v>按 CVR 变化百分点升序</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A4:F4"/>
+    <x:mergeCell ref="A12:F12"/>
+    <x:mergeCell ref="A20:F20"/>
+    <x:mergeCell ref="A28:F28"/>
+    <x:mergeCell ref="A36:F36"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="10">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R484d3bfa8ebd4556"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39e69c9f88204394"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8c54b5081564f09"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafca07002c324caf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a9c881ea3f24b16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7d3c1325bd348fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58131b65dff0424d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6373d5a6c0646ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R942c479d8d4c478e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb446d6a2fa0f4214"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="127" t="str">
+        <x:v>商品数据预警｜规则与处理队列</x:v>
+      </x:c>
+      <x:c r="B1" s="127"/>
+      <x:c r="C1" s="127"/>
+      <x:c r="D1" s="127"/>
+      <x:c r="E1" s="127"/>
+      <x:c r="F1" s="127"/>
+      <x:c r="G1" s="127"/>
+      <x:c r="H1" s="127"/>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="128" t="str">
+        <x:v>预警规则对应网站“商品数据预警”页；黄色区可维护规则和处理记录，状态必须基于真实 T+1 / T+3 / T+7 数据。</x:v>
+      </x:c>
+      <x:c r="B2" s="128"/>
+      <x:c r="C2" s="128"/>
+      <x:c r="D2" s="128"/>
+      <x:c r="E2" s="128"/>
+      <x:c r="F2" s="128"/>
+      <x:c r="G2" s="128"/>
+      <x:c r="H2" s="128"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="129" t="str">
+        <x:v>预警指标</x:v>
+      </x:c>
+      <x:c r="B5" s="129" t="str">
+        <x:v>触发条件</x:v>
+      </x:c>
+      <x:c r="C5" s="129" t="str">
+        <x:v>建议节点</x:v>
+      </x:c>
+      <x:c r="D5" s="129" t="str">
+        <x:v>启用</x:v>
+      </x:c>
+      <x:c r="F5" s="129" t="str">
+        <x:v>汇总指标</x:v>
+      </x:c>
+      <x:c r="G5" s="129" t="str">
+        <x:v>当前值</x:v>
+      </x:c>
+      <x:c r="H5" s="129" t="str">
+        <x:v>说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="130" t="str">
+        <x:v>曝光下降</x:v>
+      </x:c>
+      <x:c r="B6" s="130" t="str">
+        <x:v>环比 &gt; 20%</x:v>
+      </x:c>
+      <x:c r="C6" s="130" t="str">
+        <x:v>T+1</x:v>
+      </x:c>
+      <x:c r="D6" s="130" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>高风险预警</x:v>
+      </x:c>
+      <x:c r="G6" t="n">
+        <x:f>COUNTIF('商品数据'!$Q$6:$Q$11,"需处理")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>由商品数据的当前状态汇总</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="130" t="str">
+        <x:v>GMV 下降</x:v>
+      </x:c>
+      <x:c r="B7" s="130" t="str">
+        <x:v>环比 &gt; 15%</x:v>
+      </x:c>
+      <x:c r="C7" s="130" t="str">
+        <x:v>T+1 / T+3</x:v>
+      </x:c>
+      <x:c r="D7" s="130" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>中风险预警</x:v>
+      </x:c>
+      <x:c r="G7" t="n">
+        <x:f>COUNTIF('商品数据'!$Q$6:$Q$11,"需观察")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>由商品数据的当前状态汇总</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="130" t="str">
+        <x:v>CTR 下降</x:v>
+      </x:c>
+      <x:c r="B8" s="130" t="str">
+        <x:v>下降 &gt; 0.5 个百分点</x:v>
+      </x:c>
+      <x:c r="C8" s="130" t="str">
+        <x:v>T+1</x:v>
+      </x:c>
+      <x:c r="D8" s="130" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>低风险预警</x:v>
+      </x:c>
+      <x:c r="G8" t="n">
+        <x:f>COUNTIF('商品数据'!$Q$6:$Q$11,"表现良好")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>由商品数据的当前状态汇总</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="130" t="str">
+        <x:v>CVR 下降</x:v>
+      </x:c>
+      <x:c r="B9" s="130" t="str">
+        <x:v>下降 &gt; 0.3 个百分点</x:v>
+      </x:c>
+      <x:c r="C9" s="130" t="str">
+        <x:v>T+1 / T+3 / T+7</x:v>
+      </x:c>
+      <x:c r="D9" s="130" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>待处理商品</x:v>
+      </x:c>
+      <x:c r="G9" t="n">
+        <x:f>COUNTIF('商品数据'!$Q$6:$Q$11,"需处理")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>建议动作不为空的商品数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="130" t="str">
+        <x:v>库存/承接异常</x:v>
+      </x:c>
+      <x:c r="B10" s="130" t="str">
+        <x:v>需人工判断</x:v>
+      </x:c>
+      <x:c r="C10" s="130" t="str">
+        <x:v>发现即处理</x:v>
+      </x:c>
+      <x:c r="D10" s="130" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>今日检测商品</x:v>
+      </x:c>
+      <x:c r="G10" t="n">
+        <x:f>COUNTA('商品数据'!$C$6:$C$11)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>当前日期窗口的商品记录数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="129" t="str">
+        <x:v>商品ID</x:v>
+      </x:c>
+      <x:c r="B13" s="129" t="str">
+        <x:v>店铺</x:v>
+      </x:c>
+      <x:c r="C13" s="129" t="str">
+        <x:v>预警类型</x:v>
+      </x:c>
+      <x:c r="D13" s="129" t="str">
+        <x:v>当前指标</x:v>
+      </x:c>
+      <x:c r="E13" s="129" t="str">
+        <x:v>变化值</x:v>
+      </x:c>
+      <x:c r="F13" s="129" t="str">
+        <x:v>建议动作</x:v>
+      </x:c>
+      <x:c r="G13" s="129" t="str">
+        <x:v>处理状态</x:v>
+      </x:c>
+      <x:c r="H13" s="129" t="str">
+        <x:v>证据/备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="130" t="str">
+        <x:v>100238</x:v>
+      </x:c>
+      <x:c r="B14" s="130" t="str">
+        <x:v>US-日用店</x:v>
+      </x:c>
+      <x:c r="C14" s="130" t="str">
+        <x:v>曝光下降</x:v>
+      </x:c>
+      <x:c r="D14" s="130" t="str">
+        <x:v>曝光</x:v>
+      </x:c>
+      <x:c r="E14" s="139" t="n">
+        <x:v>-28</x:v>
+      </x:c>
+      <x:c r="F14" s="130" t="str">
+        <x:v>先核查推荐流量与主图承接</x:v>
+      </x:c>
+      <x:c r="G14" s="130" t="str">
+        <x:v>待处理</x:v>
+      </x:c>
+      <x:c r="H14" s="130"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="130" t="str">
+        <x:v>100407</x:v>
+      </x:c>
+      <x:c r="B15" s="130" t="str">
+        <x:v>TH-主店</x:v>
+      </x:c>
+      <x:c r="C15" s="130" t="str">
+        <x:v>CVR下降</x:v>
+      </x:c>
+      <x:c r="D15" s="130" t="str">
+        <x:v>CVR</x:v>
+      </x:c>
+      <x:c r="E15" s="139" t="n">
+        <x:v>-1.46</x:v>
+      </x:c>
+      <x:c r="F15" s="130" t="str">
+        <x:v>检查广告落地页、流量来源和库存承接</x:v>
+      </x:c>
+      <x:c r="G15" s="130" t="str">
+        <x:v>待处理</x:v>
+      </x:c>
+      <x:c r="H15" s="130"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="130" t="str">
+        <x:v>100091</x:v>
+      </x:c>
+      <x:c r="B16" s="130" t="str">
+        <x:v>TH-主店</x:v>
+      </x:c>
+      <x:c r="C16" s="130" t="str">
+        <x:v>CVR下降</x:v>
+      </x:c>
+      <x:c r="D16" s="130" t="str">
+        <x:v>CVR</x:v>
+      </x:c>
+      <x:c r="E16" s="139" t="n">
+        <x:v>-0.42</x:v>
+      </x:c>
+      <x:c r="F16" s="130" t="str">
+        <x:v>检查商品承接和优惠设置</x:v>
+      </x:c>
+      <x:c r="G16" s="130" t="str">
+        <x:v>观察</x:v>
+      </x:c>
+      <x:c r="H16" s="130"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="130" t="str">
+        <x:v>100512</x:v>
+      </x:c>
+      <x:c r="B17" s="130" t="str">
+        <x:v>US-日用店</x:v>
+      </x:c>
+      <x:c r="C17" s="130" t="str">
+        <x:v>CTR下降</x:v>
+      </x:c>
+      <x:c r="D17" s="130" t="str">
+        <x:v>CTR</x:v>
+      </x:c>
+      <x:c r="E17" s="139" t="n">
+        <x:v>-0.22</x:v>
+      </x:c>
+      <x:c r="F17" s="130" t="str">
+        <x:v>继续观察，不单独判定异常</x:v>
+      </x:c>
+      <x:c r="G17" s="130" t="str">
+        <x:v>观察</x:v>
+      </x:c>
+      <x:c r="H17" s="130"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="130"/>
+      <x:c r="B18" s="130"/>
+      <x:c r="C18" s="130"/>
+      <x:c r="D18" s="130"/>
+      <x:c r="E18" s="139"/>
+      <x:c r="F18" s="130"/>
+      <x:c r="G18" s="130" t="str">
+        <x:v>待填写</x:v>
+      </x:c>
+      <x:c r="H18" s="130"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="130"/>
+      <x:c r="B19" s="130"/>
+      <x:c r="C19" s="130"/>
+      <x:c r="D19" s="130"/>
+      <x:c r="E19" s="139"/>
+      <x:c r="F19" s="130"/>
+      <x:c r="G19" s="130" t="str">
+        <x:v>待填写</x:v>
+      </x:c>
+      <x:c r="H19" s="130"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+  </x:mergeCells>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="D6:D10">
+      <x:formula1>"是,否"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G14:G19">
+      <x:formula1>"待处理,观察,已处理,待填写"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="6">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85f190a32cb741cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R921e14c46024411f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f4ad298c8e446ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc74ad57aa2604b9a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dc913f5e3194079"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33a48d2a175c4449"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="127" t="str">
+        <x:v>运营知识库｜有效方法沉淀</x:v>
+      </x:c>
+      <x:c r="B1" s="127"/>
+      <x:c r="C1" s="127"/>
+      <x:c r="D1" s="127"/>
+      <x:c r="E1" s="127"/>
+      <x:c r="F1" s="127"/>
+      <x:c r="G1" s="127"/>
+      <x:c r="H1" s="127"/>
+      <x:c r="I1" s="127"/>
+      <x:c r="J1" s="127"/>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="128" t="str">
+        <x:v>对应网站“运营知识库”页；只有有真实验证证据的动作才进入有效方法库，待验证动作留在运营动作表。</x:v>
+      </x:c>
+      <x:c r="B2" s="128"/>
+      <x:c r="C2" s="128"/>
+      <x:c r="D2" s="128"/>
+      <x:c r="E2" s="128"/>
+      <x:c r="F2" s="128"/>
+      <x:c r="G2" s="128"/>
+      <x:c r="H2" s="128"/>
+      <x:c r="I2" s="128"/>
+      <x:c r="J2" s="128"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="129" t="str">
+        <x:v>方法ID</x:v>
+      </x:c>
+      <x:c r="B5" s="129" t="str">
+        <x:v>方法标题</x:v>
+      </x:c>
+      <x:c r="C5" s="129" t="str">
+        <x:v>分类</x:v>
+      </x:c>
+      <x:c r="D5" s="129" t="str">
+        <x:v>适用场景</x:v>
+      </x:c>
+      <x:c r="E5" s="129" t="str">
+        <x:v>验证商品/对象</x:v>
+      </x:c>
+      <x:c r="F5" s="129" t="str">
+        <x:v>证据摘要</x:v>
+      </x:c>
+      <x:c r="G5" s="129" t="str">
+        <x:v>验证状态</x:v>
+      </x:c>
+      <x:c r="H5" s="129" t="str">
+        <x:v>负责人</x:v>
+      </x:c>
+      <x:c r="I5" s="129" t="str">
+        <x:v>复用次数</x:v>
+      </x:c>
+      <x:c r="J5" s="129" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="130" t="str">
+        <x:v>KB-001</x:v>
+      </x:c>
+      <x:c r="B6" s="130" t="str">
+        <x:v>替换首图并增加使用场景图</x:v>
+      </x:c>
+      <x:c r="C6" s="130" t="str">
+        <x:v>主图优化</x:v>
+      </x:c>
+      <x:c r="D6" s="130" t="str">
+        <x:v>曝光但承接弱</x:v>
+      </x:c>
+      <x:c r="E6" s="130" t="str">
+        <x:v>100176</x:v>
+      </x:c>
+      <x:c r="F6" s="130" t="str">
+        <x:v>T+1 CVR +0.8pp；T+3 CVR +1.7pp</x:v>
+      </x:c>
+      <x:c r="G6" s="130" t="str">
+        <x:v>已验证有效</x:v>
+      </x:c>
+      <x:c r="H6" s="130" t="str">
+        <x:v>运营A</x:v>
+      </x:c>
+      <x:c r="I6" s="140" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J6" s="130"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="130" t="str">
+        <x:v>KB-002</x:v>
+      </x:c>
+      <x:c r="B7" s="130" t="str">
+        <x:v>组合装定价测试</x:v>
+      </x:c>
+      <x:c r="C7" s="130" t="str">
+        <x:v>价格策略</x:v>
+      </x:c>
+      <x:c r="D7" s="130" t="str">
+        <x:v>销量与 GMV 同时提升</x:v>
+      </x:c>
+      <x:c r="E7" s="130" t="str">
+        <x:v>100314</x:v>
+      </x:c>
+      <x:c r="F7" s="130" t="str">
+        <x:v>T+3 销量 +18%；T+7 GMV +26%</x:v>
+      </x:c>
+      <x:c r="G7" s="130" t="str">
+        <x:v>已验证有效</x:v>
+      </x:c>
+      <x:c r="H7" s="130" t="str">
+        <x:v>运营A</x:v>
+      </x:c>
+      <x:c r="I7" s="140" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J7" s="130"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="130" t="str">
+        <x:v>KB-003</x:v>
+      </x:c>
+      <x:c r="B8" s="130" t="str">
+        <x:v>标题前置核心卖点</x:v>
+      </x:c>
+      <x:c r="C8" s="130" t="str">
+        <x:v>标题优化</x:v>
+      </x:c>
+      <x:c r="D8" s="130" t="str">
+        <x:v>CTR 有空间</x:v>
+      </x:c>
+      <x:c r="E8" s="130" t="str">
+        <x:v>100238</x:v>
+      </x:c>
+      <x:c r="F8" s="130" t="str">
+        <x:v>等待 T+1 数据回传</x:v>
+      </x:c>
+      <x:c r="G8" s="130" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="H8" s="130" t="str">
+        <x:v>运营B</x:v>
+      </x:c>
+      <x:c r="I8" s="140" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J8" s="130"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="130" t="str">
+        <x:v>KB-004</x:v>
+      </x:c>
+      <x:c r="B9" s="130" t="str">
+        <x:v>更换广告落地页</x:v>
+      </x:c>
+      <x:c r="C9" s="130" t="str">
+        <x:v>广告投放</x:v>
+      </x:c>
+      <x:c r="D9" s="130" t="str">
+        <x:v>广告点击后承接弱</x:v>
+      </x:c>
+      <x:c r="E9" s="130" t="str">
+        <x:v>100407</x:v>
+      </x:c>
+      <x:c r="F9" s="130" t="str">
+        <x:v>T+3 曝光未恢复，销量继续下降</x:v>
+      </x:c>
+      <x:c r="G9" s="130" t="str">
+        <x:v>验证无效</x:v>
+      </x:c>
+      <x:c r="H9" s="130" t="str">
+        <x:v>运营B</x:v>
+      </x:c>
+      <x:c r="I9" s="140" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="130" t="str">
+        <x:v>停止复用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="130" t="str">
+        <x:v>KB-005</x:v>
+      </x:c>
+      <x:c r="B10" s="130"/>
+      <x:c r="C10" s="130" t="str">
+        <x:v>待填写</x:v>
+      </x:c>
+      <x:c r="D10" s="130"/>
+      <x:c r="E10" s="130"/>
+      <x:c r="F10" s="130"/>
+      <x:c r="G10" s="130" t="str">
+        <x:v>待填写</x:v>
+      </x:c>
+      <x:c r="H10" s="130"/>
+      <x:c r="I10" s="140"/>
+      <x:c r="J10" s="130"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="G6:G100">
+      <x:formula1>"已验证有效,待验证,验证无效,待填写"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="2">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2448778e138c4afe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b52d6f90fbf4950"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="127" t="str">
+        <x:v>Agent 调度中心｜运营任务登记</x:v>
+      </x:c>
+      <x:c r="B1" s="127"/>
+      <x:c r="C1" s="127"/>
+      <x:c r="D1" s="127"/>
+      <x:c r="E1" s="127"/>
+      <x:c r="F1" s="127"/>
+      <x:c r="G1" s="127"/>
+      <x:c r="H1" s="127"/>
+      <x:c r="I1" s="127"/>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="128" t="str">
+        <x:v>对应网站 Agent 调度中心；本表记录要调用哪个 Agent、处理什么输入以及输出是否已被运营复核。</x:v>
+      </x:c>
+      <x:c r="B2" s="128"/>
+      <x:c r="C2" s="128"/>
+      <x:c r="D2" s="128"/>
+      <x:c r="E2" s="128"/>
+      <x:c r="F2" s="128"/>
+      <x:c r="G2" s="128"/>
+      <x:c r="H2" s="128"/>
+      <x:c r="I2" s="128"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="129" t="str">
+        <x:v>任务日期</x:v>
+      </x:c>
+      <x:c r="B5" s="129" t="str">
+        <x:v>Agent名称</x:v>
+      </x:c>
+      <x:c r="C5" s="129" t="str">
+        <x:v>触发入口</x:v>
+      </x:c>
+      <x:c r="D5" s="129" t="str">
+        <x:v>输入范围</x:v>
+      </x:c>
+      <x:c r="E5" s="129" t="str">
+        <x:v>任务目标</x:v>
+      </x:c>
+      <x:c r="F5" s="129" t="str">
+        <x:v>输出物</x:v>
+      </x:c>
+      <x:c r="G5" s="129" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+      <x:c r="H5" s="129" t="str">
+        <x:v>复核人</x:v>
+      </x:c>
+      <x:c r="I5" s="129" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="130" t="str">
+        <x:v>2026-08-29</x:v>
+      </x:c>
+      <x:c r="B6" s="130" t="str">
+        <x:v>AI日报生成 Agent</x:v>
+      </x:c>
+      <x:c r="C6" s="130" t="str">
+        <x:v>经营总览</x:v>
+      </x:c>
+      <x:c r="D6" s="130" t="str">
+        <x:v>店铺日汇总 + 商品数据</x:v>
+      </x:c>
+      <x:c r="E6" s="130" t="str">
+        <x:v>结构化日报草稿</x:v>
+      </x:c>
+      <x:c r="F6" s="130" t="str">
+        <x:v>待复核</x:v>
+      </x:c>
+      <x:c r="G6" s="130" t="str">
+        <x:v>运营负责人</x:v>
+      </x:c>
+      <x:c r="H6" s="130"/>
+      <x:c r="I6" s="130"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="130" t="str">
+        <x:v>2026-08-29</x:v>
+      </x:c>
+      <x:c r="B7" s="130" t="str">
+        <x:v>自动巡检 Agent</x:v>
+      </x:c>
+      <x:c r="C7" s="130" t="str">
+        <x:v>商品数据预警</x:v>
+      </x:c>
+      <x:c r="D7" s="130" t="str">
+        <x:v>商品数据 + T+1/T+3/T+7</x:v>
+      </x:c>
+      <x:c r="E7" s="130" t="str">
+        <x:v>风险分级与优先队列</x:v>
+      </x:c>
+      <x:c r="F7" s="130" t="str">
+        <x:v>运行中</x:v>
+      </x:c>
+      <x:c r="G7" s="130" t="str">
+        <x:v>运营负责人</x:v>
+      </x:c>
+      <x:c r="H7" s="130"/>
+      <x:c r="I7" s="130"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="130" t="str">
+        <x:v>2026-08-29</x:v>
+      </x:c>
+      <x:c r="B8" s="130" t="str">
+        <x:v>排行榜分析 Agent</x:v>
+      </x:c>
+      <x:c r="C8" s="130" t="str">
+        <x:v>五组链接对比排行</x:v>
+      </x:c>
+      <x:c r="D8" s="130" t="str">
+        <x:v>商品数据</x:v>
+      </x:c>
+      <x:c r="E8" s="130" t="str">
+        <x:v>Top5 特征与可复用策略</x:v>
+      </x:c>
+      <x:c r="F8" s="130" t="str">
+        <x:v>待调用</x:v>
+      </x:c>
+      <x:c r="G8" s="130"/>
+      <x:c r="H8" s="130"/>
+      <x:c r="I8" s="130"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="130" t="str">
+        <x:v>2026-08-29</x:v>
+      </x:c>
+      <x:c r="B9" s="130" t="str">
+        <x:v>增长分析 Agent</x:v>
+      </x:c>
+      <x:c r="C9" s="130" t="str">
+        <x:v>GMV 上涨 Top5</x:v>
+      </x:c>
+      <x:c r="D9" s="130" t="str">
+        <x:v>商品数据 + 运营动作</x:v>
+      </x:c>
+      <x:c r="E9" s="130" t="str">
+        <x:v>上涨原因与方法沉淀</x:v>
+      </x:c>
+      <x:c r="F9" s="130" t="str">
+        <x:v>待调用</x:v>
+      </x:c>
+      <x:c r="G9" s="130"/>
+      <x:c r="H9" s="130"/>
+      <x:c r="I9" s="130"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="130" t="str">
+        <x:v>2026-08-29</x:v>
+      </x:c>
+      <x:c r="B10" s="130" t="str">
+        <x:v>下滑诊断 Agent</x:v>
+      </x:c>
+      <x:c r="C10" s="130" t="str">
+        <x:v>GMV/CVR 下降 Top5</x:v>
+      </x:c>
+      <x:c r="D10" s="130" t="str">
+        <x:v>商品数据 + 广告计划</x:v>
+      </x:c>
+      <x:c r="E10" s="130" t="str">
+        <x:v>下滑原因与挽回方案</x:v>
+      </x:c>
+      <x:c r="F10" s="130" t="str">
+        <x:v>待调用</x:v>
+      </x:c>
+      <x:c r="G10" s="130"/>
+      <x:c r="H10" s="130"/>
+      <x:c r="I10" s="130"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="130"/>
+      <x:c r="B11" s="130"/>
+      <x:c r="C11" s="130"/>
+      <x:c r="D11" s="130"/>
+      <x:c r="E11" s="130"/>
+      <x:c r="F11" s="130"/>
+      <x:c r="G11" s="130" t="str">
+        <x:v>待填写</x:v>
+      </x:c>
+      <x:c r="H11" s="130"/>
+      <x:c r="I11" s="130"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A2:I2"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="G6:G100">
+      <x:formula1>"待调用,运行中,待复核,已完成,已暂停,待填写"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="2">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbdf60bf7c92e439a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6125f1506c4d46c1"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -3306,7 +5688,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fcf6938d8f540da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R323254359a7b4c11"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5798,7 +8180,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d995f15a71a4473"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5dbf1e4086b4979"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7525,7 +9907,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc47f75886464763"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5f9d28dbca94a71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8266,7 +10648,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb80a17cbe2f3445e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf69fc45368e84655"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9324,7 +11706,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R537fcc7cba164373"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda5e79067baa4f05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10876,7 +13258,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd76e507cf5d84112"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R110b8acea2bb484a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12037,7 +14419,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2854c84570f643d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6d6d1bda4284b19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12199,7 +14581,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c087ed893e549b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R027c998a480a4502"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Polish WPS Kdocs workbook layout
</commit_message>
<xml_diff>
--- a/data/tiktok-ai-operations-center-wps-kdocs-template.xlsx
+++ b/data/tiktok-ai-operations-center-wps-kdocs-template.xlsx
@@ -2,20 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填报首页" sheetId="1" r:id="Re4c4734162514bd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺日汇总" sheetId="2" r:id="R4873af065775491d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商品数据" sheetId="3" r:id="R3ef20b9028c647c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营动作" sheetId="4" r:id="Rd9ce15900f2d436c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布趋势" sheetId="5" r:id="R7d7a0bf6a2194a7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD达人" sheetId="6" r:id="Rfdb542c1e7aa446b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="广告计划" sheetId="7" r:id="R48c0e4bfa0ee4fa1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="短视频数据" sheetId="8" r:id="Rbba2111c7d0341df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段字典" sheetId="9" r:id="Ra5771170fc40468a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺字典" sheetId="10" r:id="R4bc46cdc8f3346f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="五组排行" sheetId="11" r:id="R7db5de9247b24b30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="预警规则" sheetId="12" r:id="R25ad1ab0282f435f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营知识库" sheetId="13" r:id="R82cd823e47c14ed7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent调度" sheetId="14" r:id="R9316d242fa2f4567"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填报首页" sheetId="1" r:id="R6350ae4dcce646b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺日汇总" sheetId="2" r:id="R7430d36ff76c4e4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商品数据" sheetId="3" r:id="R57a77aa7941e4349"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营动作" sheetId="4" r:id="R5939036b9e0e46bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布趋势" sheetId="5" r:id="Rded991093f8f475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD达人" sheetId="6" r:id="Raa643ad6eda84da3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="广告计划" sheetId="7" r:id="R8a6c77a6926c493f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="短视频数据" sheetId="8" r:id="Rfe960e27bd8a4cc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段字典" sheetId="9" r:id="Rf6c751fe8b514297"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺字典" sheetId="10" r:id="Rd291f931d5f34e61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="五组排行" sheetId="11" r:id="R686e26d37bd1474f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="预警规则" sheetId="12" r:id="R3c71d1361b804c85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营知识库" sheetId="13" r:id="Rb7f1dc1de622451b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent调度" sheetId="14" r:id="R2569cf7c112947cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="云文档说明" sheetId="15" r:id="R06da3144e94449da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -113,7 +114,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="19">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -153,6 +154,31 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF4DE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1E3A8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEFF6FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -292,7 +318,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="145">
+  <x:cellXfs count="173">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -638,6 +664,56 @@
     <x:xf numFmtId="0" fontId="13" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="10" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="10" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="10" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="10" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="10" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="10" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="9" fillId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -833,6 +909,18 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="StoreDictionaryTable" displayName="StoreDictionaryTable" ref="A5:D9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="店铺名称"/>
+    <x:tableColumn id="2" name="店铺编码"/>
+    <x:tableColumn id="3" name="市场/用途"/>
+    <x:tableColumn id="4" name="状态"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="SalesTop5Table" displayName="SalesTop5Table" ref="A5:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -846,7 +934,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="GMVTop5Table" displayName="GMVTop5Table" ref="A13:F18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -860,7 +948,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="GMVUpTop5Table" displayName="GMVUpTop5Table" ref="A21:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -874,7 +962,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="GMVDownTop5Table" displayName="GMVDownTop5Table" ref="A29:F34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -888,7 +976,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="CVRDownTop5Table" displayName="CVRDownTop5Table" ref="A37:F42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -902,7 +990,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="SalesTop5Table" displayName="SalesTop5Table" ref="A5:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -916,7 +1004,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="GMVTop5Table" displayName="GMVTop5Table" ref="A13:F18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -930,22 +1018,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="GMVUpTop5Table" displayName="GMVUpTop5Table" ref="A21:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="6">
-    <x:tableColumn id="1" name="排名"/>
-    <x:tableColumn id="2" name="商品ID"/>
-    <x:tableColumn id="3" name="商品名称"/>
-    <x:tableColumn id="4" name="店铺"/>
-    <x:tableColumn id="5" name="指标值"/>
-    <x:tableColumn id="6" name="口径"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="GMVDownTop5Table" displayName="GMVDownTop5Table" ref="A29:F34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
     <x:tableColumn id="2" name="商品ID"/>
@@ -986,6 +1060,20 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="GMVDownTop5Table" displayName="GMVDownTop5Table" ref="A29:F34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="CVRDownTop5Table" displayName="CVRDownTop5Table" ref="A37:F42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -999,7 +1087,77 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="SalesTop5Table" displayName="SalesTop5Table" ref="A5:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="GMVTop5Table" displayName="GMVTop5Table" ref="A13:F18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="GMVUpTop5Table" displayName="GMVUpTop5Table" ref="A21:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="GMVDownTop5Table" displayName="GMVDownTop5Table" ref="A29:F34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="CVRDownTop5Table" displayName="CVRDownTop5Table" ref="A37:F42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="WarningRulesTable" displayName="WarningRulesTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="预警指标"/>
@@ -1011,7 +1169,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="WarningSummaryTable" displayName="WarningSummaryTable" ref="F5:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="汇总指标"/>
@@ -1022,7 +1180,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="WarningQueueTable" displayName="WarningQueueTable" ref="A13:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="商品ID"/>
@@ -1033,98 +1191,6 @@
     <x:tableColumn id="6" name="建议动作"/>
     <x:tableColumn id="7" name="处理状态"/>
     <x:tableColumn id="8" name="证据/备注"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="WarningRulesTable" displayName="WarningRulesTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="4">
-    <x:tableColumn id="1" name="预警指标"/>
-    <x:tableColumn id="2" name="触发条件"/>
-    <x:tableColumn id="3" name="建议节点"/>
-    <x:tableColumn id="4" name="启用"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="WarningSummaryTable" displayName="WarningSummaryTable" ref="F5:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="3">
-    <x:tableColumn id="1" name="汇总指标"/>
-    <x:tableColumn id="2" name="当前值"/>
-    <x:tableColumn id="3" name="说明"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WarningQueueTable" displayName="WarningQueueTable" ref="A13:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="8">
-    <x:tableColumn id="1" name="商品ID"/>
-    <x:tableColumn id="2" name="店铺"/>
-    <x:tableColumn id="3" name="预警类型"/>
-    <x:tableColumn id="4" name="当前指标"/>
-    <x:tableColumn id="5" name="变化值"/>
-    <x:tableColumn id="6" name="建议动作"/>
-    <x:tableColumn id="7" name="处理状态"/>
-    <x:tableColumn id="8" name="证据/备注"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="10">
-    <x:tableColumn id="1" name="方法ID"/>
-    <x:tableColumn id="2" name="方法标题"/>
-    <x:tableColumn id="3" name="分类"/>
-    <x:tableColumn id="4" name="适用场景"/>
-    <x:tableColumn id="5" name="验证商品/对象"/>
-    <x:tableColumn id="6" name="证据摘要"/>
-    <x:tableColumn id="7" name="验证状态"/>
-    <x:tableColumn id="8" name="负责人"/>
-    <x:tableColumn id="9" name="复用次数"/>
-    <x:tableColumn id="10" name="备注"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="10">
-    <x:tableColumn id="1" name="方法ID"/>
-    <x:tableColumn id="2" name="方法标题"/>
-    <x:tableColumn id="3" name="分类"/>
-    <x:tableColumn id="4" name="适用场景"/>
-    <x:tableColumn id="5" name="验证商品/对象"/>
-    <x:tableColumn id="6" name="证据摘要"/>
-    <x:tableColumn id="7" name="验证状态"/>
-    <x:tableColumn id="8" name="负责人"/>
-    <x:tableColumn id="9" name="复用次数"/>
-    <x:tableColumn id="10" name="备注"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="AgentDispatchTable" displayName="AgentDispatchTable" ref="A5:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="9">
-    <x:tableColumn id="1" name="任务日期"/>
-    <x:tableColumn id="2" name="Agent名称"/>
-    <x:tableColumn id="3" name="触发入口"/>
-    <x:tableColumn id="4" name="输入范围"/>
-    <x:tableColumn id="5" name="任务目标"/>
-    <x:tableColumn id="6" name="输出物"/>
-    <x:tableColumn id="7" name="状态"/>
-    <x:tableColumn id="8" name="复核人"/>
-    <x:tableColumn id="9" name="备注"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1152,7 +1218,139 @@
 </file>
 
 <file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="AgentDispatchTable" displayName="AgentDispatchTable" ref="A5:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="WarningRulesTable" displayName="WarningRulesTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="预警指标"/>
+    <x:tableColumn id="2" name="触发条件"/>
+    <x:tableColumn id="3" name="建议节点"/>
+    <x:tableColumn id="4" name="启用"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="WarningSummaryTable" displayName="WarningSummaryTable" ref="F5:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="汇总指标"/>
+    <x:tableColumn id="2" name="当前值"/>
+    <x:tableColumn id="3" name="说明"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WarningQueueTable" displayName="WarningQueueTable" ref="A13:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="商品ID"/>
+    <x:tableColumn id="2" name="店铺"/>
+    <x:tableColumn id="3" name="预警类型"/>
+    <x:tableColumn id="4" name="当前指标"/>
+    <x:tableColumn id="5" name="变化值"/>
+    <x:tableColumn id="6" name="建议动作"/>
+    <x:tableColumn id="7" name="处理状态"/>
+    <x:tableColumn id="8" name="证据/备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="WarningRulesTable" displayName="WarningRulesTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="预警指标"/>
+    <x:tableColumn id="2" name="触发条件"/>
+    <x:tableColumn id="3" name="建议节点"/>
+    <x:tableColumn id="4" name="启用"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="WarningSummaryTable" displayName="WarningSummaryTable" ref="F5:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="汇总指标"/>
+    <x:tableColumn id="2" name="当前值"/>
+    <x:tableColumn id="3" name="说明"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="WarningQueueTable" displayName="WarningQueueTable" ref="A13:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="商品ID"/>
+    <x:tableColumn id="2" name="店铺"/>
+    <x:tableColumn id="3" name="预警类型"/>
+    <x:tableColumn id="4" name="当前指标"/>
+    <x:tableColumn id="5" name="变化值"/>
+    <x:tableColumn id="6" name="建议动作"/>
+    <x:tableColumn id="7" name="处理状态"/>
+    <x:tableColumn id="8" name="证据/备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="方法ID"/>
+    <x:tableColumn id="2" name="方法标题"/>
+    <x:tableColumn id="3" name="分类"/>
+    <x:tableColumn id="4" name="适用场景"/>
+    <x:tableColumn id="5" name="验证商品/对象"/>
+    <x:tableColumn id="6" name="证据摘要"/>
+    <x:tableColumn id="7" name="验证状态"/>
+    <x:tableColumn id="8" name="负责人"/>
+    <x:tableColumn id="9" name="复用次数"/>
+    <x:tableColumn id="10" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="方法ID"/>
+    <x:tableColumn id="2" name="方法标题"/>
+    <x:tableColumn id="3" name="分类"/>
+    <x:tableColumn id="4" name="适用场景"/>
+    <x:tableColumn id="5" name="验证商品/对象"/>
+    <x:tableColumn id="6" name="证据摘要"/>
+    <x:tableColumn id="7" name="验证状态"/>
+    <x:tableColumn id="8" name="负责人"/>
+    <x:tableColumn id="9" name="复用次数"/>
+    <x:tableColumn id="10" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="方法ID"/>
+    <x:tableColumn id="2" name="方法标题"/>
+    <x:tableColumn id="3" name="分类"/>
+    <x:tableColumn id="4" name="适用场景"/>
+    <x:tableColumn id="5" name="验证商品/对象"/>
+    <x:tableColumn id="6" name="证据摘要"/>
+    <x:tableColumn id="7" name="验证状态"/>
+    <x:tableColumn id="8" name="负责人"/>
+    <x:tableColumn id="9" name="复用次数"/>
+    <x:tableColumn id="10" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="AgentDispatchTable" displayName="AgentDispatchTable" ref="A5:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="任务日期"/>
     <x:tableColumn id="2" name="Agent名称"/>
@@ -1176,6 +1374,52 @@
     <x:tableColumn id="2" name="店铺"/>
     <x:tableColumn id="3" name="自营发布数量"/>
     <x:tableColumn id="4" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table40.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="AgentDispatchTable" displayName="AgentDispatchTable" ref="A5:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="任务日期"/>
+    <x:tableColumn id="2" name="Agent名称"/>
+    <x:tableColumn id="3" name="触发入口"/>
+    <x:tableColumn id="4" name="输入范围"/>
+    <x:tableColumn id="5" name="任务目标"/>
+    <x:tableColumn id="6" name="输出物"/>
+    <x:tableColumn id="7" name="状态"/>
+    <x:tableColumn id="8" name="复核人"/>
+    <x:tableColumn id="9" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table41.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="AgentDispatchTable" displayName="AgentDispatchTable" ref="A5:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="任务日期"/>
+    <x:tableColumn id="2" name="Agent名称"/>
+    <x:tableColumn id="3" name="触发入口"/>
+    <x:tableColumn id="4" name="输入范围"/>
+    <x:tableColumn id="5" name="任务目标"/>
+    <x:tableColumn id="6" name="输出物"/>
+    <x:tableColumn id="7" name="状态"/>
+    <x:tableColumn id="8" name="复核人"/>
+    <x:tableColumn id="9" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table42.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="CloudGuideTable" displayName="CloudGuideTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="步骤"/>
+    <x:tableColumn id="2" name="运营操作"/>
+    <x:tableColumn id="3" name="涉及工作表"/>
+    <x:tableColumn id="4" name="网站对应页面"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1454,14 +1698,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="38" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="4" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="4" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="4" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="4" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
@@ -1666,118 +1910,74 @@
       <x:c r="H14" s="19"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="141" t="str">
-        <x:v>v3 网站数据接入工作流</x:v>
-      </x:c>
-      <x:c r="B16" s="141"/>
-      <x:c r="C16" s="141"/>
-      <x:c r="D16" s="141"/>
-      <x:c r="E16" s="141"/>
-      <x:c r="F16" s="141"/>
-      <x:c r="G16" s="141"/>
-      <x:c r="H16" s="141"/>
+      <x:c r="A16"/>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
     </x:row>
     <x:row r="17" ht="32" customHeight="1">
-      <x:c r="A17" s="142" t="str">
-        <x:v>步骤</x:v>
-      </x:c>
-      <x:c r="B17" s="142" t="str">
-        <x:v>运营操作</x:v>
-      </x:c>
-      <x:c r="C17" s="142" t="str">
-        <x:v>涉及工作表</x:v>
-      </x:c>
-      <x:c r="D17" s="142" t="str">
-        <x:v>网站对应页面</x:v>
-      </x:c>
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
       <x:c r="E17"/>
       <x:c r="F17"/>
       <x:c r="G17"/>
       <x:c r="H17"/>
     </x:row>
     <x:row r="18" ht="32" customHeight="1">
-      <x:c r="A18" s="143" t="str">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B18" s="143" t="str">
-        <x:v>上传到 WPS/Kdocs，设置团队协作权限</x:v>
-      </x:c>
-      <x:c r="C18" s="143" t="str">
-        <x:v>整本工作簿</x:v>
-      </x:c>
-      <x:c r="D18" s="143" t="str">
-        <x:v>数据接入</x:v>
-      </x:c>
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
       <x:c r="E18"/>
       <x:c r="F18"/>
       <x:c r="G18"/>
       <x:c r="H18"/>
     </x:row>
     <x:row r="19" ht="32" customHeight="1">
-      <x:c r="A19" s="143" t="str">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B19" s="143" t="str">
-        <x:v>先维护店铺字典，再填写店铺、商品和动作数据</x:v>
-      </x:c>
-      <x:c r="C19" s="143" t="str">
-        <x:v>店铺字典 / 店铺日汇总 / 商品数据 / 运营动作</x:v>
-      </x:c>
-      <x:c r="D19" s="143" t="str">
-        <x:v>经营总览 / 商品数据预警</x:v>
-      </x:c>
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
       <x:c r="E19"/>
       <x:c r="F19"/>
       <x:c r="G19"/>
       <x:c r="H19"/>
     </x:row>
     <x:row r="20" ht="32" customHeight="1">
-      <x:c r="A20" s="143" t="str">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B20" s="143" t="str">
-        <x:v>核对五组排行、预警队列、Agent 任务和知识库</x:v>
-      </x:c>
-      <x:c r="C20" s="143" t="str">
-        <x:v>五组排行 / 预警规则 / Agent调度 / 运营知识库</x:v>
-      </x:c>
-      <x:c r="D20" s="143" t="str">
-        <x:v>经营总览 / Agent 调度中心 / 运营知识库</x:v>
-      </x:c>
+      <x:c r="A20"/>
+      <x:c r="B20"/>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
       <x:c r="E20"/>
       <x:c r="F20"/>
       <x:c r="G20"/>
       <x:c r="H20"/>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
-      <x:c r="A21" s="143" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B21" s="143" t="str">
-        <x:v>导出 CSV 或接入后端 API；静态 GitHub Pages 不会自动读取私有文档</x:v>
-      </x:c>
-      <x:c r="C21" s="143" t="str">
-        <x:v>按字段字典映射</x:v>
-      </x:c>
-      <x:c r="D21" s="143" t="str">
-        <x:v>数据接入</x:v>
-      </x:c>
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
       <x:c r="E21"/>
       <x:c r="F21"/>
       <x:c r="G21"/>
       <x:c r="H21"/>
     </x:row>
     <x:row r="23" ht="36" customHeight="1">
-      <x:c r="A23" s="144" t="str">
-        <x:v>重要说明：当前公开 v3 网站仍是主管提供的静态演示版；本工作簿已作为 WPS/Kdocs 统一填报源整理好，但要让真实数据自动驱动网页，仍需后端同步/API 和权限控制。</x:v>
-      </x:c>
-      <x:c r="B23" s="144"/>
-      <x:c r="C23" s="144"/>
-      <x:c r="D23" s="144"/>
-      <x:c r="E23" s="144"/>
-      <x:c r="F23" s="144"/>
-      <x:c r="G23" s="144"/>
-      <x:c r="H23" s="144"/>
+      <x:c r="A23"/>
+      <x:c r="B23"/>
+      <x:c r="C23"/>
+      <x:c r="D23"/>
+      <x:c r="E23"/>
+      <x:c r="F23"/>
+      <x:c r="G23"/>
+      <x:c r="H23"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1803,98 +2003,98 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="127" t="str">
+      <x:c r="A1" s="145" t="str">
         <x:v>店铺字典｜网站筛选来源</x:v>
       </x:c>
-      <x:c r="B1" s="127"/>
-      <x:c r="C1" s="127"/>
-      <x:c r="D1" s="127"/>
+      <x:c r="B1" s="145"/>
+      <x:c r="C1" s="145"/>
+      <x:c r="D1" s="145"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
-      <x:c r="A2" s="128" t="str">
+      <x:c r="A2" s="146" t="str">
         <x:v>真实店铺上线前请把黄色示例名称替换为团队实际店铺；“全部店铺”只作为汇总口径，不是一个真实店铺。</x:v>
       </x:c>
-      <x:c r="B2" s="128"/>
-      <x:c r="C2" s="128"/>
-      <x:c r="D2" s="128"/>
+      <x:c r="B2" s="146"/>
+      <x:c r="C2" s="146"/>
+      <x:c r="D2" s="146"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="129" t="str">
+      <x:c r="A5" s="147" t="str">
         <x:v>店铺名称</x:v>
       </x:c>
-      <x:c r="B5" s="129" t="str">
+      <x:c r="B5" s="147" t="str">
         <x:v>店铺编码</x:v>
       </x:c>
-      <x:c r="C5" s="129" t="str">
+      <x:c r="C5" s="147" t="str">
         <x:v>市场/用途</x:v>
       </x:c>
-      <x:c r="D5" s="129" t="str">
+      <x:c r="D5" s="147" t="str">
         <x:v>状态</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="130" t="str">
+      <x:c r="A6" s="148" t="str">
         <x:v>全部店铺</x:v>
       </x:c>
-      <x:c r="B6" s="130" t="str">
+      <x:c r="B6" s="148" t="str">
         <x:v>ALL</x:v>
       </x:c>
-      <x:c r="C6" s="130" t="str">
+      <x:c r="C6" s="148" t="str">
         <x:v>跨店汇总口径</x:v>
       </x:c>
-      <x:c r="D6" s="130" t="str">
+      <x:c r="D6" s="148" t="str">
         <x:v>汇总</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="130" t="str">
+      <x:c r="A7" s="148" t="str">
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="B7" s="130" t="str">
+      <x:c r="B7" s="148" t="str">
         <x:v>US-MAIN</x:v>
       </x:c>
-      <x:c r="C7" s="130" t="str">
+      <x:c r="C7" s="148" t="str">
         <x:v>美国站主店</x:v>
       </x:c>
-      <x:c r="D7" s="130" t="str">
+      <x:c r="D7" s="148" t="str">
         <x:v>示例</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="130" t="str">
+      <x:c r="A8" s="148" t="str">
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="B8" s="130" t="str">
+      <x:c r="B8" s="148" t="str">
         <x:v>US-DAY</x:v>
       </x:c>
-      <x:c r="C8" s="130" t="str">
+      <x:c r="C8" s="148" t="str">
         <x:v>美国站日用店</x:v>
       </x:c>
-      <x:c r="D8" s="130" t="str">
+      <x:c r="D8" s="148" t="str">
         <x:v>示例</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="130" t="str">
+      <x:c r="A9" s="148" t="str">
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="B9" s="130" t="str">
+      <x:c r="B9" s="148" t="str">
         <x:v>TH-MAIN</x:v>
       </x:c>
-      <x:c r="C9" s="130" t="str">
+      <x:c r="C9" s="148" t="str">
         <x:v>泰国站主店</x:v>
       </x:c>
-      <x:c r="D9" s="130" t="str">
+      <x:c r="D9" s="148" t="str">
         <x:v>示例</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
-      <x:c r="A11" s="131" t="str">
+      <x:c r="A11" s="149" t="str">
         <x:v>填写规则：网站顶部的“全部店铺 / 单店”筛选，应与本表店铺名称、店铺日汇总、商品数据、运营动作中的店铺字段完全一致。</x:v>
       </x:c>
-      <x:c r="B11" s="131"/>
-      <x:c r="C11" s="131"/>
-      <x:c r="D11" s="131"/>
+      <x:c r="B11" s="149"/>
+      <x:c r="C11" s="149"/>
+      <x:c r="D11" s="149"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1903,9 +2103,10 @@
     <x:mergeCell ref="A11:D11"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb905e17429514d49"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d86b795d80b41f0"/>
+  <x:tableParts count="3">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R777edd9b2f374033"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fa4c4aa255048e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4eb7d9fd69e44dfe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1923,189 +2124,189 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="127" t="str">
+      <x:c r="A1" s="145" t="str">
         <x:v>五组链接对比排行｜网站经营总览</x:v>
       </x:c>
-      <x:c r="B1" s="127"/>
-      <x:c r="C1" s="127"/>
-      <x:c r="D1" s="127"/>
-      <x:c r="E1" s="127"/>
-      <x:c r="F1" s="127"/>
+      <x:c r="B1" s="145"/>
+      <x:c r="C1" s="145"/>
+      <x:c r="D1" s="145"/>
+      <x:c r="E1" s="145"/>
+      <x:c r="F1" s="145"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
-      <x:c r="A2" s="128" t="str">
+      <x:c r="A2" s="146" t="str">
         <x:v>蓝色区域为公式结果；公式从“商品数据”读取，运营只需更新商品数据。缺少上一周期数据时，GMV/CVR 变化不要填 0。</x:v>
       </x:c>
-      <x:c r="B2" s="128"/>
-      <x:c r="C2" s="128"/>
-      <x:c r="D2" s="128"/>
-      <x:c r="E2" s="128"/>
-      <x:c r="F2" s="128"/>
+      <x:c r="B2" s="146"/>
+      <x:c r="C2" s="146"/>
+      <x:c r="D2" s="146"/>
+      <x:c r="E2" s="146"/>
+      <x:c r="F2" s="146"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="132" t="str">
+      <x:c r="A4" s="150" t="str">
         <x:v>销量 Top5｜按成交销量降序</x:v>
       </x:c>
-      <x:c r="B4" s="132"/>
-      <x:c r="C4" s="132"/>
-      <x:c r="D4" s="132"/>
-      <x:c r="E4" s="132"/>
-      <x:c r="F4" s="132"/>
+      <x:c r="B4" s="150"/>
+      <x:c r="C4" s="150"/>
+      <x:c r="D4" s="150"/>
+      <x:c r="E4" s="150"/>
+      <x:c r="F4" s="150"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="129" t="str">
+      <x:c r="A5" s="147" t="str">
         <x:v>排名</x:v>
       </x:c>
-      <x:c r="B5" s="129" t="str">
+      <x:c r="B5" s="147" t="str">
         <x:v>商品ID</x:v>
       </x:c>
-      <x:c r="C5" s="129" t="str">
+      <x:c r="C5" s="147" t="str">
         <x:v>商品名称</x:v>
       </x:c>
-      <x:c r="D5" s="129" t="str">
+      <x:c r="D5" s="147" t="str">
         <x:v>店铺</x:v>
       </x:c>
-      <x:c r="E5" s="129" t="str">
+      <x:c r="E5" s="147" t="str">
         <x:v>指标值</x:v>
       </x:c>
-      <x:c r="F5" s="129" t="str">
+      <x:c r="F5" s="147" t="str">
         <x:v>口径</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="133" t="n">
+      <x:c r="A6" s="151" t="n">
         <x:f>ROW()-5</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B6" s="133" t="n">
+      <x:c r="B6" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E6,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>100176</x:v>
       </x:c>
-      <x:c r="C6" s="133" t="str">
+      <x:c r="C6" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E6,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>3D磁吸积木套装</x:v>
       </x:c>
-      <x:c r="D6" s="133" t="str">
+      <x:c r="D6" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E6,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E6" s="134" t="n">
+      <x:c r="E6" s="152" t="n">
         <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
         <x:v>428</x:v>
       </x:c>
-      <x:c r="F6" s="133" t="str">
+      <x:c r="F6" s="151" t="str">
         <x:v>按成交销量降序</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="133" t="n">
+      <x:c r="A7" s="151" t="n">
         <x:f>ROW()-5</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B7" s="133" t="n">
+      <x:c r="B7" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E7,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="C7" s="133" t="str">
+      <x:c r="C7" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E7,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>儿童户外泡泡机</x:v>
       </x:c>
-      <x:c r="D7" s="133" t="str">
+      <x:c r="D7" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E7,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E7" s="134" t="n">
+      <x:c r="E7" s="152" t="n">
         <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
         <x:v>198</x:v>
       </x:c>
-      <x:c r="F7" s="133" t="str">
+      <x:c r="F7" s="151" t="str">
         <x:v>按成交销量降序</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="133" t="n">
+      <x:c r="A8" s="151" t="n">
         <x:f>ROW()-5</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B8" s="133" t="n">
+      <x:c r="B8" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E8,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>100091</x:v>
       </x:c>
-      <x:c r="C8" s="133" t="str">
+      <x:c r="C8" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E8,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>益智拼图礼盒</x:v>
       </x:c>
-      <x:c r="D8" s="133" t="str">
+      <x:c r="D8" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E8,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E8" s="134" t="n">
+      <x:c r="E8" s="152" t="n">
         <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
         <x:v>176</x:v>
       </x:c>
-      <x:c r="F8" s="133" t="str">
+      <x:c r="F8" s="151" t="str">
         <x:v>按成交销量降序</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="133" t="n">
+      <x:c r="A9" s="151" t="n">
         <x:f>ROW()-5</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B9" s="133" t="n">
+      <x:c r="B9" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E9,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>100314</x:v>
       </x:c>
-      <x:c r="C9" s="133" t="str">
+      <x:c r="C9" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E9,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>儿童绘画水彩笔</x:v>
       </x:c>
-      <x:c r="D9" s="133" t="str">
+      <x:c r="D9" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E9,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E9" s="134" t="n">
+      <x:c r="E9" s="152" t="n">
         <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
         <x:v>142</x:v>
       </x:c>
-      <x:c r="F9" s="133" t="str">
+      <x:c r="F9" s="151" t="str">
         <x:v>按成交销量降序</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="133" t="n">
+      <x:c r="A10" s="151" t="n">
         <x:f>ROW()-5</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B10" s="133" t="n">
+      <x:c r="B10" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E10,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>100407</x:v>
       </x:c>
-      <x:c r="C10" s="133" t="str">
+      <x:c r="C10" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E10,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>磁力迷宫玩具</x:v>
       </x:c>
-      <x:c r="D10" s="133" t="str">
+      <x:c r="D10" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E10,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E10" s="134" t="n">
+      <x:c r="E10" s="152" t="n">
         <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
         <x:v>94</x:v>
       </x:c>
-      <x:c r="F10" s="133" t="str">
+      <x:c r="F10" s="151" t="str">
         <x:v>按成交销量降序</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="132" t="str">
+      <x:c r="A12" s="150" t="str">
         <x:v>全店 GMV Top5｜按商品链接 GMV 降序</x:v>
       </x:c>
-      <x:c r="B12" s="132"/>
-      <x:c r="C12" s="132"/>
-      <x:c r="D12" s="132"/>
-      <x:c r="E12" s="132"/>
-      <x:c r="F12" s="132"/>
+      <x:c r="B12" s="150"/>
+      <x:c r="C12" s="150"/>
+      <x:c r="D12" s="150"/>
+      <x:c r="E12" s="150"/>
+      <x:c r="F12" s="150"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
@@ -2128,139 +2329,139 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="133" t="n">
+      <x:c r="A14" s="151" t="n">
         <x:f>ROW()-13</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B14" s="133" t="n">
+      <x:c r="B14" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E14,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>100176</x:v>
       </x:c>
-      <x:c r="C14" s="133" t="str">
+      <x:c r="C14" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E14,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>3D磁吸积木套装</x:v>
       </x:c>
-      <x:c r="D14" s="133" t="str">
+      <x:c r="D14" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E14,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E14" s="135" t="n">
+      <x:c r="E14" s="153" t="n">
         <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
         <x:v>42680</x:v>
       </x:c>
-      <x:c r="F14" s="133" t="str">
+      <x:c r="F14" s="151" t="str">
         <x:v>按商品链接 GMV 降序</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="133" t="n">
+      <x:c r="A15" s="151" t="n">
         <x:f>ROW()-13</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B15" s="133" t="n">
+      <x:c r="B15" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E15,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="C15" s="133" t="str">
+      <x:c r="C15" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E15,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>儿童户外泡泡机</x:v>
       </x:c>
-      <x:c r="D15" s="133" t="str">
+      <x:c r="D15" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E15,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E15" s="135" t="n">
+      <x:c r="E15" s="153" t="n">
         <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
         <x:v>18420</x:v>
       </x:c>
-      <x:c r="F15" s="133" t="str">
+      <x:c r="F15" s="151" t="str">
         <x:v>按商品链接 GMV 降序</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="133" t="n">
+      <x:c r="A16" s="151" t="n">
         <x:f>ROW()-13</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B16" s="133" t="n">
+      <x:c r="B16" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E16,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>100091</x:v>
       </x:c>
-      <x:c r="C16" s="133" t="str">
+      <x:c r="C16" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E16,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>益智拼图礼盒</x:v>
       </x:c>
-      <x:c r="D16" s="133" t="str">
+      <x:c r="D16" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E16,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E16" s="135" t="n">
+      <x:c r="E16" s="153" t="n">
         <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
         <x:v>15760</x:v>
       </x:c>
-      <x:c r="F16" s="133" t="str">
+      <x:c r="F16" s="151" t="str">
         <x:v>按商品链接 GMV 降序</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="133" t="n">
+      <x:c r="A17" s="151" t="n">
         <x:f>ROW()-13</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B17" s="133" t="n">
+      <x:c r="B17" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E17,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>100314</x:v>
       </x:c>
-      <x:c r="C17" s="133" t="str">
+      <x:c r="C17" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E17,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>儿童绘画水彩笔</x:v>
       </x:c>
-      <x:c r="D17" s="133" t="str">
+      <x:c r="D17" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E17,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E17" s="135" t="n">
+      <x:c r="E17" s="153" t="n">
         <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
         <x:v>12360</x:v>
       </x:c>
-      <x:c r="F17" s="133" t="str">
+      <x:c r="F17" s="151" t="str">
         <x:v>按商品链接 GMV 降序</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="133" t="n">
+      <x:c r="A18" s="151" t="n">
         <x:f>ROW()-13</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B18" s="133" t="n">
+      <x:c r="B18" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E18,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>100407</x:v>
       </x:c>
-      <x:c r="C18" s="133" t="str">
+      <x:c r="C18" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E18,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>磁力迷宫玩具</x:v>
       </x:c>
-      <x:c r="D18" s="133" t="str">
+      <x:c r="D18" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E18,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E18" s="135" t="n">
+      <x:c r="E18" s="153" t="n">
         <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
         <x:v>8120</x:v>
       </x:c>
-      <x:c r="F18" s="133" t="str">
+      <x:c r="F18" s="151" t="str">
         <x:v>按商品链接 GMV 降序</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="132" t="str">
+      <x:c r="A20" s="150" t="str">
         <x:v>GMV 上涨 Top5｜按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
       </x:c>
-      <x:c r="B20" s="132"/>
-      <x:c r="C20" s="132"/>
-      <x:c r="D20" s="132"/>
-      <x:c r="E20" s="132"/>
-      <x:c r="F20" s="132"/>
+      <x:c r="B20" s="150"/>
+      <x:c r="C20" s="150"/>
+      <x:c r="D20" s="150"/>
+      <x:c r="E20" s="150"/>
+      <x:c r="F20" s="150"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
@@ -2283,139 +2484,139 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="133" t="n">
+      <x:c r="A22" s="151" t="n">
         <x:f>ROW()-21</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B22" s="133" t="n">
+      <x:c r="B22" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E22,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100314</x:v>
       </x:c>
-      <x:c r="C22" s="133" t="str">
+      <x:c r="C22" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E22,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>儿童绘画水彩笔</x:v>
       </x:c>
-      <x:c r="D22" s="133" t="str">
+      <x:c r="D22" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E22,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E22" s="137" t="n">
+      <x:c r="E22" s="154" t="n">
         <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
         <x:v>24.1</x:v>
       </x:c>
-      <x:c r="F22" s="133" t="str">
+      <x:c r="F22" s="151" t="str">
         <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="133" t="n">
+      <x:c r="A23" s="151" t="n">
         <x:f>ROW()-21</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B23" s="133" t="n">
+      <x:c r="B23" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E23,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100176</x:v>
       </x:c>
-      <x:c r="C23" s="133" t="str">
+      <x:c r="C23" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E23,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>3D磁吸积木套装</x:v>
       </x:c>
-      <x:c r="D23" s="133" t="str">
+      <x:c r="D23" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E23,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E23" s="137" t="n">
+      <x:c r="E23" s="154" t="n">
         <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
         <x:v>18.6</x:v>
       </x:c>
-      <x:c r="F23" s="133" t="str">
+      <x:c r="F23" s="151" t="str">
         <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="133" t="n">
+      <x:c r="A24" s="151" t="n">
         <x:f>ROW()-21</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B24" s="133" t="n">
+      <x:c r="B24" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E24,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100091</x:v>
       </x:c>
-      <x:c r="C24" s="133" t="str">
+      <x:c r="C24" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E24,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>益智拼图礼盒</x:v>
       </x:c>
-      <x:c r="D24" s="133" t="str">
+      <x:c r="D24" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E24,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E24" s="137" t="n">
+      <x:c r="E24" s="154" t="n">
         <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
         <x:v>6.8</x:v>
       </x:c>
-      <x:c r="F24" s="133" t="str">
+      <x:c r="F24" s="151" t="str">
         <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="133" t="n">
+      <x:c r="A25" s="151" t="n">
         <x:f>ROW()-21</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B25" s="133" t="n">
+      <x:c r="B25" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E25,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100512</x:v>
       </x:c>
-      <x:c r="C25" s="133" t="str">
+      <x:c r="C25" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E25,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>折叠儿童画板</x:v>
       </x:c>
-      <x:c r="D25" s="133" t="str">
+      <x:c r="D25" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E25,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E25" s="137" t="n">
+      <x:c r="E25" s="154" t="n">
         <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
         <x:v>-3.7</x:v>
       </x:c>
-      <x:c r="F25" s="133" t="str">
+      <x:c r="F25" s="151" t="str">
         <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="133" t="n">
+      <x:c r="A26" s="151" t="n">
         <x:f>ROW()-21</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B26" s="133" t="n">
+      <x:c r="B26" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E26,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="C26" s="133" t="str">
+      <x:c r="C26" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E26,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>儿童户外泡泡机</x:v>
       </x:c>
-      <x:c r="D26" s="133" t="str">
+      <x:c r="D26" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E26,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E26" s="137" t="n">
+      <x:c r="E26" s="154" t="n">
         <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
         <x:v>-12.4</x:v>
       </x:c>
-      <x:c r="F26" s="133" t="str">
+      <x:c r="F26" s="151" t="str">
         <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="132" t="str">
+      <x:c r="A28" s="150" t="str">
         <x:v>GMV 下降 Top5｜按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
       </x:c>
-      <x:c r="B28" s="132"/>
-      <x:c r="C28" s="132"/>
-      <x:c r="D28" s="132"/>
-      <x:c r="E28" s="132"/>
-      <x:c r="F28" s="132"/>
+      <x:c r="B28" s="150"/>
+      <x:c r="C28" s="150"/>
+      <x:c r="D28" s="150"/>
+      <x:c r="E28" s="150"/>
+      <x:c r="F28" s="150"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="str">
@@ -2438,139 +2639,139 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="133" t="n">
+      <x:c r="A30" s="151" t="n">
         <x:f>ROW()-29</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B30" s="133" t="n">
+      <x:c r="B30" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E30,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100407</x:v>
       </x:c>
-      <x:c r="C30" s="133" t="str">
+      <x:c r="C30" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E30,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>磁力迷宫玩具</x:v>
       </x:c>
-      <x:c r="D30" s="133" t="str">
+      <x:c r="D30" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E30,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E30" s="137" t="n">
+      <x:c r="E30" s="154" t="n">
         <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
         <x:v>-26.5</x:v>
       </x:c>
-      <x:c r="F30" s="133" t="str">
+      <x:c r="F30" s="151" t="str">
         <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="133" t="n">
+      <x:c r="A31" s="151" t="n">
         <x:f>ROW()-29</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B31" s="133" t="n">
+      <x:c r="B31" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E31,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="C31" s="133" t="str">
+      <x:c r="C31" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E31,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>儿童户外泡泡机</x:v>
       </x:c>
-      <x:c r="D31" s="133" t="str">
+      <x:c r="D31" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E31,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E31" s="137" t="n">
+      <x:c r="E31" s="154" t="n">
         <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
         <x:v>-12.4</x:v>
       </x:c>
-      <x:c r="F31" s="133" t="str">
+      <x:c r="F31" s="151" t="str">
         <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="133" t="n">
+      <x:c r="A32" s="151" t="n">
         <x:f>ROW()-29</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B32" s="133" t="n">
+      <x:c r="B32" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E32,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100512</x:v>
       </x:c>
-      <x:c r="C32" s="133" t="str">
+      <x:c r="C32" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E32,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>折叠儿童画板</x:v>
       </x:c>
-      <x:c r="D32" s="133" t="str">
+      <x:c r="D32" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E32,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E32" s="137" t="n">
+      <x:c r="E32" s="154" t="n">
         <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
         <x:v>-3.7</x:v>
       </x:c>
-      <x:c r="F32" s="133" t="str">
+      <x:c r="F32" s="151" t="str">
         <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="133" t="n">
+      <x:c r="A33" s="151" t="n">
         <x:f>ROW()-29</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B33" s="133" t="n">
+      <x:c r="B33" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E33,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100091</x:v>
       </x:c>
-      <x:c r="C33" s="133" t="str">
+      <x:c r="C33" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E33,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>益智拼图礼盒</x:v>
       </x:c>
-      <x:c r="D33" s="133" t="str">
+      <x:c r="D33" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E33,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E33" s="137" t="n">
+      <x:c r="E33" s="154" t="n">
         <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
         <x:v>6.8</x:v>
       </x:c>
-      <x:c r="F33" s="133" t="str">
+      <x:c r="F33" s="151" t="str">
         <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="133" t="n">
+      <x:c r="A34" s="151" t="n">
         <x:f>ROW()-29</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B34" s="133" t="n">
+      <x:c r="B34" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E34,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100176</x:v>
       </x:c>
-      <x:c r="C34" s="133" t="str">
+      <x:c r="C34" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E34,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>3D磁吸积木套装</x:v>
       </x:c>
-      <x:c r="D34" s="133" t="str">
+      <x:c r="D34" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E34,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E34" s="137" t="n">
+      <x:c r="E34" s="154" t="n">
         <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
         <x:v>18.6</x:v>
       </x:c>
-      <x:c r="F34" s="133" t="str">
+      <x:c r="F34" s="151" t="str">
         <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="132" t="str">
+      <x:c r="A36" s="150" t="str">
         <x:v>CVR 下降 Top5｜按 CVR 变化百分点升序</x:v>
       </x:c>
-      <x:c r="B36" s="132"/>
-      <x:c r="C36" s="132"/>
-      <x:c r="D36" s="132"/>
-      <x:c r="E36" s="132"/>
-      <x:c r="F36" s="132"/>
+      <x:c r="B36" s="150"/>
+      <x:c r="C36" s="150"/>
+      <x:c r="D36" s="150"/>
+      <x:c r="E36" s="150"/>
+      <x:c r="F36" s="150"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="str">
@@ -2593,127 +2794,127 @@
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="133" t="n">
+      <x:c r="A38" s="151" t="n">
         <x:f>ROW()-37</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B38" s="133" t="n">
+      <x:c r="B38" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E38,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>100407</x:v>
       </x:c>
-      <x:c r="C38" s="133" t="str">
+      <x:c r="C38" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E38,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>磁力迷宫玩具</x:v>
       </x:c>
-      <x:c r="D38" s="133" t="str">
+      <x:c r="D38" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E38,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E38" s="138" t="n">
+      <x:c r="E38" s="155" t="n">
         <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
         <x:v>-1.46</x:v>
       </x:c>
-      <x:c r="F38" s="133" t="str">
+      <x:c r="F38" s="151" t="str">
         <x:v>按 CVR 变化百分点升序</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="133" t="n">
+      <x:c r="A39" s="151" t="n">
         <x:f>ROW()-37</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B39" s="133" t="n">
+      <x:c r="B39" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E39,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="C39" s="133" t="str">
+      <x:c r="C39" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E39,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>儿童户外泡泡机</x:v>
       </x:c>
-      <x:c r="D39" s="133" t="str">
+      <x:c r="D39" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E39,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E39" s="138" t="n">
+      <x:c r="E39" s="155" t="n">
         <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
         <x:v>-1.18</x:v>
       </x:c>
-      <x:c r="F39" s="133" t="str">
+      <x:c r="F39" s="151" t="str">
         <x:v>按 CVR 变化百分点升序</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="133" t="n">
+      <x:c r="A40" s="151" t="n">
         <x:f>ROW()-37</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B40" s="133" t="n">
+      <x:c r="B40" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E40,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>100091</x:v>
       </x:c>
-      <x:c r="C40" s="133" t="str">
+      <x:c r="C40" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E40,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>益智拼图礼盒</x:v>
       </x:c>
-      <x:c r="D40" s="133" t="str">
+      <x:c r="D40" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E40,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E40" s="138" t="n">
+      <x:c r="E40" s="155" t="n">
         <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
         <x:v>-0.42</x:v>
       </x:c>
-      <x:c r="F40" s="133" t="str">
+      <x:c r="F40" s="151" t="str">
         <x:v>按 CVR 变化百分点升序</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="133" t="n">
+      <x:c r="A41" s="151" t="n">
         <x:f>ROW()-37</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B41" s="133" t="n">
+      <x:c r="B41" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E41,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>100512</x:v>
       </x:c>
-      <x:c r="C41" s="133" t="str">
+      <x:c r="C41" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E41,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>折叠儿童画板</x:v>
       </x:c>
-      <x:c r="D41" s="133" t="str">
+      <x:c r="D41" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E41,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E41" s="138" t="n">
+      <x:c r="E41" s="155" t="n">
         <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
         <x:v>-0.24</x:v>
       </x:c>
-      <x:c r="F41" s="133" t="str">
+      <x:c r="F41" s="151" t="str">
         <x:v>按 CVR 变化百分点升序</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="133" t="n">
+      <x:c r="A42" s="151" t="n">
         <x:f>ROW()-37</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B42" s="133" t="n">
+      <x:c r="B42" s="151" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E42,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>100314</x:v>
       </x:c>
-      <x:c r="C42" s="133" t="str">
+      <x:c r="C42" s="151" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E42,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>儿童绘画水彩笔</x:v>
       </x:c>
-      <x:c r="D42" s="133" t="str">
+      <x:c r="D42" s="151" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E42,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E42" s="138" t="n">
+      <x:c r="E42" s="155" t="n">
         <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
         <x:v>0.38</x:v>
       </x:c>
-      <x:c r="F42" s="133" t="str">
+      <x:c r="F42" s="151" t="str">
         <x:v>按 CVR 变化百分点升序</x:v>
       </x:c>
     </x:row>
@@ -2728,17 +2929,22 @@
     <x:mergeCell ref="A36:F36"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="10">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R484d3bfa8ebd4556"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39e69c9f88204394"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8c54b5081564f09"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafca07002c324caf"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a9c881ea3f24b16"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7d3c1325bd348fe"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58131b65dff0424d"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6373d5a6c0646ed"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R942c479d8d4c478e"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb446d6a2fa0f4214"/>
+  <x:tableParts count="15">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3467c6497784f50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4beb54ff07014d6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03cb25c6ba884754"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cfea2b9663e4c14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda86ca64eb8c413b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab43f11d43ce4cf1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb38b21a5eae4738"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1c2c7ae050c4135"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e69d14e6cc64830"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf591b00eb7a84637"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9721d150f59d4d8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3184515a90514edf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f255e6221f84b7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37b232f492d94c5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd3053fccd984378"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2758,63 +2964,63 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="127" t="str">
+      <x:c r="A1" s="145" t="str">
         <x:v>商品数据预警｜规则与处理队列</x:v>
       </x:c>
-      <x:c r="B1" s="127"/>
-      <x:c r="C1" s="127"/>
-      <x:c r="D1" s="127"/>
-      <x:c r="E1" s="127"/>
-      <x:c r="F1" s="127"/>
-      <x:c r="G1" s="127"/>
-      <x:c r="H1" s="127"/>
+      <x:c r="B1" s="145"/>
+      <x:c r="C1" s="145"/>
+      <x:c r="D1" s="145"/>
+      <x:c r="E1" s="145"/>
+      <x:c r="F1" s="145"/>
+      <x:c r="G1" s="145"/>
+      <x:c r="H1" s="145"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
-      <x:c r="A2" s="128" t="str">
+      <x:c r="A2" s="146" t="str">
         <x:v>预警规则对应网站“商品数据预警”页；黄色区可维护规则和处理记录，状态必须基于真实 T+1 / T+3 / T+7 数据。</x:v>
       </x:c>
-      <x:c r="B2" s="128"/>
-      <x:c r="C2" s="128"/>
-      <x:c r="D2" s="128"/>
-      <x:c r="E2" s="128"/>
-      <x:c r="F2" s="128"/>
-      <x:c r="G2" s="128"/>
-      <x:c r="H2" s="128"/>
+      <x:c r="B2" s="146"/>
+      <x:c r="C2" s="146"/>
+      <x:c r="D2" s="146"/>
+      <x:c r="E2" s="146"/>
+      <x:c r="F2" s="146"/>
+      <x:c r="G2" s="146"/>
+      <x:c r="H2" s="146"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="129" t="str">
+      <x:c r="A5" s="147" t="str">
         <x:v>预警指标</x:v>
       </x:c>
-      <x:c r="B5" s="129" t="str">
+      <x:c r="B5" s="147" t="str">
         <x:v>触发条件</x:v>
       </x:c>
-      <x:c r="C5" s="129" t="str">
+      <x:c r="C5" s="147" t="str">
         <x:v>建议节点</x:v>
       </x:c>
-      <x:c r="D5" s="129" t="str">
+      <x:c r="D5" s="147" t="str">
         <x:v>启用</x:v>
       </x:c>
-      <x:c r="F5" s="129" t="str">
+      <x:c r="F5" s="147" t="str">
         <x:v>汇总指标</x:v>
       </x:c>
-      <x:c r="G5" s="129" t="str">
+      <x:c r="G5" s="147" t="str">
         <x:v>当前值</x:v>
       </x:c>
-      <x:c r="H5" s="129" t="str">
+      <x:c r="H5" s="147" t="str">
         <x:v>说明</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="130" t="str">
+      <x:c r="A6" s="148" t="str">
         <x:v>曝光下降</x:v>
       </x:c>
-      <x:c r="B6" s="130" t="str">
+      <x:c r="B6" s="148" t="str">
         <x:v>环比 &gt; 20%</x:v>
       </x:c>
-      <x:c r="C6" s="130" t="str">
+      <x:c r="C6" s="148" t="str">
         <x:v>T+1</x:v>
       </x:c>
-      <x:c r="D6" s="130" t="str">
+      <x:c r="D6" s="148" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="F6" t="str">
@@ -2829,16 +3035,16 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="130" t="str">
+      <x:c r="A7" s="148" t="str">
         <x:v>GMV 下降</x:v>
       </x:c>
-      <x:c r="B7" s="130" t="str">
+      <x:c r="B7" s="148" t="str">
         <x:v>环比 &gt; 15%</x:v>
       </x:c>
-      <x:c r="C7" s="130" t="str">
+      <x:c r="C7" s="148" t="str">
         <x:v>T+1 / T+3</x:v>
       </x:c>
-      <x:c r="D7" s="130" t="str">
+      <x:c r="D7" s="148" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="F7" t="str">
@@ -2853,16 +3059,16 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="130" t="str">
+      <x:c r="A8" s="148" t="str">
         <x:v>CTR 下降</x:v>
       </x:c>
-      <x:c r="B8" s="130" t="str">
+      <x:c r="B8" s="148" t="str">
         <x:v>下降 &gt; 0.5 个百分点</x:v>
       </x:c>
-      <x:c r="C8" s="130" t="str">
+      <x:c r="C8" s="148" t="str">
         <x:v>T+1</x:v>
       </x:c>
-      <x:c r="D8" s="130" t="str">
+      <x:c r="D8" s="148" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="F8" t="str">
@@ -2877,16 +3083,16 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="130" t="str">
+      <x:c r="A9" s="148" t="str">
         <x:v>CVR 下降</x:v>
       </x:c>
-      <x:c r="B9" s="130" t="str">
+      <x:c r="B9" s="148" t="str">
         <x:v>下降 &gt; 0.3 个百分点</x:v>
       </x:c>
-      <x:c r="C9" s="130" t="str">
+      <x:c r="C9" s="148" t="str">
         <x:v>T+1 / T+3 / T+7</x:v>
       </x:c>
-      <x:c r="D9" s="130" t="str">
+      <x:c r="D9" s="148" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="F9" t="str">
@@ -2901,16 +3107,16 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="130" t="str">
+      <x:c r="A10" s="148" t="str">
         <x:v>库存/承接异常</x:v>
       </x:c>
-      <x:c r="B10" s="130" t="str">
+      <x:c r="B10" s="148" t="str">
         <x:v>需人工判断</x:v>
       </x:c>
-      <x:c r="C10" s="130" t="str">
+      <x:c r="C10" s="148" t="str">
         <x:v>发现即处理</x:v>
       </x:c>
-      <x:c r="D10" s="130" t="str">
+      <x:c r="D10" s="148" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="F10" t="str">
@@ -2925,150 +3131,150 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
-      <x:c r="A13" s="129" t="str">
+      <x:c r="A13" s="147" t="str">
         <x:v>商品ID</x:v>
       </x:c>
-      <x:c r="B13" s="129" t="str">
+      <x:c r="B13" s="147" t="str">
         <x:v>店铺</x:v>
       </x:c>
-      <x:c r="C13" s="129" t="str">
+      <x:c r="C13" s="147" t="str">
         <x:v>预警类型</x:v>
       </x:c>
-      <x:c r="D13" s="129" t="str">
+      <x:c r="D13" s="147" t="str">
         <x:v>当前指标</x:v>
       </x:c>
-      <x:c r="E13" s="129" t="str">
+      <x:c r="E13" s="147" t="str">
         <x:v>变化值</x:v>
       </x:c>
-      <x:c r="F13" s="129" t="str">
+      <x:c r="F13" s="147" t="str">
         <x:v>建议动作</x:v>
       </x:c>
-      <x:c r="G13" s="129" t="str">
+      <x:c r="G13" s="147" t="str">
         <x:v>处理状态</x:v>
       </x:c>
-      <x:c r="H13" s="129" t="str">
+      <x:c r="H13" s="147" t="str">
         <x:v>证据/备注</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="130" t="str">
+      <x:c r="A14" s="148" t="str">
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="B14" s="130" t="str">
+      <x:c r="B14" s="148" t="str">
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="C14" s="130" t="str">
+      <x:c r="C14" s="148" t="str">
         <x:v>曝光下降</x:v>
       </x:c>
-      <x:c r="D14" s="130" t="str">
+      <x:c r="D14" s="148" t="str">
         <x:v>曝光</x:v>
       </x:c>
-      <x:c r="E14" s="139" t="n">
+      <x:c r="E14" s="156" t="n">
         <x:v>-28</x:v>
       </x:c>
-      <x:c r="F14" s="130" t="str">
+      <x:c r="F14" s="148" t="str">
         <x:v>先核查推荐流量与主图承接</x:v>
       </x:c>
-      <x:c r="G14" s="130" t="str">
+      <x:c r="G14" s="148" t="str">
         <x:v>待处理</x:v>
       </x:c>
-      <x:c r="H14" s="130"/>
+      <x:c r="H14" s="148"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="130" t="str">
+      <x:c r="A15" s="148" t="str">
         <x:v>100407</x:v>
       </x:c>
-      <x:c r="B15" s="130" t="str">
+      <x:c r="B15" s="148" t="str">
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="C15" s="130" t="str">
+      <x:c r="C15" s="148" t="str">
         <x:v>CVR下降</x:v>
       </x:c>
-      <x:c r="D15" s="130" t="str">
+      <x:c r="D15" s="148" t="str">
         <x:v>CVR</x:v>
       </x:c>
-      <x:c r="E15" s="139" t="n">
+      <x:c r="E15" s="156" t="n">
         <x:v>-1.46</x:v>
       </x:c>
-      <x:c r="F15" s="130" t="str">
+      <x:c r="F15" s="148" t="str">
         <x:v>检查广告落地页、流量来源和库存承接</x:v>
       </x:c>
-      <x:c r="G15" s="130" t="str">
+      <x:c r="G15" s="148" t="str">
         <x:v>待处理</x:v>
       </x:c>
-      <x:c r="H15" s="130"/>
+      <x:c r="H15" s="148"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="130" t="str">
+      <x:c r="A16" s="148" t="str">
         <x:v>100091</x:v>
       </x:c>
-      <x:c r="B16" s="130" t="str">
+      <x:c r="B16" s="148" t="str">
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="C16" s="130" t="str">
+      <x:c r="C16" s="148" t="str">
         <x:v>CVR下降</x:v>
       </x:c>
-      <x:c r="D16" s="130" t="str">
+      <x:c r="D16" s="148" t="str">
         <x:v>CVR</x:v>
       </x:c>
-      <x:c r="E16" s="139" t="n">
+      <x:c r="E16" s="156" t="n">
         <x:v>-0.42</x:v>
       </x:c>
-      <x:c r="F16" s="130" t="str">
+      <x:c r="F16" s="148" t="str">
         <x:v>检查商品承接和优惠设置</x:v>
       </x:c>
-      <x:c r="G16" s="130" t="str">
+      <x:c r="G16" s="148" t="str">
         <x:v>观察</x:v>
       </x:c>
-      <x:c r="H16" s="130"/>
+      <x:c r="H16" s="148"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="130" t="str">
+      <x:c r="A17" s="148" t="str">
         <x:v>100512</x:v>
       </x:c>
-      <x:c r="B17" s="130" t="str">
+      <x:c r="B17" s="148" t="str">
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="C17" s="130" t="str">
+      <x:c r="C17" s="148" t="str">
         <x:v>CTR下降</x:v>
       </x:c>
-      <x:c r="D17" s="130" t="str">
+      <x:c r="D17" s="148" t="str">
         <x:v>CTR</x:v>
       </x:c>
-      <x:c r="E17" s="139" t="n">
+      <x:c r="E17" s="156" t="n">
         <x:v>-0.22</x:v>
       </x:c>
-      <x:c r="F17" s="130" t="str">
+      <x:c r="F17" s="148" t="str">
         <x:v>继续观察，不单独判定异常</x:v>
       </x:c>
-      <x:c r="G17" s="130" t="str">
+      <x:c r="G17" s="148" t="str">
         <x:v>观察</x:v>
       </x:c>
-      <x:c r="H17" s="130"/>
+      <x:c r="H17" s="148"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="130"/>
-      <x:c r="B18" s="130"/>
-      <x:c r="C18" s="130"/>
-      <x:c r="D18" s="130"/>
-      <x:c r="E18" s="139"/>
-      <x:c r="F18" s="130"/>
-      <x:c r="G18" s="130" t="str">
+      <x:c r="A18" s="148"/>
+      <x:c r="B18" s="148"/>
+      <x:c r="C18" s="148"/>
+      <x:c r="D18" s="148"/>
+      <x:c r="E18" s="156"/>
+      <x:c r="F18" s="148"/>
+      <x:c r="G18" s="148" t="str">
         <x:v>待填写</x:v>
       </x:c>
-      <x:c r="H18" s="130"/>
+      <x:c r="H18" s="148"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="130"/>
-      <x:c r="B19" s="130"/>
-      <x:c r="C19" s="130"/>
-      <x:c r="D19" s="130"/>
-      <x:c r="E19" s="139"/>
-      <x:c r="F19" s="130"/>
-      <x:c r="G19" s="130" t="str">
+      <x:c r="A19" s="148"/>
+      <x:c r="B19" s="148"/>
+      <x:c r="C19" s="148"/>
+      <x:c r="D19" s="148"/>
+      <x:c r="E19" s="156"/>
+      <x:c r="F19" s="148"/>
+      <x:c r="G19" s="148" t="str">
         <x:v>待填写</x:v>
       </x:c>
-      <x:c r="H19" s="130"/>
+      <x:c r="H19" s="148"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3084,13 +3290,16 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="6">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85f190a32cb741cd"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R921e14c46024411f"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f4ad298c8e446ab"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc74ad57aa2604b9a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dc913f5e3194079"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33a48d2a175c4449"/>
+  <x:tableParts count="9">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc898bd111f00425b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8c0314cf05f4b0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra83981bbfd1a4733"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cab14e705184a7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd08d0d2baed342e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34ead97d06cd4596"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f4a538fc80f4b73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re25a5b28c6704b30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5e86e589aa24bfc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3112,204 +3321,204 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="127" t="str">
+      <x:c r="A1" s="145" t="str">
         <x:v>运营知识库｜有效方法沉淀</x:v>
       </x:c>
-      <x:c r="B1" s="127"/>
-      <x:c r="C1" s="127"/>
-      <x:c r="D1" s="127"/>
-      <x:c r="E1" s="127"/>
-      <x:c r="F1" s="127"/>
-      <x:c r="G1" s="127"/>
-      <x:c r="H1" s="127"/>
-      <x:c r="I1" s="127"/>
-      <x:c r="J1" s="127"/>
+      <x:c r="B1" s="145"/>
+      <x:c r="C1" s="145"/>
+      <x:c r="D1" s="145"/>
+      <x:c r="E1" s="145"/>
+      <x:c r="F1" s="145"/>
+      <x:c r="G1" s="145"/>
+      <x:c r="H1" s="145"/>
+      <x:c r="I1" s="145"/>
+      <x:c r="J1" s="145"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
-      <x:c r="A2" s="128" t="str">
+      <x:c r="A2" s="146" t="str">
         <x:v>对应网站“运营知识库”页；只有有真实验证证据的动作才进入有效方法库，待验证动作留在运营动作表。</x:v>
       </x:c>
-      <x:c r="B2" s="128"/>
-      <x:c r="C2" s="128"/>
-      <x:c r="D2" s="128"/>
-      <x:c r="E2" s="128"/>
-      <x:c r="F2" s="128"/>
-      <x:c r="G2" s="128"/>
-      <x:c r="H2" s="128"/>
-      <x:c r="I2" s="128"/>
-      <x:c r="J2" s="128"/>
+      <x:c r="B2" s="146"/>
+      <x:c r="C2" s="146"/>
+      <x:c r="D2" s="146"/>
+      <x:c r="E2" s="146"/>
+      <x:c r="F2" s="146"/>
+      <x:c r="G2" s="146"/>
+      <x:c r="H2" s="146"/>
+      <x:c r="I2" s="146"/>
+      <x:c r="J2" s="146"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="129" t="str">
+      <x:c r="A5" s="147" t="str">
         <x:v>方法ID</x:v>
       </x:c>
-      <x:c r="B5" s="129" t="str">
+      <x:c r="B5" s="147" t="str">
         <x:v>方法标题</x:v>
       </x:c>
-      <x:c r="C5" s="129" t="str">
+      <x:c r="C5" s="147" t="str">
         <x:v>分类</x:v>
       </x:c>
-      <x:c r="D5" s="129" t="str">
+      <x:c r="D5" s="147" t="str">
         <x:v>适用场景</x:v>
       </x:c>
-      <x:c r="E5" s="129" t="str">
+      <x:c r="E5" s="147" t="str">
         <x:v>验证商品/对象</x:v>
       </x:c>
-      <x:c r="F5" s="129" t="str">
+      <x:c r="F5" s="147" t="str">
         <x:v>证据摘要</x:v>
       </x:c>
-      <x:c r="G5" s="129" t="str">
+      <x:c r="G5" s="147" t="str">
         <x:v>验证状态</x:v>
       </x:c>
-      <x:c r="H5" s="129" t="str">
+      <x:c r="H5" s="147" t="str">
         <x:v>负责人</x:v>
       </x:c>
-      <x:c r="I5" s="129" t="str">
+      <x:c r="I5" s="147" t="str">
         <x:v>复用次数</x:v>
       </x:c>
-      <x:c r="J5" s="129" t="str">
+      <x:c r="J5" s="147" t="str">
         <x:v>备注</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="130" t="str">
+      <x:c r="A6" s="148" t="str">
         <x:v>KB-001</x:v>
       </x:c>
-      <x:c r="B6" s="130" t="str">
+      <x:c r="B6" s="148" t="str">
         <x:v>替换首图并增加使用场景图</x:v>
       </x:c>
-      <x:c r="C6" s="130" t="str">
+      <x:c r="C6" s="148" t="str">
         <x:v>主图优化</x:v>
       </x:c>
-      <x:c r="D6" s="130" t="str">
+      <x:c r="D6" s="148" t="str">
         <x:v>曝光但承接弱</x:v>
       </x:c>
-      <x:c r="E6" s="130" t="str">
+      <x:c r="E6" s="148" t="str">
         <x:v>100176</x:v>
       </x:c>
-      <x:c r="F6" s="130" t="str">
+      <x:c r="F6" s="148" t="str">
         <x:v>T+1 CVR +0.8pp；T+3 CVR +1.7pp</x:v>
       </x:c>
-      <x:c r="G6" s="130" t="str">
+      <x:c r="G6" s="148" t="str">
         <x:v>已验证有效</x:v>
       </x:c>
-      <x:c r="H6" s="130" t="str">
+      <x:c r="H6" s="148" t="str">
         <x:v>运营A</x:v>
       </x:c>
-      <x:c r="I6" s="140" t="n">
+      <x:c r="I6" s="157" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J6" s="130"/>
+      <x:c r="J6" s="148"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="130" t="str">
+      <x:c r="A7" s="148" t="str">
         <x:v>KB-002</x:v>
       </x:c>
-      <x:c r="B7" s="130" t="str">
+      <x:c r="B7" s="148" t="str">
         <x:v>组合装定价测试</x:v>
       </x:c>
-      <x:c r="C7" s="130" t="str">
+      <x:c r="C7" s="148" t="str">
         <x:v>价格策略</x:v>
       </x:c>
-      <x:c r="D7" s="130" t="str">
+      <x:c r="D7" s="148" t="str">
         <x:v>销量与 GMV 同时提升</x:v>
       </x:c>
-      <x:c r="E7" s="130" t="str">
+      <x:c r="E7" s="148" t="str">
         <x:v>100314</x:v>
       </x:c>
-      <x:c r="F7" s="130" t="str">
+      <x:c r="F7" s="148" t="str">
         <x:v>T+3 销量 +18%；T+7 GMV +26%</x:v>
       </x:c>
-      <x:c r="G7" s="130" t="str">
+      <x:c r="G7" s="148" t="str">
         <x:v>已验证有效</x:v>
       </x:c>
-      <x:c r="H7" s="130" t="str">
+      <x:c r="H7" s="148" t="str">
         <x:v>运营A</x:v>
       </x:c>
-      <x:c r="I7" s="140" t="n">
+      <x:c r="I7" s="157" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="J7" s="130"/>
+      <x:c r="J7" s="148"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="130" t="str">
+      <x:c r="A8" s="148" t="str">
         <x:v>KB-003</x:v>
       </x:c>
-      <x:c r="B8" s="130" t="str">
+      <x:c r="B8" s="148" t="str">
         <x:v>标题前置核心卖点</x:v>
       </x:c>
-      <x:c r="C8" s="130" t="str">
+      <x:c r="C8" s="148" t="str">
         <x:v>标题优化</x:v>
       </x:c>
-      <x:c r="D8" s="130" t="str">
+      <x:c r="D8" s="148" t="str">
         <x:v>CTR 有空间</x:v>
       </x:c>
-      <x:c r="E8" s="130" t="str">
+      <x:c r="E8" s="148" t="str">
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="F8" s="130" t="str">
+      <x:c r="F8" s="148" t="str">
         <x:v>等待 T+1 数据回传</x:v>
       </x:c>
-      <x:c r="G8" s="130" t="str">
+      <x:c r="G8" s="148" t="str">
         <x:v>待验证</x:v>
       </x:c>
-      <x:c r="H8" s="130" t="str">
+      <x:c r="H8" s="148" t="str">
         <x:v>运营B</x:v>
       </x:c>
-      <x:c r="I8" s="140" t="n">
+      <x:c r="I8" s="157" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J8" s="130"/>
+      <x:c r="J8" s="148"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="130" t="str">
+      <x:c r="A9" s="148" t="str">
         <x:v>KB-004</x:v>
       </x:c>
-      <x:c r="B9" s="130" t="str">
+      <x:c r="B9" s="148" t="str">
         <x:v>更换广告落地页</x:v>
       </x:c>
-      <x:c r="C9" s="130" t="str">
+      <x:c r="C9" s="148" t="str">
         <x:v>广告投放</x:v>
       </x:c>
-      <x:c r="D9" s="130" t="str">
+      <x:c r="D9" s="148" t="str">
         <x:v>广告点击后承接弱</x:v>
       </x:c>
-      <x:c r="E9" s="130" t="str">
+      <x:c r="E9" s="148" t="str">
         <x:v>100407</x:v>
       </x:c>
-      <x:c r="F9" s="130" t="str">
+      <x:c r="F9" s="148" t="str">
         <x:v>T+3 曝光未恢复，销量继续下降</x:v>
       </x:c>
-      <x:c r="G9" s="130" t="str">
+      <x:c r="G9" s="148" t="str">
         <x:v>验证无效</x:v>
       </x:c>
-      <x:c r="H9" s="130" t="str">
+      <x:c r="H9" s="148" t="str">
         <x:v>运营B</x:v>
       </x:c>
-      <x:c r="I9" s="140" t="n">
+      <x:c r="I9" s="157" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J9" s="130" t="str">
+      <x:c r="J9" s="148" t="str">
         <x:v>停止复用</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="130" t="str">
+      <x:c r="A10" s="148" t="str">
         <x:v>KB-005</x:v>
       </x:c>
-      <x:c r="B10" s="130"/>
-      <x:c r="C10" s="130" t="str">
+      <x:c r="B10" s="148"/>
+      <x:c r="C10" s="148" t="str">
         <x:v>待填写</x:v>
       </x:c>
-      <x:c r="D10" s="130"/>
-      <x:c r="E10" s="130"/>
-      <x:c r="F10" s="130"/>
-      <x:c r="G10" s="130" t="str">
+      <x:c r="D10" s="148"/>
+      <x:c r="E10" s="148"/>
+      <x:c r="F10" s="148"/>
+      <x:c r="G10" s="148" t="str">
         <x:v>待填写</x:v>
       </x:c>
-      <x:c r="H10" s="130"/>
-      <x:c r="I10" s="140"/>
-      <x:c r="J10" s="130"/>
+      <x:c r="H10" s="148"/>
+      <x:c r="I10" s="157"/>
+      <x:c r="J10" s="148"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3322,9 +3531,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2448778e138c4afe"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b52d6f90fbf4950"/>
+  <x:tableParts count="3">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29d6f175f70c45b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R118d2f11873f4129"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0443cbe6df742b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3345,191 +3555,191 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="127" t="str">
+      <x:c r="A1" s="145" t="str">
         <x:v>Agent 调度中心｜运营任务登记</x:v>
       </x:c>
-      <x:c r="B1" s="127"/>
-      <x:c r="C1" s="127"/>
-      <x:c r="D1" s="127"/>
-      <x:c r="E1" s="127"/>
-      <x:c r="F1" s="127"/>
-      <x:c r="G1" s="127"/>
-      <x:c r="H1" s="127"/>
-      <x:c r="I1" s="127"/>
+      <x:c r="B1" s="145"/>
+      <x:c r="C1" s="145"/>
+      <x:c r="D1" s="145"/>
+      <x:c r="E1" s="145"/>
+      <x:c r="F1" s="145"/>
+      <x:c r="G1" s="145"/>
+      <x:c r="H1" s="145"/>
+      <x:c r="I1" s="145"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
-      <x:c r="A2" s="128" t="str">
+      <x:c r="A2" s="146" t="str">
         <x:v>对应网站 Agent 调度中心；本表记录要调用哪个 Agent、处理什么输入以及输出是否已被运营复核。</x:v>
       </x:c>
-      <x:c r="B2" s="128"/>
-      <x:c r="C2" s="128"/>
-      <x:c r="D2" s="128"/>
-      <x:c r="E2" s="128"/>
-      <x:c r="F2" s="128"/>
-      <x:c r="G2" s="128"/>
-      <x:c r="H2" s="128"/>
-      <x:c r="I2" s="128"/>
+      <x:c r="B2" s="146"/>
+      <x:c r="C2" s="146"/>
+      <x:c r="D2" s="146"/>
+      <x:c r="E2" s="146"/>
+      <x:c r="F2" s="146"/>
+      <x:c r="G2" s="146"/>
+      <x:c r="H2" s="146"/>
+      <x:c r="I2" s="146"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="129" t="str">
+      <x:c r="A5" s="147" t="str">
         <x:v>任务日期</x:v>
       </x:c>
-      <x:c r="B5" s="129" t="str">
+      <x:c r="B5" s="147" t="str">
         <x:v>Agent名称</x:v>
       </x:c>
-      <x:c r="C5" s="129" t="str">
+      <x:c r="C5" s="147" t="str">
         <x:v>触发入口</x:v>
       </x:c>
-      <x:c r="D5" s="129" t="str">
+      <x:c r="D5" s="147" t="str">
         <x:v>输入范围</x:v>
       </x:c>
-      <x:c r="E5" s="129" t="str">
+      <x:c r="E5" s="147" t="str">
         <x:v>任务目标</x:v>
       </x:c>
-      <x:c r="F5" s="129" t="str">
+      <x:c r="F5" s="147" t="str">
         <x:v>输出物</x:v>
       </x:c>
-      <x:c r="G5" s="129" t="str">
+      <x:c r="G5" s="147" t="str">
         <x:v>状态</x:v>
       </x:c>
-      <x:c r="H5" s="129" t="str">
+      <x:c r="H5" s="147" t="str">
         <x:v>复核人</x:v>
       </x:c>
-      <x:c r="I5" s="129" t="str">
+      <x:c r="I5" s="147" t="str">
         <x:v>备注</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="130" t="str">
+      <x:c r="A6" s="148" t="str">
         <x:v>2026-08-29</x:v>
       </x:c>
-      <x:c r="B6" s="130" t="str">
+      <x:c r="B6" s="148" t="str">
         <x:v>AI日报生成 Agent</x:v>
       </x:c>
-      <x:c r="C6" s="130" t="str">
+      <x:c r="C6" s="148" t="str">
         <x:v>经营总览</x:v>
       </x:c>
-      <x:c r="D6" s="130" t="str">
+      <x:c r="D6" s="148" t="str">
         <x:v>店铺日汇总 + 商品数据</x:v>
       </x:c>
-      <x:c r="E6" s="130" t="str">
+      <x:c r="E6" s="148" t="str">
         <x:v>结构化日报草稿</x:v>
       </x:c>
-      <x:c r="F6" s="130" t="str">
+      <x:c r="F6" s="148" t="str">
         <x:v>待复核</x:v>
       </x:c>
-      <x:c r="G6" s="130" t="str">
+      <x:c r="G6" s="148" t="str">
         <x:v>运营负责人</x:v>
       </x:c>
-      <x:c r="H6" s="130"/>
-      <x:c r="I6" s="130"/>
+      <x:c r="H6" s="148"/>
+      <x:c r="I6" s="148"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="130" t="str">
+      <x:c r="A7" s="148" t="str">
         <x:v>2026-08-29</x:v>
       </x:c>
-      <x:c r="B7" s="130" t="str">
+      <x:c r="B7" s="148" t="str">
         <x:v>自动巡检 Agent</x:v>
       </x:c>
-      <x:c r="C7" s="130" t="str">
+      <x:c r="C7" s="148" t="str">
         <x:v>商品数据预警</x:v>
       </x:c>
-      <x:c r="D7" s="130" t="str">
+      <x:c r="D7" s="148" t="str">
         <x:v>商品数据 + T+1/T+3/T+7</x:v>
       </x:c>
-      <x:c r="E7" s="130" t="str">
+      <x:c r="E7" s="148" t="str">
         <x:v>风险分级与优先队列</x:v>
       </x:c>
-      <x:c r="F7" s="130" t="str">
+      <x:c r="F7" s="148" t="str">
         <x:v>运行中</x:v>
       </x:c>
-      <x:c r="G7" s="130" t="str">
+      <x:c r="G7" s="148" t="str">
         <x:v>运营负责人</x:v>
       </x:c>
-      <x:c r="H7" s="130"/>
-      <x:c r="I7" s="130"/>
+      <x:c r="H7" s="148"/>
+      <x:c r="I7" s="148"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="130" t="str">
+      <x:c r="A8" s="148" t="str">
         <x:v>2026-08-29</x:v>
       </x:c>
-      <x:c r="B8" s="130" t="str">
+      <x:c r="B8" s="148" t="str">
         <x:v>排行榜分析 Agent</x:v>
       </x:c>
-      <x:c r="C8" s="130" t="str">
+      <x:c r="C8" s="148" t="str">
         <x:v>五组链接对比排行</x:v>
       </x:c>
-      <x:c r="D8" s="130" t="str">
+      <x:c r="D8" s="148" t="str">
         <x:v>商品数据</x:v>
       </x:c>
-      <x:c r="E8" s="130" t="str">
+      <x:c r="E8" s="148" t="str">
         <x:v>Top5 特征与可复用策略</x:v>
       </x:c>
-      <x:c r="F8" s="130" t="str">
+      <x:c r="F8" s="148" t="str">
         <x:v>待调用</x:v>
       </x:c>
-      <x:c r="G8" s="130"/>
-      <x:c r="H8" s="130"/>
-      <x:c r="I8" s="130"/>
+      <x:c r="G8" s="148"/>
+      <x:c r="H8" s="148"/>
+      <x:c r="I8" s="148"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="130" t="str">
+      <x:c r="A9" s="148" t="str">
         <x:v>2026-08-29</x:v>
       </x:c>
-      <x:c r="B9" s="130" t="str">
+      <x:c r="B9" s="148" t="str">
         <x:v>增长分析 Agent</x:v>
       </x:c>
-      <x:c r="C9" s="130" t="str">
+      <x:c r="C9" s="148" t="str">
         <x:v>GMV 上涨 Top5</x:v>
       </x:c>
-      <x:c r="D9" s="130" t="str">
+      <x:c r="D9" s="148" t="str">
         <x:v>商品数据 + 运营动作</x:v>
       </x:c>
-      <x:c r="E9" s="130" t="str">
+      <x:c r="E9" s="148" t="str">
         <x:v>上涨原因与方法沉淀</x:v>
       </x:c>
-      <x:c r="F9" s="130" t="str">
+      <x:c r="F9" s="148" t="str">
         <x:v>待调用</x:v>
       </x:c>
-      <x:c r="G9" s="130"/>
-      <x:c r="H9" s="130"/>
-      <x:c r="I9" s="130"/>
+      <x:c r="G9" s="148"/>
+      <x:c r="H9" s="148"/>
+      <x:c r="I9" s="148"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="130" t="str">
+      <x:c r="A10" s="148" t="str">
         <x:v>2026-08-29</x:v>
       </x:c>
-      <x:c r="B10" s="130" t="str">
+      <x:c r="B10" s="148" t="str">
         <x:v>下滑诊断 Agent</x:v>
       </x:c>
-      <x:c r="C10" s="130" t="str">
+      <x:c r="C10" s="148" t="str">
         <x:v>GMV/CVR 下降 Top5</x:v>
       </x:c>
-      <x:c r="D10" s="130" t="str">
+      <x:c r="D10" s="148" t="str">
         <x:v>商品数据 + 广告计划</x:v>
       </x:c>
-      <x:c r="E10" s="130" t="str">
+      <x:c r="E10" s="148" t="str">
         <x:v>下滑原因与挽回方案</x:v>
       </x:c>
-      <x:c r="F10" s="130" t="str">
+      <x:c r="F10" s="148" t="str">
         <x:v>待调用</x:v>
       </x:c>
-      <x:c r="G10" s="130"/>
-      <x:c r="H10" s="130"/>
-      <x:c r="I10" s="130"/>
+      <x:c r="G10" s="148"/>
+      <x:c r="H10" s="148"/>
+      <x:c r="I10" s="148"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="130"/>
-      <x:c r="B11" s="130"/>
-      <x:c r="C11" s="130"/>
-      <x:c r="D11" s="130"/>
-      <x:c r="E11" s="130"/>
-      <x:c r="F11" s="130"/>
-      <x:c r="G11" s="130" t="str">
+      <x:c r="A11" s="148"/>
+      <x:c r="B11" s="148"/>
+      <x:c r="C11" s="148"/>
+      <x:c r="D11" s="148"/>
+      <x:c r="E11" s="148"/>
+      <x:c r="F11" s="148"/>
+      <x:c r="G11" s="148" t="str">
         <x:v>待填写</x:v>
       </x:c>
-      <x:c r="H11" s="130"/>
-      <x:c r="I11" s="130"/>
+      <x:c r="H11" s="148"/>
+      <x:c r="I11" s="148"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3542,9 +3752,141 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbdf60bf7c92e439a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6125f1506c4d46c1"/>
+  <x:tableParts count="3">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R921eb3b1098e4979"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbc136563cb54a91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree0cda171a1743b1"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="46" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="145" t="str">
+        <x:v>云文档说明｜WPS/Kdocs 使用流程</x:v>
+      </x:c>
+      <x:c r="B1" s="145"/>
+      <x:c r="C1" s="145"/>
+      <x:c r="D1" s="145"/>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="146" t="str">
+        <x:v>这张表是给运营看的操作说明；填报数据请回到黄色输入区域，公式排行和预警汇总不要手工改写。</x:v>
+      </x:c>
+      <x:c r="B2" s="146"/>
+      <x:c r="C2" s="146"/>
+      <x:c r="D2" s="146"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="147" t="str">
+        <x:v>步骤</x:v>
+      </x:c>
+      <x:c r="B5" s="147" t="str">
+        <x:v>运营操作</x:v>
+      </x:c>
+      <x:c r="C5" s="147" t="str">
+        <x:v>涉及工作表</x:v>
+      </x:c>
+      <x:c r="D5" s="147" t="str">
+        <x:v>网站对应页面</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="148" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B6" s="148" t="str">
+        <x:v>上传本文件到 WPS/Kdocs，设置团队协作权限</x:v>
+      </x:c>
+      <x:c r="C6" s="148" t="str">
+        <x:v>整本工作簿</x:v>
+      </x:c>
+      <x:c r="D6" s="148" t="str">
+        <x:v>数据接入</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="148" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="148" t="str">
+        <x:v>先维护店铺字典，再填写店铺、商品和已执行动作</x:v>
+      </x:c>
+      <x:c r="C7" s="148" t="str">
+        <x:v>店铺字典 / 店铺日汇总 / 商品数据 / 运营动作</x:v>
+      </x:c>
+      <x:c r="D7" s="148" t="str">
+        <x:v>经营总览 / 商品数据预警</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="148" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B8" s="148" t="str">
+        <x:v>核对五组排行、预警队列、Agent 任务和知识库</x:v>
+      </x:c>
+      <x:c r="C8" s="148" t="str">
+        <x:v>五组排行 / 预警规则 / Agent调度 / 运营知识库</x:v>
+      </x:c>
+      <x:c r="D8" s="148" t="str">
+        <x:v>经营总览 / Agent 调度中心 / 运营知识库</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="148" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="148" t="str">
+        <x:v>导出 CSV 或交给后端 API；静态 GitHub Pages 不会自动读取私有文档</x:v>
+      </x:c>
+      <x:c r="C9" s="148" t="str">
+        <x:v>按字段字典映射</x:v>
+      </x:c>
+      <x:c r="D9" s="148" t="str">
+        <x:v>数据接入</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="148" t="str">
+        <x:v>注意</x:v>
+      </x:c>
+      <x:c r="B10" s="148" t="str">
+        <x:v>当前内容是演示模板；真实数据请保持缺失为空，不能用 0 代替未知。</x:v>
+      </x:c>
+      <x:c r="C10" s="148" t="str">
+        <x:v>字段字典</x:v>
+      </x:c>
+      <x:c r="D10" s="148" t="str">
+        <x:v>全部页面</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="38" customHeight="1">
+      <x:c r="A12" s="172" t="str">
+        <x:v>公开网站当前为静态演示版。WPS/Kdocs 文档可以作为统一填报源，但真实数据自动刷新仍需要后端同步/API 和认证权限。</x:v>
+      </x:c>
+      <x:c r="B12" s="172"/>
+      <x:c r="C12" s="172"/>
+      <x:c r="D12" s="172"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="A12:D12"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42b8a7cdd0534ce5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5688,7 +6030,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R323254359a7b4c11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb966784531af4294"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8180,7 +8522,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5dbf1e4086b4979"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc13ef3c3a5a1405a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9907,7 +10249,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5f9d28dbca94a71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d0dc64c7e3f4719"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10648,7 +10990,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf69fc45368e84655"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7715adb9a128491d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11706,7 +12048,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda5e79067baa4f05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85b97472b3bb4522"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13258,7 +13600,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R110b8acea2bb484a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7179c49351134b66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14419,7 +14761,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6d6d1bda4284b19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dfaf32231f147f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14581,7 +14923,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R027c998a480a4502"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e8ed2bd03f54253"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Polish WPS Kdocs workbook styling
</commit_message>
<xml_diff>
--- a/data/tiktok-ai-operations-center-wps-kdocs-template.xlsx
+++ b/data/tiktok-ai-operations-center-wps-kdocs-template.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填报首页" sheetId="1" r:id="R6350ae4dcce646b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺日汇总" sheetId="2" r:id="R7430d36ff76c4e4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商品数据" sheetId="3" r:id="R57a77aa7941e4349"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营动作" sheetId="4" r:id="R5939036b9e0e46bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布趋势" sheetId="5" r:id="Rded991093f8f475b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD达人" sheetId="6" r:id="Raa643ad6eda84da3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="广告计划" sheetId="7" r:id="R8a6c77a6926c493f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="短视频数据" sheetId="8" r:id="Rfe960e27bd8a4cc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段字典" sheetId="9" r:id="Rf6c751fe8b514297"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺字典" sheetId="10" r:id="Rd291f931d5f34e61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="五组排行" sheetId="11" r:id="R686e26d37bd1474f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="预警规则" sheetId="12" r:id="R3c71d1361b804c85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营知识库" sheetId="13" r:id="Rb7f1dc1de622451b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent调度" sheetId="14" r:id="R2569cf7c112947cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="云文档说明" sheetId="15" r:id="R06da3144e94449da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填报首页" sheetId="1" r:id="R306f56cc3a004747"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺日汇总" sheetId="2" r:id="Rdc76b9c3390645dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商品数据" sheetId="3" r:id="Rb268268a4607473f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营动作" sheetId="4" r:id="R92e3901e877f4c8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布趋势" sheetId="5" r:id="R597c828a92de47b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD达人" sheetId="6" r:id="R727c1871b4144e59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="广告计划" sheetId="7" r:id="Rc599842fae834b5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="短视频数据" sheetId="8" r:id="R5b2865b7d1b54a0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段字典" sheetId="9" r:id="R5441e027d2df42da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="店铺字典" sheetId="10" r:id="R3f8f5872bab048fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="五组排行" sheetId="11" r:id="R426a7f96cea64b08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="预警规则" sheetId="12" r:id="R48e0341c0fb8480d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运营知识库" sheetId="13" r:id="R57d004341d7d47dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent调度" sheetId="14" r:id="Rf80724e3bf2a4d20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="云文档说明" sheetId="15" r:id="Rf22e6ed3bd144a62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -37,7 +37,7 @@
     <x:numFmt numFmtId="206" formatCode="&quot;¥&quot;#,##0"/>
     <x:numFmt numFmtId="207" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="19">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -113,8 +113,37 @@
       <x:color rgb="FF92400E"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF0F172A"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1E3A8A"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF166534"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF991B1B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="24">
+  <x:fills count="32">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -231,8 +260,48 @@
         <x:fgColor rgb="FFFEF3C7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1E3A8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEFF6FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDFF7F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCFCE7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEE2E2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="11">
+  <x:borders count="23">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -314,11 +383,119 @@
         <x:color rgb="FFAFC0F5"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="173">
+  <x:cellXfs count="312">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -713,6 +890,333 @@
     <x:xf numFmtId="0" fontId="13" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="13" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="10" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="10" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="10" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="10" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="10" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="10" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="24" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="24" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="27" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="27" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="27" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="27" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="27" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="27" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="27" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="27" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="25" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="25" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="25" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="25" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="25" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="25" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="25" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="25" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="28" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="28" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="28" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="28" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="28" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="28" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="26" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="26" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="26" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="26" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="26" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="26" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="25" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="25" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="10" fillId="25" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="25" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="25" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="203" fontId="10" fillId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="10" fillId="25" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="25" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="25" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="10" fillId="25" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="25" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="10" fillId="25" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="10" fillId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="206" fontId="10" fillId="25" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="10" fillId="25" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="10" fillId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="204" fontId="10" fillId="25" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="10" fillId="25" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="10" fillId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="202" fontId="10" fillId="25" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="27" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="27" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="27" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="27" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="27" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="10" fillId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="10" fillId="27" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="25" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="10" fillId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="10" fillId="27" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="28" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="28" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="25" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="25" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="25" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="25" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="25" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="25" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="24" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="24" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="24" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="24" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="24" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="24" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -921,6 +1425,18 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="StoreDictionaryTable" displayName="StoreDictionaryTable" ref="A5:D9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="店铺名称"/>
+    <x:tableColumn id="2" name="店铺编码"/>
+    <x:tableColumn id="3" name="市场/用途"/>
+    <x:tableColumn id="4" name="状态"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="SalesTop5Table" displayName="SalesTop5Table" ref="A5:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -934,7 +1450,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="GMVTop5Table" displayName="GMVTop5Table" ref="A13:F18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -948,7 +1464,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="GMVUpTop5Table" displayName="GMVUpTop5Table" ref="A21:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -962,7 +1478,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="GMVDownTop5Table" displayName="GMVDownTop5Table" ref="A29:F34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -976,7 +1492,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="CVRDownTop5Table" displayName="CVRDownTop5Table" ref="A37:F42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -990,7 +1506,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="SalesTop5Table" displayName="SalesTop5Table" ref="A5:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -1004,22 +1520,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="GMVTop5Table" displayName="GMVTop5Table" ref="A13:F18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="6">
-    <x:tableColumn id="1" name="排名"/>
-    <x:tableColumn id="2" name="商品ID"/>
-    <x:tableColumn id="3" name="商品名称"/>
-    <x:tableColumn id="4" name="店铺"/>
-    <x:tableColumn id="5" name="指标值"/>
-    <x:tableColumn id="6" name="口径"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="GMVUpTop5Table" displayName="GMVUpTop5Table" ref="A21:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
     <x:tableColumn id="2" name="商品ID"/>
@@ -1060,6 +1562,20 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="GMVUpTop5Table" displayName="GMVUpTop5Table" ref="A21:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="GMVDownTop5Table" displayName="GMVDownTop5Table" ref="A29:F34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -1073,7 +1589,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="CVRDownTop5Table" displayName="CVRDownTop5Table" ref="A37:F42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -1087,7 +1603,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="SalesTop5Table" displayName="SalesTop5Table" ref="A5:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -1101,7 +1617,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="GMVTop5Table" displayName="GMVTop5Table" ref="A13:F18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -1115,7 +1631,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="GMVUpTop5Table" displayName="GMVUpTop5Table" ref="A21:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -1129,7 +1645,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="GMVDownTop5Table" displayName="GMVDownTop5Table" ref="A29:F34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -1143,7 +1659,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="CVRDownTop5Table" displayName="CVRDownTop5Table" ref="A37:F42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="排名"/>
@@ -1157,40 +1673,29 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="WarningRulesTable" displayName="WarningRulesTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="4">
-    <x:tableColumn id="1" name="预警指标"/>
-    <x:tableColumn id="2" name="触发条件"/>
-    <x:tableColumn id="3" name="建议节点"/>
-    <x:tableColumn id="4" name="启用"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
 <file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="WarningSummaryTable" displayName="WarningSummaryTable" ref="F5:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="3">
-    <x:tableColumn id="1" name="汇总指标"/>
-    <x:tableColumn id="2" name="当前值"/>
-    <x:tableColumn id="3" name="说明"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="SalesTop5Table" displayName="SalesTop5Table" ref="A5:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="WarningQueueTable" displayName="WarningQueueTable" ref="A13:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="8">
-    <x:tableColumn id="1" name="商品ID"/>
-    <x:tableColumn id="2" name="店铺"/>
-    <x:tableColumn id="3" name="预警类型"/>
-    <x:tableColumn id="4" name="当前指标"/>
-    <x:tableColumn id="5" name="变化值"/>
-    <x:tableColumn id="6" name="建议动作"/>
-    <x:tableColumn id="7" name="处理状态"/>
-    <x:tableColumn id="8" name="证据/备注"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="GMVTop5Table" displayName="GMVTop5Table" ref="A13:F18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1218,6 +1723,87 @@
 </file>
 
 <file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="GMVUpTop5Table" displayName="GMVUpTop5Table" ref="A21:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="GMVDownTop5Table" displayName="GMVDownTop5Table" ref="A29:F34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="CVRDownTop5Table" displayName="CVRDownTop5Table" ref="A37:F42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="排名"/>
+    <x:tableColumn id="2" name="商品ID"/>
+    <x:tableColumn id="3" name="商品名称"/>
+    <x:tableColumn id="4" name="店铺"/>
+    <x:tableColumn id="5" name="指标值"/>
+    <x:tableColumn id="6" name="口径"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="WarningRulesTable" displayName="WarningRulesTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="预警指标"/>
+    <x:tableColumn id="2" name="触发条件"/>
+    <x:tableColumn id="3" name="建议节点"/>
+    <x:tableColumn id="4" name="启用"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="WarningSummaryTable" displayName="WarningSummaryTable" ref="F5:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="汇总指标"/>
+    <x:tableColumn id="2" name="当前值"/>
+    <x:tableColumn id="3" name="说明"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="WarningQueueTable" displayName="WarningQueueTable" ref="A13:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="商品ID"/>
+    <x:tableColumn id="2" name="店铺"/>
+    <x:tableColumn id="3" name="预警类型"/>
+    <x:tableColumn id="4" name="当前指标"/>
+    <x:tableColumn id="5" name="变化值"/>
+    <x:tableColumn id="6" name="建议动作"/>
+    <x:tableColumn id="7" name="处理状态"/>
+    <x:tableColumn id="8" name="证据/备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="WarningRulesTable" displayName="WarningRulesTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="预警指标"/>
@@ -1229,7 +1815,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="WarningSummaryTable" displayName="WarningSummaryTable" ref="F5:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="汇总指标"/>
@@ -1240,7 +1826,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WarningQueueTable" displayName="WarningQueueTable" ref="A13:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="商品ID"/>
@@ -1256,111 +1842,13 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="WarningRulesTable" displayName="WarningRulesTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="预警指标"/>
     <x:tableColumn id="2" name="触发条件"/>
     <x:tableColumn id="3" name="建议节点"/>
     <x:tableColumn id="4" name="启用"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="WarningSummaryTable" displayName="WarningSummaryTable" ref="F5:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="3">
-    <x:tableColumn id="1" name="汇总指标"/>
-    <x:tableColumn id="2" name="当前值"/>
-    <x:tableColumn id="3" name="说明"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="WarningQueueTable" displayName="WarningQueueTable" ref="A13:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="8">
-    <x:tableColumn id="1" name="商品ID"/>
-    <x:tableColumn id="2" name="店铺"/>
-    <x:tableColumn id="3" name="预警类型"/>
-    <x:tableColumn id="4" name="当前指标"/>
-    <x:tableColumn id="5" name="变化值"/>
-    <x:tableColumn id="6" name="建议动作"/>
-    <x:tableColumn id="7" name="处理状态"/>
-    <x:tableColumn id="8" name="证据/备注"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="10">
-    <x:tableColumn id="1" name="方法ID"/>
-    <x:tableColumn id="2" name="方法标题"/>
-    <x:tableColumn id="3" name="分类"/>
-    <x:tableColumn id="4" name="适用场景"/>
-    <x:tableColumn id="5" name="验证商品/对象"/>
-    <x:tableColumn id="6" name="证据摘要"/>
-    <x:tableColumn id="7" name="验证状态"/>
-    <x:tableColumn id="8" name="负责人"/>
-    <x:tableColumn id="9" name="复用次数"/>
-    <x:tableColumn id="10" name="备注"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="10">
-    <x:tableColumn id="1" name="方法ID"/>
-    <x:tableColumn id="2" name="方法标题"/>
-    <x:tableColumn id="3" name="分类"/>
-    <x:tableColumn id="4" name="适用场景"/>
-    <x:tableColumn id="5" name="验证商品/对象"/>
-    <x:tableColumn id="6" name="证据摘要"/>
-    <x:tableColumn id="7" name="验证状态"/>
-    <x:tableColumn id="8" name="负责人"/>
-    <x:tableColumn id="9" name="复用次数"/>
-    <x:tableColumn id="10" name="备注"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="10">
-    <x:tableColumn id="1" name="方法ID"/>
-    <x:tableColumn id="2" name="方法标题"/>
-    <x:tableColumn id="3" name="分类"/>
-    <x:tableColumn id="4" name="适用场景"/>
-    <x:tableColumn id="5" name="验证商品/对象"/>
-    <x:tableColumn id="6" name="证据摘要"/>
-    <x:tableColumn id="7" name="验证状态"/>
-    <x:tableColumn id="8" name="负责人"/>
-    <x:tableColumn id="9" name="复用次数"/>
-    <x:tableColumn id="10" name="备注"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="AgentDispatchTable" displayName="AgentDispatchTable" ref="A5:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="9">
-    <x:tableColumn id="1" name="任务日期"/>
-    <x:tableColumn id="2" name="Agent名称"/>
-    <x:tableColumn id="3" name="触发入口"/>
-    <x:tableColumn id="4" name="输入范围"/>
-    <x:tableColumn id="5" name="任务目标"/>
-    <x:tableColumn id="6" name="输出物"/>
-    <x:tableColumn id="7" name="状态"/>
-    <x:tableColumn id="8" name="复核人"/>
-    <x:tableColumn id="9" name="备注"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1380,6 +1868,177 @@
 </file>
 
 <file path=xl/tables/table40.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="WarningSummaryTable" displayName="WarningSummaryTable" ref="F5:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="汇总指标"/>
+    <x:tableColumn id="2" name="当前值"/>
+    <x:tableColumn id="3" name="说明"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table41.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="WarningQueueTable" displayName="WarningQueueTable" ref="A13:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="商品ID"/>
+    <x:tableColumn id="2" name="店铺"/>
+    <x:tableColumn id="3" name="预警类型"/>
+    <x:tableColumn id="4" name="当前指标"/>
+    <x:tableColumn id="5" name="变化值"/>
+    <x:tableColumn id="6" name="建议动作"/>
+    <x:tableColumn id="7" name="处理状态"/>
+    <x:tableColumn id="8" name="证据/备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table42.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="WarningRulesTable" displayName="WarningRulesTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="预警指标"/>
+    <x:tableColumn id="2" name="触发条件"/>
+    <x:tableColumn id="3" name="建议节点"/>
+    <x:tableColumn id="4" name="启用"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table43.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="WarningSummaryTable" displayName="WarningSummaryTable" ref="F5:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="汇总指标"/>
+    <x:tableColumn id="2" name="当前值"/>
+    <x:tableColumn id="3" name="说明"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table44.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="WarningQueueTable" displayName="WarningQueueTable" ref="A13:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="商品ID"/>
+    <x:tableColumn id="2" name="店铺"/>
+    <x:tableColumn id="3" name="预警类型"/>
+    <x:tableColumn id="4" name="当前指标"/>
+    <x:tableColumn id="5" name="变化值"/>
+    <x:tableColumn id="6" name="建议动作"/>
+    <x:tableColumn id="7" name="处理状态"/>
+    <x:tableColumn id="8" name="证据/备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table45.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="方法ID"/>
+    <x:tableColumn id="2" name="方法标题"/>
+    <x:tableColumn id="3" name="分类"/>
+    <x:tableColumn id="4" name="适用场景"/>
+    <x:tableColumn id="5" name="验证商品/对象"/>
+    <x:tableColumn id="6" name="证据摘要"/>
+    <x:tableColumn id="7" name="验证状态"/>
+    <x:tableColumn id="8" name="负责人"/>
+    <x:tableColumn id="9" name="复用次数"/>
+    <x:tableColumn id="10" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table46.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="方法ID"/>
+    <x:tableColumn id="2" name="方法标题"/>
+    <x:tableColumn id="3" name="分类"/>
+    <x:tableColumn id="4" name="适用场景"/>
+    <x:tableColumn id="5" name="验证商品/对象"/>
+    <x:tableColumn id="6" name="证据摘要"/>
+    <x:tableColumn id="7" name="验证状态"/>
+    <x:tableColumn id="8" name="负责人"/>
+    <x:tableColumn id="9" name="复用次数"/>
+    <x:tableColumn id="10" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table47.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="方法ID"/>
+    <x:tableColumn id="2" name="方法标题"/>
+    <x:tableColumn id="3" name="分类"/>
+    <x:tableColumn id="4" name="适用场景"/>
+    <x:tableColumn id="5" name="验证商品/对象"/>
+    <x:tableColumn id="6" name="证据摘要"/>
+    <x:tableColumn id="7" name="验证状态"/>
+    <x:tableColumn id="8" name="负责人"/>
+    <x:tableColumn id="9" name="复用次数"/>
+    <x:tableColumn id="10" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table48.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="KnowledgeBaseTable" displayName="KnowledgeBaseTable" ref="A5:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="方法ID"/>
+    <x:tableColumn id="2" name="方法标题"/>
+    <x:tableColumn id="3" name="分类"/>
+    <x:tableColumn id="4" name="适用场景"/>
+    <x:tableColumn id="5" name="验证商品/对象"/>
+    <x:tableColumn id="6" name="证据摘要"/>
+    <x:tableColumn id="7" name="验证状态"/>
+    <x:tableColumn id="8" name="负责人"/>
+    <x:tableColumn id="9" name="复用次数"/>
+    <x:tableColumn id="10" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table49.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="AgentDispatchTable" displayName="AgentDispatchTable" ref="A5:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="任务日期"/>
+    <x:tableColumn id="2" name="Agent名称"/>
+    <x:tableColumn id="3" name="触发入口"/>
+    <x:tableColumn id="4" name="输入范围"/>
+    <x:tableColumn id="5" name="任务目标"/>
+    <x:tableColumn id="6" name="输出物"/>
+    <x:tableColumn id="7" name="状态"/>
+    <x:tableColumn id="8" name="复核人"/>
+    <x:tableColumn id="9" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CreatorSummaryTable" displayName="CreatorSummaryTable" ref="A5:G6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:G6"/>
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="店铺"/>
+    <x:tableColumn id="2" name="合作中达人"/>
+    <x:tableColumn id="3" name="待跟进"/>
+    <x:tableColumn id="4" name="本周交付视频"/>
+    <x:tableColumn id="5" name="履约率(%)"/>
+    <x:tableColumn id="6" name="状态"/>
+    <x:tableColumn id="7" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table50.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="AgentDispatchTable" displayName="AgentDispatchTable" ref="A5:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="任务日期"/>
@@ -1396,7 +2055,7 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table51.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="AgentDispatchTable" displayName="AgentDispatchTable" ref="A5:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="任务日期"/>
@@ -1413,7 +2072,24 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table52.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="AgentDispatchTable" displayName="AgentDispatchTable" ref="A5:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="任务日期"/>
+    <x:tableColumn id="2" name="Agent名称"/>
+    <x:tableColumn id="3" name="触发入口"/>
+    <x:tableColumn id="4" name="输入范围"/>
+    <x:tableColumn id="5" name="任务目标"/>
+    <x:tableColumn id="6" name="输出物"/>
+    <x:tableColumn id="7" name="状态"/>
+    <x:tableColumn id="8" name="复核人"/>
+    <x:tableColumn id="9" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table53.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="CloudGuideTable" displayName="CloudGuideTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="步骤"/>
@@ -1425,17 +2101,13 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CreatorSummaryTable" displayName="CreatorSummaryTable" ref="A5:G6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:G6"/>
-  <x:tableColumns count="7">
-    <x:tableColumn id="1" name="店铺"/>
-    <x:tableColumn id="2" name="合作中达人"/>
-    <x:tableColumn id="3" name="待跟进"/>
-    <x:tableColumn id="4" name="本周交付视频"/>
-    <x:tableColumn id="5" name="履约率(%)"/>
-    <x:tableColumn id="6" name="状态"/>
-    <x:tableColumn id="7" name="备注"/>
+<file path=xl/tables/table54.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="CloudGuideTable" displayName="CloudGuideTable" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="步骤"/>
+    <x:tableColumn id="2" name="运营操作"/>
+    <x:tableColumn id="3" name="涉及工作表"/>
+    <x:tableColumn id="4" name="网站对应页面"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1743,35 +2415,35 @@
       <x:c r="H3" s="3"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="11" t="str">
+      <x:c r="A4" s="197" t="str">
         <x:v>使用步骤</x:v>
       </x:c>
-      <x:c r="B4" s="11" t="str">
+      <x:c r="B4" s="198" t="str">
         <x:v>说明</x:v>
       </x:c>
       <x:c r="C4" s="3"/>
-      <x:c r="D4" s="11" t="str">
+      <x:c r="D4" s="197" t="str">
         <x:v>当前模板概览</x:v>
       </x:c>
-      <x:c r="E4" s="11" t="str">
+      <x:c r="E4" s="198" t="str">
         <x:v>数量</x:v>
       </x:c>
       <x:c r="F4" s="3"/>
       <x:c r="G4" s="3"/>
       <x:c r="H4" s="3"/>
     </x:row>
-    <x:row r="5" ht="24" customHeight="1">
-      <x:c r="A5" s="13" t="str">
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="219" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B5" s="13" t="str">
+      <x:c r="B5" s="204" t="str">
         <x:v>把本文件上传到 WPS/Kdocs，作为团队唯一的数据填报表。</x:v>
       </x:c>
       <x:c r="C5" s="3"/>
-      <x:c r="D5" s="15" t="str">
+      <x:c r="D5" s="211" t="str">
         <x:v>店铺</x:v>
       </x:c>
-      <x:c r="E5" s="15" t="n">
+      <x:c r="E5" s="225" t="n">
         <x:f>COUNTA('店铺日汇总'!B6:B105)</x:f>
         <x:v>4</x:v>
       </x:c>
@@ -1779,18 +2451,18 @@
       <x:c r="G5" s="3"/>
       <x:c r="H5" s="3"/>
     </x:row>
-    <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="13" t="str">
+    <x:row r="6" ht="30" customHeight="1">
+      <x:c r="A6" s="219" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B6" s="13" t="str">
+      <x:c r="B6" s="204" t="str">
         <x:v>运营只编辑黄色输入区域，不要修改表头和字段名。</x:v>
       </x:c>
       <x:c r="C6" s="3"/>
-      <x:c r="D6" s="15" t="str">
+      <x:c r="D6" s="211" t="str">
         <x:v>商品记录</x:v>
       </x:c>
-      <x:c r="E6" s="15" t="n">
+      <x:c r="E6" s="225" t="n">
         <x:f>COUNTA('商品数据'!C6:C105)</x:f>
         <x:v>6</x:v>
       </x:c>
@@ -1798,18 +2470,18 @@
       <x:c r="G6" s="3"/>
       <x:c r="H6" s="3"/>
     </x:row>
-    <x:row r="7" ht="24" customHeight="1">
-      <x:c r="A7" s="13" t="str">
+    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="A7" s="219" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B7" s="13" t="str">
+      <x:c r="B7" s="204" t="str">
         <x:v>每天补充店铺汇总、商品数据和已执行动作；缺失数据留空。</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
-      <x:c r="D7" s="15" t="str">
+      <x:c r="D7" s="211" t="str">
         <x:v>运营动作</x:v>
       </x:c>
-      <x:c r="E7" s="15" t="n">
+      <x:c r="E7" s="225" t="n">
         <x:f>COUNTA('运营动作'!D6:D105)</x:f>
         <x:v>5</x:v>
       </x:c>
@@ -1817,18 +2489,18 @@
       <x:c r="G7" s="3"/>
       <x:c r="H7" s="3"/>
     </x:row>
-    <x:row r="8" ht="24" customHeight="1">
-      <x:c r="A8" s="13" t="str">
+    <x:row r="8" ht="30" customHeight="1">
+      <x:c r="A8" s="219" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B8" s="13" t="str">
+      <x:c r="B8" s="204" t="str">
         <x:v>维护完成后导出对应 CSV，或将公开数据链接接入网站同步。</x:v>
       </x:c>
       <x:c r="C8" s="3"/>
-      <x:c r="D8" s="15" t="str">
+      <x:c r="D8" s="211" t="str">
         <x:v>广告计划</x:v>
       </x:c>
-      <x:c r="E8" s="15" t="n">
+      <x:c r="E8" s="225" t="n">
         <x:f>COUNTA('广告计划'!C6:C105)</x:f>
         <x:v>3</x:v>
       </x:c>
@@ -1836,18 +2508,18 @@
       <x:c r="G8" s="3"/>
       <x:c r="H8" s="3"/>
     </x:row>
-    <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="13" t="str">
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="220" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B9" s="13" t="str">
+      <x:c r="B9" s="206" t="str">
         <x:v>有效/无效必须有 T+1、T+3、T+7 的真实证据，不能凭感觉填写。</x:v>
       </x:c>
       <x:c r="C9" s="3"/>
-      <x:c r="D9" s="15" t="str">
+      <x:c r="D9" s="213" t="str">
         <x:v>发布趋势记录</x:v>
       </x:c>
-      <x:c r="E9" s="15" t="n">
+      <x:c r="E9" s="226" t="n">
         <x:f>COUNTA('发布趋势'!A6:A105)</x:f>
         <x:v>7</x:v>
       </x:c>
@@ -2003,98 +2675,98 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="145" t="str">
+      <x:c r="A1" s="173" t="str">
         <x:v>店铺字典｜网站筛选来源</x:v>
       </x:c>
-      <x:c r="B1" s="145"/>
-      <x:c r="C1" s="145"/>
-      <x:c r="D1" s="145"/>
+      <x:c r="B1" s="173"/>
+      <x:c r="C1" s="173"/>
+      <x:c r="D1" s="173"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
-      <x:c r="A2" s="146" t="str">
+      <x:c r="A2" s="174" t="str">
         <x:v>真实店铺上线前请把黄色示例名称替换为团队实际店铺；“全部店铺”只作为汇总口径，不是一个真实店铺。</x:v>
       </x:c>
-      <x:c r="B2" s="146"/>
-      <x:c r="C2" s="146"/>
-      <x:c r="D2" s="146"/>
+      <x:c r="B2" s="174"/>
+      <x:c r="C2" s="174"/>
+      <x:c r="D2" s="174"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="147" t="str">
+      <x:c r="A5" s="260" t="str">
         <x:v>店铺名称</x:v>
       </x:c>
-      <x:c r="B5" s="147" t="str">
+      <x:c r="B5" s="261" t="str">
         <x:v>店铺编码</x:v>
       </x:c>
-      <x:c r="C5" s="147" t="str">
+      <x:c r="C5" s="261" t="str">
         <x:v>市场/用途</x:v>
       </x:c>
-      <x:c r="D5" s="147" t="str">
+      <x:c r="D5" s="262" t="str">
         <x:v>状态</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="148" t="str">
+      <x:c r="A6" s="304" t="str">
         <x:v>全部店铺</x:v>
       </x:c>
-      <x:c r="B6" s="148" t="str">
+      <x:c r="B6" s="299" t="str">
         <x:v>ALL</x:v>
       </x:c>
-      <x:c r="C6" s="148" t="str">
+      <x:c r="C6" s="299" t="str">
         <x:v>跨店汇总口径</x:v>
       </x:c>
-      <x:c r="D6" s="148" t="str">
+      <x:c r="D6" s="305" t="str">
         <x:v>汇总</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="148" t="str">
+      <x:c r="A7" s="263" t="str">
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="B7" s="148" t="str">
+      <x:c r="B7" s="264" t="str">
         <x:v>US-MAIN</x:v>
       </x:c>
-      <x:c r="C7" s="148" t="str">
+      <x:c r="C7" s="264" t="str">
         <x:v>美国站主店</x:v>
       </x:c>
-      <x:c r="D7" s="148" t="str">
+      <x:c r="D7" s="265" t="str">
         <x:v>示例</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="148" t="str">
+      <x:c r="A8" s="263" t="str">
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="B8" s="148" t="str">
+      <x:c r="B8" s="264" t="str">
         <x:v>US-DAY</x:v>
       </x:c>
-      <x:c r="C8" s="148" t="str">
+      <x:c r="C8" s="264" t="str">
         <x:v>美国站日用店</x:v>
       </x:c>
-      <x:c r="D8" s="148" t="str">
+      <x:c r="D8" s="265" t="str">
         <x:v>示例</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="148" t="str">
+      <x:c r="A9" s="266" t="str">
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="B9" s="148" t="str">
+      <x:c r="B9" s="267" t="str">
         <x:v>TH-MAIN</x:v>
       </x:c>
-      <x:c r="C9" s="148" t="str">
+      <x:c r="C9" s="267" t="str">
         <x:v>泰国站主店</x:v>
       </x:c>
-      <x:c r="D9" s="148" t="str">
+      <x:c r="D9" s="268" t="str">
         <x:v>示例</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
-      <x:c r="A11" s="149" t="str">
+      <x:c r="A11" s="177" t="str">
         <x:v>填写规则：网站顶部的“全部店铺 / 单店”筛选，应与本表店铺名称、店铺日汇总、商品数据、运营动作中的店铺字段完全一致。</x:v>
       </x:c>
-      <x:c r="B11" s="149"/>
-      <x:c r="C11" s="149"/>
-      <x:c r="D11" s="149"/>
+      <x:c r="B11" s="177"/>
+      <x:c r="C11" s="177"/>
+      <x:c r="D11" s="177"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2103,10 +2775,11 @@
     <x:mergeCell ref="A11:D11"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R777edd9b2f374033"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fa4c4aa255048e1"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4eb7d9fd69e44dfe"/>
+  <x:tableParts count="4">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02a9cc53e4e24981"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79f1b320cb7942c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06000813a4584e31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4a6ad3fcb024f8d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2124,797 +2797,797 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="145" t="str">
+      <x:c r="A1" s="173" t="str">
         <x:v>五组链接对比排行｜网站经营总览</x:v>
       </x:c>
-      <x:c r="B1" s="145"/>
-      <x:c r="C1" s="145"/>
-      <x:c r="D1" s="145"/>
-      <x:c r="E1" s="145"/>
-      <x:c r="F1" s="145"/>
+      <x:c r="B1" s="173"/>
+      <x:c r="C1" s="173"/>
+      <x:c r="D1" s="173"/>
+      <x:c r="E1" s="173"/>
+      <x:c r="F1" s="173"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
-      <x:c r="A2" s="146" t="str">
+      <x:c r="A2" s="174" t="str">
         <x:v>蓝色区域为公式结果；公式从“商品数据”读取，运营只需更新商品数据。缺少上一周期数据时，GMV/CVR 变化不要填 0。</x:v>
       </x:c>
-      <x:c r="B2" s="146"/>
-      <x:c r="C2" s="146"/>
-      <x:c r="D2" s="146"/>
-      <x:c r="E2" s="146"/>
-      <x:c r="F2" s="146"/>
+      <x:c r="B2" s="174"/>
+      <x:c r="C2" s="174"/>
+      <x:c r="D2" s="174"/>
+      <x:c r="E2" s="174"/>
+      <x:c r="F2" s="174"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="150" t="str">
+      <x:c r="A4" s="178" t="str">
         <x:v>销量 Top5｜按成交销量降序</x:v>
       </x:c>
-      <x:c r="B4" s="150"/>
-      <x:c r="C4" s="150"/>
-      <x:c r="D4" s="150"/>
-      <x:c r="E4" s="150"/>
-      <x:c r="F4" s="150"/>
+      <x:c r="B4" s="178"/>
+      <x:c r="C4" s="178"/>
+      <x:c r="D4" s="178"/>
+      <x:c r="E4" s="178"/>
+      <x:c r="F4" s="178"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="147" t="str">
+      <x:c r="A5" s="175" t="str">
         <x:v>排名</x:v>
       </x:c>
-      <x:c r="B5" s="147" t="str">
+      <x:c r="B5" s="175" t="str">
         <x:v>商品ID</x:v>
       </x:c>
-      <x:c r="C5" s="147" t="str">
+      <x:c r="C5" s="175" t="str">
         <x:v>商品名称</x:v>
       </x:c>
-      <x:c r="D5" s="147" t="str">
+      <x:c r="D5" s="175" t="str">
         <x:v>店铺</x:v>
       </x:c>
-      <x:c r="E5" s="147" t="str">
+      <x:c r="E5" s="175" t="str">
         <x:v>指标值</x:v>
       </x:c>
-      <x:c r="F5" s="147" t="str">
+      <x:c r="F5" s="175" t="str">
         <x:v>口径</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="151" t="n">
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="227" t="n">
         <x:f>ROW()-5</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B6" s="151" t="n">
+      <x:c r="B6" s="228" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E6,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>100176</x:v>
       </x:c>
-      <x:c r="C6" s="151" t="str">
+      <x:c r="C6" s="228" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E6,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>3D磁吸积木套装</x:v>
       </x:c>
-      <x:c r="D6" s="151" t="str">
+      <x:c r="D6" s="228" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E6,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E6" s="152" t="n">
+      <x:c r="E6" s="229" t="n">
         <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
         <x:v>428</x:v>
       </x:c>
-      <x:c r="F6" s="151" t="str">
+      <x:c r="F6" s="230" t="str">
         <x:v>按成交销量降序</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="151" t="n">
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="231" t="n">
         <x:f>ROW()-5</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B7" s="151" t="n">
+      <x:c r="B7" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E7,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="C7" s="151" t="str">
+      <x:c r="C7" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E7,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>儿童户外泡泡机</x:v>
       </x:c>
-      <x:c r="D7" s="151" t="str">
+      <x:c r="D7" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E7,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E7" s="152" t="n">
+      <x:c r="E7" s="233" t="n">
         <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
         <x:v>198</x:v>
       </x:c>
-      <x:c r="F7" s="151" t="str">
+      <x:c r="F7" s="234" t="str">
         <x:v>按成交销量降序</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="151" t="n">
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="231" t="n">
         <x:f>ROW()-5</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B8" s="151" t="n">
+      <x:c r="B8" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E8,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>100091</x:v>
       </x:c>
-      <x:c r="C8" s="151" t="str">
+      <x:c r="C8" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E8,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>益智拼图礼盒</x:v>
       </x:c>
-      <x:c r="D8" s="151" t="str">
+      <x:c r="D8" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E8,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E8" s="152" t="n">
+      <x:c r="E8" s="233" t="n">
         <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
         <x:v>176</x:v>
       </x:c>
-      <x:c r="F8" s="151" t="str">
+      <x:c r="F8" s="234" t="str">
         <x:v>按成交销量降序</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="151" t="n">
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="231" t="n">
         <x:f>ROW()-5</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B9" s="151" t="n">
+      <x:c r="B9" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E9,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>100314</x:v>
       </x:c>
-      <x:c r="C9" s="151" t="str">
+      <x:c r="C9" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E9,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>儿童绘画水彩笔</x:v>
       </x:c>
-      <x:c r="D9" s="151" t="str">
+      <x:c r="D9" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E9,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E9" s="152" t="n">
+      <x:c r="E9" s="233" t="n">
         <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
         <x:v>142</x:v>
       </x:c>
-      <x:c r="F9" s="151" t="str">
+      <x:c r="F9" s="234" t="str">
         <x:v>按成交销量降序</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="151" t="n">
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="235" t="n">
         <x:f>ROW()-5</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B10" s="151" t="n">
+      <x:c r="B10" s="236" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E10,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>100407</x:v>
       </x:c>
-      <x:c r="C10" s="151" t="str">
+      <x:c r="C10" s="236" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E10,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>磁力迷宫玩具</x:v>
       </x:c>
-      <x:c r="D10" s="151" t="str">
+      <x:c r="D10" s="236" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E10,'商品数据'!$I$6:$I$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E10" s="152" t="n">
+      <x:c r="E10" s="237" t="n">
         <x:f>LARGE('商品数据'!$I$6:$I$11,ROW()-5)</x:f>
         <x:v>94</x:v>
       </x:c>
-      <x:c r="F10" s="151" t="str">
+      <x:c r="F10" s="238" t="str">
         <x:v>按成交销量降序</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="150" t="str">
+      <x:c r="A12" s="178" t="str">
         <x:v>全店 GMV Top5｜按商品链接 GMV 降序</x:v>
       </x:c>
-      <x:c r="B12" s="150"/>
-      <x:c r="C12" s="150"/>
-      <x:c r="D12" s="150"/>
-      <x:c r="E12" s="150"/>
-      <x:c r="F12" s="150"/>
+      <x:c r="B12" s="178"/>
+      <x:c r="C12" s="178"/>
+      <x:c r="D12" s="178"/>
+      <x:c r="E12" s="178"/>
+      <x:c r="F12" s="178"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="str">
+      <x:c r="A13" s="241" t="str">
         <x:v>排名</x:v>
       </x:c>
-      <x:c r="B13" t="str">
+      <x:c r="B13" s="241" t="str">
         <x:v>商品ID</x:v>
       </x:c>
-      <x:c r="C13" t="str">
+      <x:c r="C13" s="241" t="str">
         <x:v>商品名称</x:v>
       </x:c>
-      <x:c r="D13" t="str">
+      <x:c r="D13" s="241" t="str">
         <x:v>店铺</x:v>
       </x:c>
-      <x:c r="E13" t="str">
+      <x:c r="E13" s="241" t="str">
         <x:v>指标值</x:v>
       </x:c>
-      <x:c r="F13" t="str">
+      <x:c r="F13" s="241" t="str">
         <x:v>口径</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="151" t="n">
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="227" t="n">
         <x:f>ROW()-13</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B14" s="151" t="n">
+      <x:c r="B14" s="228" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E14,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>100176</x:v>
       </x:c>
-      <x:c r="C14" s="151" t="str">
+      <x:c r="C14" s="228" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E14,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>3D磁吸积木套装</x:v>
       </x:c>
-      <x:c r="D14" s="151" t="str">
+      <x:c r="D14" s="228" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E14,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E14" s="153" t="n">
+      <x:c r="E14" s="242" t="n">
         <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
         <x:v>42680</x:v>
       </x:c>
-      <x:c r="F14" s="151" t="str">
+      <x:c r="F14" s="230" t="str">
         <x:v>按商品链接 GMV 降序</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="151" t="n">
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="231" t="n">
         <x:f>ROW()-13</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B15" s="151" t="n">
+      <x:c r="B15" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E15,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="C15" s="151" t="str">
+      <x:c r="C15" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E15,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>儿童户外泡泡机</x:v>
       </x:c>
-      <x:c r="D15" s="151" t="str">
+      <x:c r="D15" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E15,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E15" s="153" t="n">
+      <x:c r="E15" s="243" t="n">
         <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
         <x:v>18420</x:v>
       </x:c>
-      <x:c r="F15" s="151" t="str">
+      <x:c r="F15" s="234" t="str">
         <x:v>按商品链接 GMV 降序</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="151" t="n">
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="231" t="n">
         <x:f>ROW()-13</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B16" s="151" t="n">
+      <x:c r="B16" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E16,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>100091</x:v>
       </x:c>
-      <x:c r="C16" s="151" t="str">
+      <x:c r="C16" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E16,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>益智拼图礼盒</x:v>
       </x:c>
-      <x:c r="D16" s="151" t="str">
+      <x:c r="D16" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E16,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E16" s="153" t="n">
+      <x:c r="E16" s="243" t="n">
         <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
         <x:v>15760</x:v>
       </x:c>
-      <x:c r="F16" s="151" t="str">
+      <x:c r="F16" s="234" t="str">
         <x:v>按商品链接 GMV 降序</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="151" t="n">
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="231" t="n">
         <x:f>ROW()-13</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B17" s="151" t="n">
+      <x:c r="B17" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E17,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>100314</x:v>
       </x:c>
-      <x:c r="C17" s="151" t="str">
+      <x:c r="C17" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E17,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>儿童绘画水彩笔</x:v>
       </x:c>
-      <x:c r="D17" s="151" t="str">
+      <x:c r="D17" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E17,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E17" s="153" t="n">
+      <x:c r="E17" s="243" t="n">
         <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
         <x:v>12360</x:v>
       </x:c>
-      <x:c r="F17" s="151" t="str">
+      <x:c r="F17" s="234" t="str">
         <x:v>按商品链接 GMV 降序</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="151" t="n">
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" s="235" t="n">
         <x:f>ROW()-13</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B18" s="151" t="n">
+      <x:c r="B18" s="236" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E18,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>100407</x:v>
       </x:c>
-      <x:c r="C18" s="151" t="str">
+      <x:c r="C18" s="236" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E18,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>磁力迷宫玩具</x:v>
       </x:c>
-      <x:c r="D18" s="151" t="str">
+      <x:c r="D18" s="236" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E18,'商品数据'!$J$6:$J$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E18" s="153" t="n">
+      <x:c r="E18" s="244" t="n">
         <x:f>LARGE('商品数据'!$J$6:$J$11,ROW()-13)</x:f>
         <x:v>8120</x:v>
       </x:c>
-      <x:c r="F18" s="151" t="str">
+      <x:c r="F18" s="238" t="str">
         <x:v>按商品链接 GMV 降序</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="150" t="str">
+      <x:c r="A20" s="178" t="str">
         <x:v>GMV 上涨 Top5｜按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
       </x:c>
-      <x:c r="B20" s="150"/>
-      <x:c r="C20" s="150"/>
-      <x:c r="D20" s="150"/>
-      <x:c r="E20" s="150"/>
-      <x:c r="F20" s="150"/>
+      <x:c r="B20" s="178"/>
+      <x:c r="C20" s="178"/>
+      <x:c r="D20" s="178"/>
+      <x:c r="E20" s="178"/>
+      <x:c r="F20" s="178"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" t="str">
+      <x:c r="A21" s="247" t="str">
         <x:v>排名</x:v>
       </x:c>
-      <x:c r="B21" t="str">
+      <x:c r="B21" s="247" t="str">
         <x:v>商品ID</x:v>
       </x:c>
-      <x:c r="C21" t="str">
+      <x:c r="C21" s="247" t="str">
         <x:v>商品名称</x:v>
       </x:c>
-      <x:c r="D21" t="str">
+      <x:c r="D21" s="247" t="str">
         <x:v>店铺</x:v>
       </x:c>
-      <x:c r="E21" t="str">
+      <x:c r="E21" s="247" t="str">
         <x:v>指标值</x:v>
       </x:c>
-      <x:c r="F21" t="str">
+      <x:c r="F21" s="247" t="str">
         <x:v>口径</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="151" t="n">
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="227" t="n">
         <x:f>ROW()-21</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B22" s="151" t="n">
+      <x:c r="B22" s="228" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E22,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100314</x:v>
       </x:c>
-      <x:c r="C22" s="151" t="str">
+      <x:c r="C22" s="228" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E22,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>儿童绘画水彩笔</x:v>
       </x:c>
-      <x:c r="D22" s="151" t="str">
+      <x:c r="D22" s="228" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E22,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E22" s="154" t="n">
+      <x:c r="E22" s="248" t="n">
         <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
         <x:v>24.1</x:v>
       </x:c>
-      <x:c r="F22" s="151" t="str">
+      <x:c r="F22" s="230" t="str">
         <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="151" t="n">
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="231" t="n">
         <x:f>ROW()-21</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B23" s="151" t="n">
+      <x:c r="B23" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E23,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100176</x:v>
       </x:c>
-      <x:c r="C23" s="151" t="str">
+      <x:c r="C23" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E23,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>3D磁吸积木套装</x:v>
       </x:c>
-      <x:c r="D23" s="151" t="str">
+      <x:c r="D23" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E23,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E23" s="154" t="n">
+      <x:c r="E23" s="249" t="n">
         <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
         <x:v>18.6</x:v>
       </x:c>
-      <x:c r="F23" s="151" t="str">
+      <x:c r="F23" s="234" t="str">
         <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="151" t="n">
+    <x:row r="24" ht="22" customHeight="1">
+      <x:c r="A24" s="231" t="n">
         <x:f>ROW()-21</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B24" s="151" t="n">
+      <x:c r="B24" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E24,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100091</x:v>
       </x:c>
-      <x:c r="C24" s="151" t="str">
+      <x:c r="C24" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E24,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>益智拼图礼盒</x:v>
       </x:c>
-      <x:c r="D24" s="151" t="str">
+      <x:c r="D24" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E24,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E24" s="154" t="n">
+      <x:c r="E24" s="249" t="n">
         <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
         <x:v>6.8</x:v>
       </x:c>
-      <x:c r="F24" s="151" t="str">
+      <x:c r="F24" s="234" t="str">
         <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="151" t="n">
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="231" t="n">
         <x:f>ROW()-21</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B25" s="151" t="n">
+      <x:c r="B25" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E25,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100512</x:v>
       </x:c>
-      <x:c r="C25" s="151" t="str">
+      <x:c r="C25" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E25,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>折叠儿童画板</x:v>
       </x:c>
-      <x:c r="D25" s="151" t="str">
+      <x:c r="D25" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E25,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E25" s="154" t="n">
+      <x:c r="E25" s="249" t="n">
         <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
         <x:v>-3.7</x:v>
       </x:c>
-      <x:c r="F25" s="151" t="str">
+      <x:c r="F25" s="234" t="str">
         <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="151" t="n">
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="235" t="n">
         <x:f>ROW()-21</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B26" s="151" t="n">
+      <x:c r="B26" s="236" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E26,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="C26" s="151" t="str">
+      <x:c r="C26" s="236" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E26,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>儿童户外泡泡机</x:v>
       </x:c>
-      <x:c r="D26" s="151" t="str">
+      <x:c r="D26" s="236" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E26,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E26" s="154" t="n">
+      <x:c r="E26" s="250" t="n">
         <x:f>LARGE('商品数据'!$K$6:$K$11,ROW()-21)</x:f>
         <x:v>-12.4</x:v>
       </x:c>
-      <x:c r="F26" s="151" t="str">
+      <x:c r="F26" s="238" t="str">
         <x:v>按 GMV 环比/上一周期变化降序，数值单位为 %</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="150" t="str">
+      <x:c r="A28" s="178" t="str">
         <x:v>GMV 下降 Top5｜按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
       </x:c>
-      <x:c r="B28" s="150"/>
-      <x:c r="C28" s="150"/>
-      <x:c r="D28" s="150"/>
-      <x:c r="E28" s="150"/>
-      <x:c r="F28" s="150"/>
+      <x:c r="B28" s="178"/>
+      <x:c r="C28" s="178"/>
+      <x:c r="D28" s="178"/>
+      <x:c r="E28" s="178"/>
+      <x:c r="F28" s="178"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" t="str">
+      <x:c r="A29" s="253" t="str">
         <x:v>排名</x:v>
       </x:c>
-      <x:c r="B29" t="str">
+      <x:c r="B29" s="253" t="str">
         <x:v>商品ID</x:v>
       </x:c>
-      <x:c r="C29" t="str">
+      <x:c r="C29" s="253" t="str">
         <x:v>商品名称</x:v>
       </x:c>
-      <x:c r="D29" t="str">
+      <x:c r="D29" s="253" t="str">
         <x:v>店铺</x:v>
       </x:c>
-      <x:c r="E29" t="str">
+      <x:c r="E29" s="253" t="str">
         <x:v>指标值</x:v>
       </x:c>
-      <x:c r="F29" t="str">
+      <x:c r="F29" s="253" t="str">
         <x:v>口径</x:v>
       </x:c>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="151" t="n">
+    <x:row r="30" ht="22" customHeight="1">
+      <x:c r="A30" s="227" t="n">
         <x:f>ROW()-29</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B30" s="151" t="n">
+      <x:c r="B30" s="228" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E30,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100407</x:v>
       </x:c>
-      <x:c r="C30" s="151" t="str">
+      <x:c r="C30" s="228" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E30,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>磁力迷宫玩具</x:v>
       </x:c>
-      <x:c r="D30" s="151" t="str">
+      <x:c r="D30" s="228" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E30,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E30" s="154" t="n">
+      <x:c r="E30" s="248" t="n">
         <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
         <x:v>-26.5</x:v>
       </x:c>
-      <x:c r="F30" s="151" t="str">
+      <x:c r="F30" s="230" t="str">
         <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
       </x:c>
     </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="151" t="n">
+    <x:row r="31" ht="22" customHeight="1">
+      <x:c r="A31" s="231" t="n">
         <x:f>ROW()-29</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B31" s="151" t="n">
+      <x:c r="B31" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E31,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="C31" s="151" t="str">
+      <x:c r="C31" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E31,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>儿童户外泡泡机</x:v>
       </x:c>
-      <x:c r="D31" s="151" t="str">
+      <x:c r="D31" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E31,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E31" s="154" t="n">
+      <x:c r="E31" s="249" t="n">
         <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
         <x:v>-12.4</x:v>
       </x:c>
-      <x:c r="F31" s="151" t="str">
+      <x:c r="F31" s="234" t="str">
         <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
       </x:c>
     </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="151" t="n">
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="A32" s="231" t="n">
         <x:f>ROW()-29</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B32" s="151" t="n">
+      <x:c r="B32" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E32,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100512</x:v>
       </x:c>
-      <x:c r="C32" s="151" t="str">
+      <x:c r="C32" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E32,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>折叠儿童画板</x:v>
       </x:c>
-      <x:c r="D32" s="151" t="str">
+      <x:c r="D32" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E32,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E32" s="154" t="n">
+      <x:c r="E32" s="249" t="n">
         <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
         <x:v>-3.7</x:v>
       </x:c>
-      <x:c r="F32" s="151" t="str">
+      <x:c r="F32" s="234" t="str">
         <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
       </x:c>
     </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="151" t="n">
+    <x:row r="33" ht="22" customHeight="1">
+      <x:c r="A33" s="231" t="n">
         <x:f>ROW()-29</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B33" s="151" t="n">
+      <x:c r="B33" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E33,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100091</x:v>
       </x:c>
-      <x:c r="C33" s="151" t="str">
+      <x:c r="C33" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E33,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>益智拼图礼盒</x:v>
       </x:c>
-      <x:c r="D33" s="151" t="str">
+      <x:c r="D33" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E33,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E33" s="154" t="n">
+      <x:c r="E33" s="249" t="n">
         <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
         <x:v>6.8</x:v>
       </x:c>
-      <x:c r="F33" s="151" t="str">
+      <x:c r="F33" s="234" t="str">
         <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
       </x:c>
     </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="151" t="n">
+    <x:row r="34" ht="22" customHeight="1">
+      <x:c r="A34" s="235" t="n">
         <x:f>ROW()-29</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B34" s="151" t="n">
+      <x:c r="B34" s="236" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E34,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>100176</x:v>
       </x:c>
-      <x:c r="C34" s="151" t="str">
+      <x:c r="C34" s="236" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E34,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>3D磁吸积木套装</x:v>
       </x:c>
-      <x:c r="D34" s="151" t="str">
+      <x:c r="D34" s="236" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E34,'商品数据'!$K$6:$K$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E34" s="154" t="n">
+      <x:c r="E34" s="250" t="n">
         <x:f>SMALL('商品数据'!$K$6:$K$11,ROW()-29)</x:f>
         <x:v>18.6</x:v>
       </x:c>
-      <x:c r="F34" s="151" t="str">
+      <x:c r="F34" s="238" t="str">
         <x:v>按 GMV 环比/上一周期变化升序，数值单位为 %</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="150" t="str">
+      <x:c r="A36" s="178" t="str">
         <x:v>CVR 下降 Top5｜按 CVR 变化百分点升序</x:v>
       </x:c>
-      <x:c r="B36" s="150"/>
-      <x:c r="C36" s="150"/>
-      <x:c r="D36" s="150"/>
-      <x:c r="E36" s="150"/>
-      <x:c r="F36" s="150"/>
+      <x:c r="B36" s="178"/>
+      <x:c r="C36" s="178"/>
+      <x:c r="D36" s="178"/>
+      <x:c r="E36" s="178"/>
+      <x:c r="F36" s="178"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" t="str">
+      <x:c r="A37" s="256" t="str">
         <x:v>排名</x:v>
       </x:c>
-      <x:c r="B37" t="str">
+      <x:c r="B37" s="256" t="str">
         <x:v>商品ID</x:v>
       </x:c>
-      <x:c r="C37" t="str">
+      <x:c r="C37" s="256" t="str">
         <x:v>商品名称</x:v>
       </x:c>
-      <x:c r="D37" t="str">
+      <x:c r="D37" s="256" t="str">
         <x:v>店铺</x:v>
       </x:c>
-      <x:c r="E37" t="str">
+      <x:c r="E37" s="256" t="str">
         <x:v>指标值</x:v>
       </x:c>
-      <x:c r="F37" t="str">
+      <x:c r="F37" s="256" t="str">
         <x:v>口径</x:v>
       </x:c>
     </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="151" t="n">
+    <x:row r="38" ht="22" customHeight="1">
+      <x:c r="A38" s="227" t="n">
         <x:f>ROW()-37</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B38" s="151" t="n">
+      <x:c r="B38" s="228" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E38,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>100407</x:v>
       </x:c>
-      <x:c r="C38" s="151" t="str">
+      <x:c r="C38" s="228" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E38,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>磁力迷宫玩具</x:v>
       </x:c>
-      <x:c r="D38" s="151" t="str">
+      <x:c r="D38" s="228" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E38,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E38" s="155" t="n">
+      <x:c r="E38" s="257" t="n">
         <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
         <x:v>-1.46</x:v>
       </x:c>
-      <x:c r="F38" s="151" t="str">
+      <x:c r="F38" s="230" t="str">
         <x:v>按 CVR 变化百分点升序</x:v>
       </x:c>
     </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="151" t="n">
+    <x:row r="39" ht="22" customHeight="1">
+      <x:c r="A39" s="231" t="n">
         <x:f>ROW()-37</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B39" s="151" t="n">
+      <x:c r="B39" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E39,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="C39" s="151" t="str">
+      <x:c r="C39" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E39,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>儿童户外泡泡机</x:v>
       </x:c>
-      <x:c r="D39" s="151" t="str">
+      <x:c r="D39" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E39,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E39" s="155" t="n">
+      <x:c r="E39" s="258" t="n">
         <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
         <x:v>-1.18</x:v>
       </x:c>
-      <x:c r="F39" s="151" t="str">
+      <x:c r="F39" s="234" t="str">
         <x:v>按 CVR 变化百分点升序</x:v>
       </x:c>
     </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="151" t="n">
+    <x:row r="40" ht="22" customHeight="1">
+      <x:c r="A40" s="231" t="n">
         <x:f>ROW()-37</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B40" s="151" t="n">
+      <x:c r="B40" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E40,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>100091</x:v>
       </x:c>
-      <x:c r="C40" s="151" t="str">
+      <x:c r="C40" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E40,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>益智拼图礼盒</x:v>
       </x:c>
-      <x:c r="D40" s="151" t="str">
+      <x:c r="D40" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E40,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="E40" s="155" t="n">
+      <x:c r="E40" s="258" t="n">
         <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
         <x:v>-0.42</x:v>
       </x:c>
-      <x:c r="F40" s="151" t="str">
+      <x:c r="F40" s="234" t="str">
         <x:v>按 CVR 变化百分点升序</x:v>
       </x:c>
     </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="151" t="n">
+    <x:row r="41" ht="22" customHeight="1">
+      <x:c r="A41" s="231" t="n">
         <x:f>ROW()-37</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B41" s="151" t="n">
+      <x:c r="B41" s="232" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E41,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>100512</x:v>
       </x:c>
-      <x:c r="C41" s="151" t="str">
+      <x:c r="C41" s="232" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E41,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>折叠儿童画板</x:v>
       </x:c>
-      <x:c r="D41" s="151" t="str">
+      <x:c r="D41" s="232" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E41,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="E41" s="155" t="n">
+      <x:c r="E41" s="258" t="n">
         <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
         <x:v>-0.24</x:v>
       </x:c>
-      <x:c r="F41" s="151" t="str">
+      <x:c r="F41" s="234" t="str">
         <x:v>按 CVR 变化百分点升序</x:v>
       </x:c>
     </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="151" t="n">
+    <x:row r="42" ht="22" customHeight="1">
+      <x:c r="A42" s="235" t="n">
         <x:f>ROW()-37</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B42" s="151" t="n">
+      <x:c r="B42" s="236" t="n">
         <x:f>INDEX('商品数据'!$C$6:$C$11,MATCH($E42,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>100314</x:v>
       </x:c>
-      <x:c r="C42" s="151" t="str">
+      <x:c r="C42" s="236" t="str">
         <x:f>INDEX('商品数据'!$D$6:$D$11,MATCH($E42,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>儿童绘画水彩笔</x:v>
       </x:c>
-      <x:c r="D42" s="151" t="str">
+      <x:c r="D42" s="236" t="str">
         <x:f>INDEX('商品数据'!$B$6:$B$11,MATCH($E42,'商品数据'!$N$6:$N$11,0))</x:f>
         <x:v>US-旗舰店</x:v>
       </x:c>
-      <x:c r="E42" s="155" t="n">
+      <x:c r="E42" s="259" t="n">
         <x:f>SMALL('商品数据'!$N$6:$N$11,ROW()-37)</x:f>
         <x:v>0.38</x:v>
       </x:c>
-      <x:c r="F42" s="151" t="str">
+      <x:c r="F42" s="238" t="str">
         <x:v>按 CVR 变化百分点升序</x:v>
       </x:c>
     </x:row>
@@ -2929,22 +3602,27 @@
     <x:mergeCell ref="A36:F36"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="15">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3467c6497784f50"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4beb54ff07014d6c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03cb25c6ba884754"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cfea2b9663e4c14"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda86ca64eb8c413b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab43f11d43ce4cf1"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb38b21a5eae4738"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1c2c7ae050c4135"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e69d14e6cc64830"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf591b00eb7a84637"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9721d150f59d4d8d"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3184515a90514edf"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f255e6221f84b7e"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37b232f492d94c5a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd3053fccd984378"/>
+  <x:tableParts count="20">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7357b81ca4c74283"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7baeba3e567b45ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a80f1cd0cd74774"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54919b9ac5534b1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5868c63495f545df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ebcdf2059b3498e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d1a1f606dbe4b6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R955338c87a044e0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R116c3ad528c14029"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ae2a8cbd83748cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78611875befe4676"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re655ba8c83bc4a81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf1e2611dff8426d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeed514329ad4871"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62384a40ce9c441e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1204de4d06f541c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bb70954cbe748ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fc85ca3cb5546c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75826d8e1d924671"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R403c32a42dad4256"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2964,317 +3642,317 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="145" t="str">
+      <x:c r="A1" s="173" t="str">
         <x:v>商品数据预警｜规则与处理队列</x:v>
       </x:c>
-      <x:c r="B1" s="145"/>
-      <x:c r="C1" s="145"/>
-      <x:c r="D1" s="145"/>
-      <x:c r="E1" s="145"/>
-      <x:c r="F1" s="145"/>
-      <x:c r="G1" s="145"/>
-      <x:c r="H1" s="145"/>
+      <x:c r="B1" s="173"/>
+      <x:c r="C1" s="173"/>
+      <x:c r="D1" s="173"/>
+      <x:c r="E1" s="173"/>
+      <x:c r="F1" s="173"/>
+      <x:c r="G1" s="173"/>
+      <x:c r="H1" s="173"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
-      <x:c r="A2" s="146" t="str">
+      <x:c r="A2" s="174" t="str">
         <x:v>预警规则对应网站“商品数据预警”页；黄色区可维护规则和处理记录，状态必须基于真实 T+1 / T+3 / T+7 数据。</x:v>
       </x:c>
-      <x:c r="B2" s="146"/>
-      <x:c r="C2" s="146"/>
-      <x:c r="D2" s="146"/>
-      <x:c r="E2" s="146"/>
-      <x:c r="F2" s="146"/>
-      <x:c r="G2" s="146"/>
-      <x:c r="H2" s="146"/>
+      <x:c r="B2" s="174"/>
+      <x:c r="C2" s="174"/>
+      <x:c r="D2" s="174"/>
+      <x:c r="E2" s="174"/>
+      <x:c r="F2" s="174"/>
+      <x:c r="G2" s="174"/>
+      <x:c r="H2" s="174"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="147" t="str">
+      <x:c r="A5" s="260" t="str">
         <x:v>预警指标</x:v>
       </x:c>
-      <x:c r="B5" s="147" t="str">
+      <x:c r="B5" s="261" t="str">
         <x:v>触发条件</x:v>
       </x:c>
-      <x:c r="C5" s="147" t="str">
+      <x:c r="C5" s="261" t="str">
         <x:v>建议节点</x:v>
       </x:c>
-      <x:c r="D5" s="147" t="str">
+      <x:c r="D5" s="262" t="str">
         <x:v>启用</x:v>
       </x:c>
-      <x:c r="F5" s="147" t="str">
+      <x:c r="F5" s="260" t="str">
         <x:v>汇总指标</x:v>
       </x:c>
-      <x:c r="G5" s="147" t="str">
+      <x:c r="G5" s="261" t="str">
         <x:v>当前值</x:v>
       </x:c>
-      <x:c r="H5" s="147" t="str">
+      <x:c r="H5" s="262" t="str">
         <x:v>说明</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="148" t="str">
+      <x:c r="A6" s="263" t="str">
         <x:v>曝光下降</x:v>
       </x:c>
-      <x:c r="B6" s="148" t="str">
+      <x:c r="B6" s="264" t="str">
         <x:v>环比 &gt; 20%</x:v>
       </x:c>
-      <x:c r="C6" s="148" t="str">
+      <x:c r="C6" s="264" t="str">
         <x:v>T+1</x:v>
       </x:c>
-      <x:c r="D6" s="148" t="str">
+      <x:c r="D6" s="265" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="F6" t="str">
+      <x:c r="F6" s="269" t="str">
         <x:v>高风险预警</x:v>
       </x:c>
-      <x:c r="G6" t="n">
+      <x:c r="G6" s="283" t="n">
         <x:f>COUNTIF('商品数据'!$Q$6:$Q$11,"需处理")</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H6" t="str">
+      <x:c r="H6" s="271" t="str">
         <x:v>由商品数据的当前状态汇总</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="148" t="str">
+      <x:c r="A7" s="263" t="str">
         <x:v>GMV 下降</x:v>
       </x:c>
-      <x:c r="B7" s="148" t="str">
+      <x:c r="B7" s="264" t="str">
         <x:v>环比 &gt; 15%</x:v>
       </x:c>
-      <x:c r="C7" s="148" t="str">
+      <x:c r="C7" s="264" t="str">
         <x:v>T+1 / T+3</x:v>
       </x:c>
-      <x:c r="D7" s="148" t="str">
+      <x:c r="D7" s="265" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="F7" t="str">
+      <x:c r="F7" s="269" t="str">
         <x:v>中风险预警</x:v>
       </x:c>
-      <x:c r="G7" t="n">
+      <x:c r="G7" s="284" t="n">
         <x:f>COUNTIF('商品数据'!$Q$6:$Q$11,"需观察")</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H7" t="str">
+      <x:c r="H7" s="271" t="str">
         <x:v>由商品数据的当前状态汇总</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="148" t="str">
+      <x:c r="A8" s="263" t="str">
         <x:v>CTR 下降</x:v>
       </x:c>
-      <x:c r="B8" s="148" t="str">
+      <x:c r="B8" s="264" t="str">
         <x:v>下降 &gt; 0.5 个百分点</x:v>
       </x:c>
-      <x:c r="C8" s="148" t="str">
+      <x:c r="C8" s="264" t="str">
         <x:v>T+1</x:v>
       </x:c>
-      <x:c r="D8" s="148" t="str">
+      <x:c r="D8" s="265" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="F8" t="str">
+      <x:c r="F8" s="269" t="str">
         <x:v>低风险预警</x:v>
       </x:c>
-      <x:c r="G8" t="n">
+      <x:c r="G8" s="285" t="n">
         <x:f>COUNTIF('商品数据'!$Q$6:$Q$11,"表现良好")</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H8" t="str">
+      <x:c r="H8" s="271" t="str">
         <x:v>由商品数据的当前状态汇总</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="148" t="str">
+      <x:c r="A9" s="263" t="str">
         <x:v>CVR 下降</x:v>
       </x:c>
-      <x:c r="B9" s="148" t="str">
+      <x:c r="B9" s="264" t="str">
         <x:v>下降 &gt; 0.3 个百分点</x:v>
       </x:c>
-      <x:c r="C9" s="148" t="str">
+      <x:c r="C9" s="264" t="str">
         <x:v>T+1 / T+3 / T+7</x:v>
       </x:c>
-      <x:c r="D9" s="148" t="str">
+      <x:c r="D9" s="265" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="F9" t="str">
+      <x:c r="F9" s="269" t="str">
         <x:v>待处理商品</x:v>
       </x:c>
-      <x:c r="G9" t="n">
+      <x:c r="G9" s="286" t="n">
         <x:f>COUNTIF('商品数据'!$Q$6:$Q$11,"需处理")</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H9" t="str">
+      <x:c r="H9" s="271" t="str">
         <x:v>建议动作不为空的商品数</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="148" t="str">
+      <x:c r="A10" s="266" t="str">
         <x:v>库存/承接异常</x:v>
       </x:c>
-      <x:c r="B10" s="148" t="str">
+      <x:c r="B10" s="267" t="str">
         <x:v>需人工判断</x:v>
       </x:c>
-      <x:c r="C10" s="148" t="str">
+      <x:c r="C10" s="267" t="str">
         <x:v>发现即处理</x:v>
       </x:c>
-      <x:c r="D10" s="148" t="str">
+      <x:c r="D10" s="268" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="F10" t="str">
+      <x:c r="F10" s="272" t="str">
         <x:v>今日检测商品</x:v>
       </x:c>
-      <x:c r="G10" t="n">
+      <x:c r="G10" s="287" t="n">
         <x:f>COUNTA('商品数据'!$C$6:$C$11)</x:f>
         <x:v>6</x:v>
       </x:c>
-      <x:c r="H10" t="str">
+      <x:c r="H10" s="274" t="str">
         <x:v>当前日期窗口的商品记录数</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
-      <x:c r="A13" s="147" t="str">
+      <x:c r="A13" s="260" t="str">
         <x:v>商品ID</x:v>
       </x:c>
-      <x:c r="B13" s="147" t="str">
+      <x:c r="B13" s="261" t="str">
         <x:v>店铺</x:v>
       </x:c>
-      <x:c r="C13" s="147" t="str">
+      <x:c r="C13" s="261" t="str">
         <x:v>预警类型</x:v>
       </x:c>
-      <x:c r="D13" s="147" t="str">
+      <x:c r="D13" s="261" t="str">
         <x:v>当前指标</x:v>
       </x:c>
-      <x:c r="E13" s="147" t="str">
+      <x:c r="E13" s="261" t="str">
         <x:v>变化值</x:v>
       </x:c>
-      <x:c r="F13" s="147" t="str">
+      <x:c r="F13" s="261" t="str">
         <x:v>建议动作</x:v>
       </x:c>
-      <x:c r="G13" s="147" t="str">
+      <x:c r="G13" s="261" t="str">
         <x:v>处理状态</x:v>
       </x:c>
-      <x:c r="H13" s="147" t="str">
+      <x:c r="H13" s="262" t="str">
         <x:v>证据/备注</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="148" t="str">
+    <x:row r="14" ht="26" customHeight="1">
+      <x:c r="A14" s="263" t="str">
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="B14" s="148" t="str">
+      <x:c r="B14" s="264" t="str">
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="C14" s="148" t="str">
+      <x:c r="C14" s="264" t="str">
         <x:v>曝光下降</x:v>
       </x:c>
-      <x:c r="D14" s="148" t="str">
+      <x:c r="D14" s="264" t="str">
         <x:v>曝光</x:v>
       </x:c>
-      <x:c r="E14" s="156" t="n">
+      <x:c r="E14" s="275" t="n">
         <x:v>-28</x:v>
       </x:c>
-      <x:c r="F14" s="148" t="str">
+      <x:c r="F14" s="264" t="str">
         <x:v>先核查推荐流量与主图承接</x:v>
       </x:c>
-      <x:c r="G14" s="148" t="str">
+      <x:c r="G14" s="264" t="str">
         <x:v>待处理</x:v>
       </x:c>
-      <x:c r="H14" s="148"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="148" t="str">
+      <x:c r="H14" s="265"/>
+    </x:row>
+    <x:row r="15" ht="26" customHeight="1">
+      <x:c r="A15" s="263" t="str">
         <x:v>100407</x:v>
       </x:c>
-      <x:c r="B15" s="148" t="str">
+      <x:c r="B15" s="264" t="str">
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="C15" s="148" t="str">
+      <x:c r="C15" s="264" t="str">
         <x:v>CVR下降</x:v>
       </x:c>
-      <x:c r="D15" s="148" t="str">
+      <x:c r="D15" s="264" t="str">
         <x:v>CVR</x:v>
       </x:c>
-      <x:c r="E15" s="156" t="n">
+      <x:c r="E15" s="275" t="n">
         <x:v>-1.46</x:v>
       </x:c>
-      <x:c r="F15" s="148" t="str">
+      <x:c r="F15" s="264" t="str">
         <x:v>检查广告落地页、流量来源和库存承接</x:v>
       </x:c>
-      <x:c r="G15" s="148" t="str">
+      <x:c r="G15" s="264" t="str">
         <x:v>待处理</x:v>
       </x:c>
-      <x:c r="H15" s="148"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="148" t="str">
+      <x:c r="H15" s="265"/>
+    </x:row>
+    <x:row r="16" ht="26" customHeight="1">
+      <x:c r="A16" s="263" t="str">
         <x:v>100091</x:v>
       </x:c>
-      <x:c r="B16" s="148" t="str">
+      <x:c r="B16" s="264" t="str">
         <x:v>TH-主店</x:v>
       </x:c>
-      <x:c r="C16" s="148" t="str">
+      <x:c r="C16" s="264" t="str">
         <x:v>CVR下降</x:v>
       </x:c>
-      <x:c r="D16" s="148" t="str">
+      <x:c r="D16" s="264" t="str">
         <x:v>CVR</x:v>
       </x:c>
-      <x:c r="E16" s="156" t="n">
+      <x:c r="E16" s="275" t="n">
         <x:v>-0.42</x:v>
       </x:c>
-      <x:c r="F16" s="148" t="str">
+      <x:c r="F16" s="264" t="str">
         <x:v>检查商品承接和优惠设置</x:v>
       </x:c>
-      <x:c r="G16" s="148" t="str">
+      <x:c r="G16" s="264" t="str">
         <x:v>观察</x:v>
       </x:c>
-      <x:c r="H16" s="148"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="148" t="str">
+      <x:c r="H16" s="265"/>
+    </x:row>
+    <x:row r="17" ht="26" customHeight="1">
+      <x:c r="A17" s="263" t="str">
         <x:v>100512</x:v>
       </x:c>
-      <x:c r="B17" s="148" t="str">
+      <x:c r="B17" s="264" t="str">
         <x:v>US-日用店</x:v>
       </x:c>
-      <x:c r="C17" s="148" t="str">
+      <x:c r="C17" s="264" t="str">
         <x:v>CTR下降</x:v>
       </x:c>
-      <x:c r="D17" s="148" t="str">
+      <x:c r="D17" s="264" t="str">
         <x:v>CTR</x:v>
       </x:c>
-      <x:c r="E17" s="156" t="n">
+      <x:c r="E17" s="275" t="n">
         <x:v>-0.22</x:v>
       </x:c>
-      <x:c r="F17" s="148" t="str">
+      <x:c r="F17" s="264" t="str">
         <x:v>继续观察，不单独判定异常</x:v>
       </x:c>
-      <x:c r="G17" s="148" t="str">
+      <x:c r="G17" s="264" t="str">
         <x:v>观察</x:v>
       </x:c>
-      <x:c r="H17" s="148"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="148"/>
-      <x:c r="B18" s="148"/>
-      <x:c r="C18" s="148"/>
-      <x:c r="D18" s="148"/>
-      <x:c r="E18" s="156"/>
-      <x:c r="F18" s="148"/>
-      <x:c r="G18" s="148" t="str">
+      <x:c r="H17" s="265"/>
+    </x:row>
+    <x:row r="18" ht="26" customHeight="1">
+      <x:c r="A18" s="263"/>
+      <x:c r="B18" s="264"/>
+      <x:c r="C18" s="264"/>
+      <x:c r="D18" s="264"/>
+      <x:c r="E18" s="275"/>
+      <x:c r="F18" s="264"/>
+      <x:c r="G18" s="264" t="str">
         <x:v>待填写</x:v>
       </x:c>
-      <x:c r="H18" s="148"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="148"/>
-      <x:c r="B19" s="148"/>
-      <x:c r="C19" s="148"/>
-      <x:c r="D19" s="148"/>
-      <x:c r="E19" s="156"/>
-      <x:c r="F19" s="148"/>
-      <x:c r="G19" s="148" t="str">
+      <x:c r="H18" s="265"/>
+    </x:row>
+    <x:row r="19" ht="26" customHeight="1">
+      <x:c r="A19" s="266"/>
+      <x:c r="B19" s="267"/>
+      <x:c r="C19" s="267"/>
+      <x:c r="D19" s="267"/>
+      <x:c r="E19" s="276"/>
+      <x:c r="F19" s="267"/>
+      <x:c r="G19" s="267" t="str">
         <x:v>待填写</x:v>
       </x:c>
-      <x:c r="H19" s="148"/>
+      <x:c r="H19" s="268"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3290,16 +3968,19 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="9">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc898bd111f00425b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8c0314cf05f4b0a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra83981bbfd1a4733"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cab14e705184a7b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd08d0d2baed342e7"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34ead97d06cd4596"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f4a538fc80f4b73"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re25a5b28c6704b30"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5e86e589aa24bfc"/>
+  <x:tableParts count="12">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb4958d209464383"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7283bbd1c21b43d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b18e034901a45b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rece4a406001642bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcff78d8d23774d02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7536223e2714e6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcae34c32a4eb4e08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46d2fca408aa42aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e16034218ee4da4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89a6ab0db90e443c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb60dcfa4ef44928"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f2cf813c94648b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3321,204 +4002,204 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="145" t="str">
+      <x:c r="A1" s="173" t="str">
         <x:v>运营知识库｜有效方法沉淀</x:v>
       </x:c>
-      <x:c r="B1" s="145"/>
-      <x:c r="C1" s="145"/>
-      <x:c r="D1" s="145"/>
-      <x:c r="E1" s="145"/>
-      <x:c r="F1" s="145"/>
-      <x:c r="G1" s="145"/>
-      <x:c r="H1" s="145"/>
-      <x:c r="I1" s="145"/>
-      <x:c r="J1" s="145"/>
+      <x:c r="B1" s="173"/>
+      <x:c r="C1" s="173"/>
+      <x:c r="D1" s="173"/>
+      <x:c r="E1" s="173"/>
+      <x:c r="F1" s="173"/>
+      <x:c r="G1" s="173"/>
+      <x:c r="H1" s="173"/>
+      <x:c r="I1" s="173"/>
+      <x:c r="J1" s="173"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
-      <x:c r="A2" s="146" t="str">
+      <x:c r="A2" s="174" t="str">
         <x:v>对应网站“运营知识库”页；只有有真实验证证据的动作才进入有效方法库，待验证动作留在运营动作表。</x:v>
       </x:c>
-      <x:c r="B2" s="146"/>
-      <x:c r="C2" s="146"/>
-      <x:c r="D2" s="146"/>
-      <x:c r="E2" s="146"/>
-      <x:c r="F2" s="146"/>
-      <x:c r="G2" s="146"/>
-      <x:c r="H2" s="146"/>
-      <x:c r="I2" s="146"/>
-      <x:c r="J2" s="146"/>
+      <x:c r="B2" s="174"/>
+      <x:c r="C2" s="174"/>
+      <x:c r="D2" s="174"/>
+      <x:c r="E2" s="174"/>
+      <x:c r="F2" s="174"/>
+      <x:c r="G2" s="174"/>
+      <x:c r="H2" s="174"/>
+      <x:c r="I2" s="174"/>
+      <x:c r="J2" s="174"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="147" t="str">
+      <x:c r="A5" s="260" t="str">
         <x:v>方法ID</x:v>
       </x:c>
-      <x:c r="B5" s="147" t="str">
+      <x:c r="B5" s="261" t="str">
         <x:v>方法标题</x:v>
       </x:c>
-      <x:c r="C5" s="147" t="str">
+      <x:c r="C5" s="261" t="str">
         <x:v>分类</x:v>
       </x:c>
-      <x:c r="D5" s="147" t="str">
+      <x:c r="D5" s="261" t="str">
         <x:v>适用场景</x:v>
       </x:c>
-      <x:c r="E5" s="147" t="str">
+      <x:c r="E5" s="261" t="str">
         <x:v>验证商品/对象</x:v>
       </x:c>
-      <x:c r="F5" s="147" t="str">
+      <x:c r="F5" s="261" t="str">
         <x:v>证据摘要</x:v>
       </x:c>
-      <x:c r="G5" s="147" t="str">
+      <x:c r="G5" s="261" t="str">
         <x:v>验证状态</x:v>
       </x:c>
-      <x:c r="H5" s="147" t="str">
+      <x:c r="H5" s="261" t="str">
         <x:v>负责人</x:v>
       </x:c>
-      <x:c r="I5" s="147" t="str">
+      <x:c r="I5" s="261" t="str">
         <x:v>复用次数</x:v>
       </x:c>
-      <x:c r="J5" s="147" t="str">
+      <x:c r="J5" s="262" t="str">
         <x:v>备注</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="148" t="str">
+      <x:c r="A6" s="263" t="str">
         <x:v>KB-001</x:v>
       </x:c>
-      <x:c r="B6" s="148" t="str">
+      <x:c r="B6" s="264" t="str">
         <x:v>替换首图并增加使用场景图</x:v>
       </x:c>
-      <x:c r="C6" s="148" t="str">
+      <x:c r="C6" s="264" t="str">
         <x:v>主图优化</x:v>
       </x:c>
-      <x:c r="D6" s="148" t="str">
+      <x:c r="D6" s="264" t="str">
         <x:v>曝光但承接弱</x:v>
       </x:c>
-      <x:c r="E6" s="148" t="str">
+      <x:c r="E6" s="264" t="str">
         <x:v>100176</x:v>
       </x:c>
-      <x:c r="F6" s="148" t="str">
+      <x:c r="F6" s="264" t="str">
         <x:v>T+1 CVR +0.8pp；T+3 CVR +1.7pp</x:v>
       </x:c>
-      <x:c r="G6" s="148" t="str">
+      <x:c r="G6" s="291" t="str">
         <x:v>已验证有效</x:v>
       </x:c>
-      <x:c r="H6" s="148" t="str">
+      <x:c r="H6" s="264" t="str">
         <x:v>运营A</x:v>
       </x:c>
-      <x:c r="I6" s="157" t="n">
+      <x:c r="I6" s="288" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J6" s="148"/>
+      <x:c r="J6" s="265"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="148" t="str">
+      <x:c r="A7" s="263" t="str">
         <x:v>KB-002</x:v>
       </x:c>
-      <x:c r="B7" s="148" t="str">
+      <x:c r="B7" s="264" t="str">
         <x:v>组合装定价测试</x:v>
       </x:c>
-      <x:c r="C7" s="148" t="str">
+      <x:c r="C7" s="264" t="str">
         <x:v>价格策略</x:v>
       </x:c>
-      <x:c r="D7" s="148" t="str">
+      <x:c r="D7" s="264" t="str">
         <x:v>销量与 GMV 同时提升</x:v>
       </x:c>
-      <x:c r="E7" s="148" t="str">
+      <x:c r="E7" s="264" t="str">
         <x:v>100314</x:v>
       </x:c>
-      <x:c r="F7" s="148" t="str">
+      <x:c r="F7" s="264" t="str">
         <x:v>T+3 销量 +18%；T+7 GMV +26%</x:v>
       </x:c>
-      <x:c r="G7" s="148" t="str">
+      <x:c r="G7" s="291" t="str">
         <x:v>已验证有效</x:v>
       </x:c>
-      <x:c r="H7" s="148" t="str">
+      <x:c r="H7" s="264" t="str">
         <x:v>运营A</x:v>
       </x:c>
-      <x:c r="I7" s="157" t="n">
+      <x:c r="I7" s="288" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="J7" s="148"/>
+      <x:c r="J7" s="265"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="148" t="str">
+      <x:c r="A8" s="263" t="str">
         <x:v>KB-003</x:v>
       </x:c>
-      <x:c r="B8" s="148" t="str">
+      <x:c r="B8" s="264" t="str">
         <x:v>标题前置核心卖点</x:v>
       </x:c>
-      <x:c r="C8" s="148" t="str">
+      <x:c r="C8" s="264" t="str">
         <x:v>标题优化</x:v>
       </x:c>
-      <x:c r="D8" s="148" t="str">
+      <x:c r="D8" s="264" t="str">
         <x:v>CTR 有空间</x:v>
       </x:c>
-      <x:c r="E8" s="148" t="str">
+      <x:c r="E8" s="264" t="str">
         <x:v>100238</x:v>
       </x:c>
-      <x:c r="F8" s="148" t="str">
+      <x:c r="F8" s="264" t="str">
         <x:v>等待 T+1 数据回传</x:v>
       </x:c>
-      <x:c r="G8" s="148" t="str">
+      <x:c r="G8" s="293" t="str">
         <x:v>待验证</x:v>
       </x:c>
-      <x:c r="H8" s="148" t="str">
+      <x:c r="H8" s="264" t="str">
         <x:v>运营B</x:v>
       </x:c>
-      <x:c r="I8" s="157" t="n">
+      <x:c r="I8" s="288" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J8" s="148"/>
+      <x:c r="J8" s="265"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="148" t="str">
+      <x:c r="A9" s="263" t="str">
         <x:v>KB-004</x:v>
       </x:c>
-      <x:c r="B9" s="148" t="str">
+      <x:c r="B9" s="264" t="str">
         <x:v>更换广告落地页</x:v>
       </x:c>
-      <x:c r="C9" s="148" t="str">
+      <x:c r="C9" s="264" t="str">
         <x:v>广告投放</x:v>
       </x:c>
-      <x:c r="D9" s="148" t="str">
+      <x:c r="D9" s="264" t="str">
         <x:v>广告点击后承接弱</x:v>
       </x:c>
-      <x:c r="E9" s="148" t="str">
+      <x:c r="E9" s="264" t="str">
         <x:v>100407</x:v>
       </x:c>
-      <x:c r="F9" s="148" t="str">
+      <x:c r="F9" s="264" t="str">
         <x:v>T+3 曝光未恢复，销量继续下降</x:v>
       </x:c>
-      <x:c r="G9" s="148" t="str">
+      <x:c r="G9" s="295" t="str">
         <x:v>验证无效</x:v>
       </x:c>
-      <x:c r="H9" s="148" t="str">
+      <x:c r="H9" s="264" t="str">
         <x:v>运营B</x:v>
       </x:c>
-      <x:c r="I9" s="157" t="n">
+      <x:c r="I9" s="288" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J9" s="148" t="str">
+      <x:c r="J9" s="265" t="str">
         <x:v>停止复用</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="148" t="str">
+      <x:c r="A10" s="266" t="str">
         <x:v>KB-005</x:v>
       </x:c>
-      <x:c r="B10" s="148"/>
-      <x:c r="C10" s="148" t="str">
+      <x:c r="B10" s="267"/>
+      <x:c r="C10" s="267" t="str">
         <x:v>待填写</x:v>
       </x:c>
-      <x:c r="D10" s="148"/>
-      <x:c r="E10" s="148"/>
-      <x:c r="F10" s="148"/>
-      <x:c r="G10" s="148" t="str">
+      <x:c r="D10" s="267"/>
+      <x:c r="E10" s="267"/>
+      <x:c r="F10" s="267"/>
+      <x:c r="G10" s="297" t="str">
         <x:v>待填写</x:v>
       </x:c>
-      <x:c r="H10" s="148"/>
-      <x:c r="I10" s="157"/>
-      <x:c r="J10" s="148"/>
+      <x:c r="H10" s="267"/>
+      <x:c r="I10" s="289"/>
+      <x:c r="J10" s="268"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3531,10 +4212,11 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29d6f175f70c45b3"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R118d2f11873f4129"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0443cbe6df742b6"/>
+  <x:tableParts count="4">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb6ad6c6f1ad475a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83b8db6fa8e54f76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31f8203221b44b0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39cd867827604b0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3555,191 +4237,191 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="145" t="str">
+      <x:c r="A1" s="173" t="str">
         <x:v>Agent 调度中心｜运营任务登记</x:v>
       </x:c>
-      <x:c r="B1" s="145"/>
-      <x:c r="C1" s="145"/>
-      <x:c r="D1" s="145"/>
-      <x:c r="E1" s="145"/>
-      <x:c r="F1" s="145"/>
-      <x:c r="G1" s="145"/>
-      <x:c r="H1" s="145"/>
-      <x:c r="I1" s="145"/>
+      <x:c r="B1" s="173"/>
+      <x:c r="C1" s="173"/>
+      <x:c r="D1" s="173"/>
+      <x:c r="E1" s="173"/>
+      <x:c r="F1" s="173"/>
+      <x:c r="G1" s="173"/>
+      <x:c r="H1" s="173"/>
+      <x:c r="I1" s="173"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
-      <x:c r="A2" s="146" t="str">
+      <x:c r="A2" s="174" t="str">
         <x:v>对应网站 Agent 调度中心；本表记录要调用哪个 Agent、处理什么输入以及输出是否已被运营复核。</x:v>
       </x:c>
-      <x:c r="B2" s="146"/>
-      <x:c r="C2" s="146"/>
-      <x:c r="D2" s="146"/>
-      <x:c r="E2" s="146"/>
-      <x:c r="F2" s="146"/>
-      <x:c r="G2" s="146"/>
-      <x:c r="H2" s="146"/>
-      <x:c r="I2" s="146"/>
+      <x:c r="B2" s="174"/>
+      <x:c r="C2" s="174"/>
+      <x:c r="D2" s="174"/>
+      <x:c r="E2" s="174"/>
+      <x:c r="F2" s="174"/>
+      <x:c r="G2" s="174"/>
+      <x:c r="H2" s="174"/>
+      <x:c r="I2" s="174"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="147" t="str">
+      <x:c r="A5" s="260" t="str">
         <x:v>任务日期</x:v>
       </x:c>
-      <x:c r="B5" s="147" t="str">
+      <x:c r="B5" s="261" t="str">
         <x:v>Agent名称</x:v>
       </x:c>
-      <x:c r="C5" s="147" t="str">
+      <x:c r="C5" s="261" t="str">
         <x:v>触发入口</x:v>
       </x:c>
-      <x:c r="D5" s="147" t="str">
+      <x:c r="D5" s="261" t="str">
         <x:v>输入范围</x:v>
       </x:c>
-      <x:c r="E5" s="147" t="str">
+      <x:c r="E5" s="261" t="str">
         <x:v>任务目标</x:v>
       </x:c>
-      <x:c r="F5" s="147" t="str">
+      <x:c r="F5" s="261" t="str">
         <x:v>输出物</x:v>
       </x:c>
-      <x:c r="G5" s="147" t="str">
+      <x:c r="G5" s="261" t="str">
         <x:v>状态</x:v>
       </x:c>
-      <x:c r="H5" s="147" t="str">
+      <x:c r="H5" s="261" t="str">
         <x:v>复核人</x:v>
       </x:c>
-      <x:c r="I5" s="147" t="str">
+      <x:c r="I5" s="262" t="str">
         <x:v>备注</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="148" t="str">
+      <x:c r="A6" s="263" t="str">
         <x:v>2026-08-29</x:v>
       </x:c>
-      <x:c r="B6" s="148" t="str">
+      <x:c r="B6" s="264" t="str">
         <x:v>AI日报生成 Agent</x:v>
       </x:c>
-      <x:c r="C6" s="148" t="str">
+      <x:c r="C6" s="264" t="str">
         <x:v>经营总览</x:v>
       </x:c>
-      <x:c r="D6" s="148" t="str">
+      <x:c r="D6" s="264" t="str">
         <x:v>店铺日汇总 + 商品数据</x:v>
       </x:c>
-      <x:c r="E6" s="148" t="str">
+      <x:c r="E6" s="264" t="str">
         <x:v>结构化日报草稿</x:v>
       </x:c>
-      <x:c r="F6" s="148" t="str">
+      <x:c r="F6" s="264" t="str">
         <x:v>待复核</x:v>
       </x:c>
-      <x:c r="G6" s="148" t="str">
+      <x:c r="G6" s="293" t="str">
         <x:v>运营负责人</x:v>
       </x:c>
-      <x:c r="H6" s="148"/>
-      <x:c r="I6" s="148"/>
+      <x:c r="H6" s="264"/>
+      <x:c r="I6" s="265"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="148" t="str">
+      <x:c r="A7" s="263" t="str">
         <x:v>2026-08-29</x:v>
       </x:c>
-      <x:c r="B7" s="148" t="str">
+      <x:c r="B7" s="264" t="str">
         <x:v>自动巡检 Agent</x:v>
       </x:c>
-      <x:c r="C7" s="148" t="str">
+      <x:c r="C7" s="264" t="str">
         <x:v>商品数据预警</x:v>
       </x:c>
-      <x:c r="D7" s="148" t="str">
+      <x:c r="D7" s="264" t="str">
         <x:v>商品数据 + T+1/T+3/T+7</x:v>
       </x:c>
-      <x:c r="E7" s="148" t="str">
+      <x:c r="E7" s="264" t="str">
         <x:v>风险分级与优先队列</x:v>
       </x:c>
-      <x:c r="F7" s="148" t="str">
+      <x:c r="F7" s="264" t="str">
         <x:v>运行中</x:v>
       </x:c>
-      <x:c r="G7" s="148" t="str">
+      <x:c r="G7" s="293" t="str">
         <x:v>运营负责人</x:v>
       </x:c>
-      <x:c r="H7" s="148"/>
-      <x:c r="I7" s="148"/>
+      <x:c r="H7" s="264"/>
+      <x:c r="I7" s="265"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="148" t="str">
+      <x:c r="A8" s="263" t="str">
         <x:v>2026-08-29</x:v>
       </x:c>
-      <x:c r="B8" s="148" t="str">
+      <x:c r="B8" s="264" t="str">
         <x:v>排行榜分析 Agent</x:v>
       </x:c>
-      <x:c r="C8" s="148" t="str">
+      <x:c r="C8" s="264" t="str">
         <x:v>五组链接对比排行</x:v>
       </x:c>
-      <x:c r="D8" s="148" t="str">
+      <x:c r="D8" s="264" t="str">
         <x:v>商品数据</x:v>
       </x:c>
-      <x:c r="E8" s="148" t="str">
+      <x:c r="E8" s="264" t="str">
         <x:v>Top5 特征与可复用策略</x:v>
       </x:c>
-      <x:c r="F8" s="148" t="str">
+      <x:c r="F8" s="264" t="str">
         <x:v>待调用</x:v>
       </x:c>
-      <x:c r="G8" s="148"/>
-      <x:c r="H8" s="148"/>
-      <x:c r="I8" s="148"/>
+      <x:c r="G8" s="299"/>
+      <x:c r="H8" s="264"/>
+      <x:c r="I8" s="265"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="148" t="str">
+      <x:c r="A9" s="263" t="str">
         <x:v>2026-08-29</x:v>
       </x:c>
-      <x:c r="B9" s="148" t="str">
+      <x:c r="B9" s="264" t="str">
         <x:v>增长分析 Agent</x:v>
       </x:c>
-      <x:c r="C9" s="148" t="str">
+      <x:c r="C9" s="264" t="str">
         <x:v>GMV 上涨 Top5</x:v>
       </x:c>
-      <x:c r="D9" s="148" t="str">
+      <x:c r="D9" s="264" t="str">
         <x:v>商品数据 + 运营动作</x:v>
       </x:c>
-      <x:c r="E9" s="148" t="str">
+      <x:c r="E9" s="264" t="str">
         <x:v>上涨原因与方法沉淀</x:v>
       </x:c>
-      <x:c r="F9" s="148" t="str">
+      <x:c r="F9" s="264" t="str">
         <x:v>待调用</x:v>
       </x:c>
-      <x:c r="G9" s="148"/>
-      <x:c r="H9" s="148"/>
-      <x:c r="I9" s="148"/>
+      <x:c r="G9" s="299"/>
+      <x:c r="H9" s="264"/>
+      <x:c r="I9" s="265"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="148" t="str">
+      <x:c r="A10" s="263" t="str">
         <x:v>2026-08-29</x:v>
       </x:c>
-      <x:c r="B10" s="148" t="str">
+      <x:c r="B10" s="264" t="str">
         <x:v>下滑诊断 Agent</x:v>
       </x:c>
-      <x:c r="C10" s="148" t="str">
+      <x:c r="C10" s="264" t="str">
         <x:v>GMV/CVR 下降 Top5</x:v>
       </x:c>
-      <x:c r="D10" s="148" t="str">
+      <x:c r="D10" s="264" t="str">
         <x:v>商品数据 + 广告计划</x:v>
       </x:c>
-      <x:c r="E10" s="148" t="str">
+      <x:c r="E10" s="264" t="str">
         <x:v>下滑原因与挽回方案</x:v>
       </x:c>
-      <x:c r="F10" s="148" t="str">
+      <x:c r="F10" s="264" t="str">
         <x:v>待调用</x:v>
       </x:c>
-      <x:c r="G10" s="148"/>
-      <x:c r="H10" s="148"/>
-      <x:c r="I10" s="148"/>
+      <x:c r="G10" s="299"/>
+      <x:c r="H10" s="264"/>
+      <x:c r="I10" s="265"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="148"/>
-      <x:c r="B11" s="148"/>
-      <x:c r="C11" s="148"/>
-      <x:c r="D11" s="148"/>
-      <x:c r="E11" s="148"/>
-      <x:c r="F11" s="148"/>
-      <x:c r="G11" s="148" t="str">
+      <x:c r="A11" s="266"/>
+      <x:c r="B11" s="267"/>
+      <x:c r="C11" s="267"/>
+      <x:c r="D11" s="267"/>
+      <x:c r="E11" s="267"/>
+      <x:c r="F11" s="267"/>
+      <x:c r="G11" s="301" t="str">
         <x:v>待填写</x:v>
       </x:c>
-      <x:c r="H11" s="148"/>
-      <x:c r="I11" s="148"/>
+      <x:c r="H11" s="267"/>
+      <x:c r="I11" s="268"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3752,10 +4434,11 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R921eb3b1098e4979"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbc136563cb54a91"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree0cda171a1743b1"/>
+  <x:tableParts count="4">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbaee334c7bca4a01"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5b90df1b11b4e64"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf48e540672f24465"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R210c574442c34b28"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3771,112 +4454,112 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="145" t="str">
+      <x:c r="A1" s="173" t="str">
         <x:v>云文档说明｜WPS/Kdocs 使用流程</x:v>
       </x:c>
-      <x:c r="B1" s="145"/>
-      <x:c r="C1" s="145"/>
-      <x:c r="D1" s="145"/>
+      <x:c r="B1" s="173"/>
+      <x:c r="C1" s="173"/>
+      <x:c r="D1" s="173"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
-      <x:c r="A2" s="146" t="str">
+      <x:c r="A2" s="174" t="str">
         <x:v>这张表是给运营看的操作说明；填报数据请回到黄色输入区域，公式排行和预警汇总不要手工改写。</x:v>
       </x:c>
-      <x:c r="B2" s="146"/>
-      <x:c r="C2" s="146"/>
-      <x:c r="D2" s="146"/>
+      <x:c r="B2" s="174"/>
+      <x:c r="C2" s="174"/>
+      <x:c r="D2" s="174"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="147" t="str">
+      <x:c r="A5" s="309" t="str">
         <x:v>步骤</x:v>
       </x:c>
-      <x:c r="B5" s="147" t="str">
+      <x:c r="B5" s="310" t="str">
         <x:v>运营操作</x:v>
       </x:c>
-      <x:c r="C5" s="147" t="str">
+      <x:c r="C5" s="310" t="str">
         <x:v>涉及工作表</x:v>
       </x:c>
-      <x:c r="D5" s="147" t="str">
+      <x:c r="D5" s="311" t="str">
         <x:v>网站对应页面</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="148" t="str">
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="A6" s="263" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B6" s="148" t="str">
+      <x:c r="B6" s="264" t="str">
         <x:v>上传本文件到 WPS/Kdocs，设置团队协作权限</x:v>
       </x:c>
-      <x:c r="C6" s="148" t="str">
+      <x:c r="C6" s="264" t="str">
         <x:v>整本工作簿</x:v>
       </x:c>
-      <x:c r="D6" s="148" t="str">
+      <x:c r="D6" s="265" t="str">
         <x:v>数据接入</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="148" t="str">
+    <x:row r="7" ht="28" customHeight="1">
+      <x:c r="A7" s="263" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B7" s="148" t="str">
+      <x:c r="B7" s="264" t="str">
         <x:v>先维护店铺字典，再填写店铺、商品和已执行动作</x:v>
       </x:c>
-      <x:c r="C7" s="148" t="str">
+      <x:c r="C7" s="264" t="str">
         <x:v>店铺字典 / 店铺日汇总 / 商品数据 / 运营动作</x:v>
       </x:c>
-      <x:c r="D7" s="148" t="str">
+      <x:c r="D7" s="265" t="str">
         <x:v>经营总览 / 商品数据预警</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="148" t="str">
+    <x:row r="8" ht="28" customHeight="1">
+      <x:c r="A8" s="263" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B8" s="148" t="str">
+      <x:c r="B8" s="264" t="str">
         <x:v>核对五组排行、预警队列、Agent 任务和知识库</x:v>
       </x:c>
-      <x:c r="C8" s="148" t="str">
+      <x:c r="C8" s="264" t="str">
         <x:v>五组排行 / 预警规则 / Agent调度 / 运营知识库</x:v>
       </x:c>
-      <x:c r="D8" s="148" t="str">
+      <x:c r="D8" s="265" t="str">
         <x:v>经营总览 / Agent 调度中心 / 运营知识库</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="148" t="str">
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="A9" s="263" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B9" s="148" t="str">
+      <x:c r="B9" s="264" t="str">
         <x:v>导出 CSV 或交给后端 API；静态 GitHub Pages 不会自动读取私有文档</x:v>
       </x:c>
-      <x:c r="C9" s="148" t="str">
+      <x:c r="C9" s="264" t="str">
         <x:v>按字段字典映射</x:v>
       </x:c>
-      <x:c r="D9" s="148" t="str">
+      <x:c r="D9" s="265" t="str">
         <x:v>数据接入</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="148" t="str">
+    <x:row r="10" ht="28" customHeight="1">
+      <x:c r="A10" s="266" t="str">
         <x:v>注意</x:v>
       </x:c>
-      <x:c r="B10" s="148" t="str">
+      <x:c r="B10" s="267" t="str">
         <x:v>当前内容是演示模板；真实数据请保持缺失为空，不能用 0 代替未知。</x:v>
       </x:c>
-      <x:c r="C10" s="148" t="str">
+      <x:c r="C10" s="267" t="str">
         <x:v>字段字典</x:v>
       </x:c>
-      <x:c r="D10" s="148" t="str">
+      <x:c r="D10" s="268" t="str">
         <x:v>全部页面</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
-      <x:c r="A12" s="172" t="str">
+      <x:c r="A12" s="186" t="str">
         <x:v>公开网站当前为静态演示版。WPS/Kdocs 文档可以作为统一填报源，但真实数据自动刷新仍需要后端同步/API 和认证权限。</x:v>
       </x:c>
-      <x:c r="B12" s="172"/>
-      <x:c r="C12" s="172"/>
-      <x:c r="D12" s="172"/>
+      <x:c r="B12" s="186"/>
+      <x:c r="C12" s="186"/>
+      <x:c r="D12" s="186"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3885,8 +4568,9 @@
     <x:mergeCell ref="A12:D12"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42b8a7cdd0534ce5"/>
+  <x:tableParts count="2">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36e06dad58184947"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc94cabd287145b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6030,7 +6714,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb966784531af4294"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a3083ac405748d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8522,7 +9206,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc13ef3c3a5a1405a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ca8eaf22736417b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10249,7 +10933,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d0dc64c7e3f4719"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc992083adf2f47f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10990,7 +11674,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7715adb9a128491d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f1e80c53d8e41e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12048,7 +12732,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85b97472b3bb4522"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33e6517606774301"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13600,7 +14284,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7179c49351134b66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd883b24f3b847a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14761,7 +15445,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dfaf32231f147f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddc9d8c121424635"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14923,7 +15607,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e8ed2bd03f54253"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e0e9683743a4a7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>